<commit_message>
Add validated run and trace contract
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R539773c874034a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R0ee9d4e1b2594185"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.05</x:v>
+        <x:v>0.06666666666666667</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>274</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.07407407407407407</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>18.5</x:v>
+        <x:v>18.166666666666668</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1243,7 +1243,7 @@
         <x:v>Define run and trace contracts</x:v>
       </x:c>
       <x:c r="D15" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E15" s="19" t="str">
         <x:v>TB-002</x:v>
@@ -1253,7 +1253,7 @@
       </x:c>
       <x:c r="G15" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E15="",TRUE,COUNTIFS($A$12:$A$71,E15)=1),IF(F15="",TRUE,COUNTIFS($A$12:$A$71,F15)=1))),"Bad dependency",IF(NOT(AND(IF(E15="",TRUE,COUNTIFS($A$12:$A$71,E15,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F15="",TRUE,COUNTIFS($A$12:$A$71,F15,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D15="Completed","Check prerequisites","Waiting"),IF(D15="Completed",IF(S15="","Evidence needed","Done"),IF(D15="Blocked","Blocked",IF(D15="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H15" s="27" t="n">
         <x:v>4</x:v>
@@ -1282,11 +1282,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R15" s="19" t="str"/>
-      <x:c r="S15" s="23" t="str"/>
+      <x:c r="S15" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/docs/trace-contract.md</x:v>
+      </x:c>
       <x:c r="T15" s="23" t="str"/>
       <x:c r="U15" s="19" t="n">
         <x:f>IF(LEN(S15)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
@@ -1365,7 +1367,7 @@
       </x:c>
       <x:c r="G17" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E17="",TRUE,COUNTIFS($A$12:$A$71,E17)=1),IF(F17="",TRUE,COUNTIFS($A$12:$A$71,F17)=1))),"Bad dependency",IF(NOT(AND(IF(E17="",TRUE,COUNTIFS($A$12:$A$71,E17,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F17="",TRUE,COUNTIFS($A$12:$A$71,F17,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D17="Completed","Check prerequisites","Waiting"),IF(D17="Completed",IF(S17="","Evidence needed","Done"),IF(D17="Blocked","Blocked",IF(D17="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H17" s="27" t="n">
         <x:v>4</x:v>
@@ -4588,11 +4590,11 @@
       </x:c>
       <x:c r="C79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"Completed")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"In Progress")</x:f>
@@ -4604,7 +4606,7 @@
       </x:c>
       <x:c r="G79" s="29" t="n">
         <x:f>IF(B79=0,0,C79/B79)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="H79" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A79)</x:f>
@@ -4612,7 +4614,7 @@
       </x:c>
       <x:c r="I79" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A79,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>10</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$G$12:$G$71,"Ready")</x:f>
@@ -7383,13 +7385,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb874ae98f7c344eb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d0e830573e74039"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb30a08255ea4222"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11bd8bb6d0ae434c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R018951229cc44225"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0736a7e9920143d0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b93b56a166a432c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red45e2414db5481b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9086f44fc7244ea0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a61c5a88d244452"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2df75fc6ec26439a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4608a25adfaf4732"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdddea8df32f54f2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57e0341f189343c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Enforce completion gate and freeze experiment protocol
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R0ee9d4e1b2594185"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R12269e845b8047a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.06666666666666667</x:v>
+        <x:v>0.08333333333333333</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>270</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.07407407407407407</x:v>
+        <x:v>0.09259259259259259</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>18.166666666666668</x:v>
+        <x:v>17.833333333333332</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1302,7 +1302,7 @@
         <x:v>Set compute and spend limits</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E16" s="20" t="str">
         <x:v>TB-003</x:v>
@@ -1310,7 +1310,7 @@
       <x:c r="F16" s="20" t="str"/>
       <x:c r="G16" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E16="",TRUE,COUNTIFS($A$12:$A$71,E16)=1),IF(F16="",TRUE,COUNTIFS($A$12:$A$71,F16)=1))),"Bad dependency",IF(NOT(AND(IF(E16="",TRUE,COUNTIFS($A$12:$A$71,E16,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F16="",TRUE,COUNTIFS($A$12:$A$71,F16,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D16="Completed","Check prerequisites","Waiting"),IF(D16="Completed",IF(S16="","Evidence needed","Done"),IF(D16="Blocked","Blocked",IF(D16="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H16" s="27" t="n">
         <x:v>2</x:v>
@@ -1339,11 +1339,15 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R16" s="20" t="str"/>
-      <x:c r="S16" s="23" t="str"/>
-      <x:c r="T16" s="23" t="str"/>
+      <x:c r="S16" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/docs/budget-policy.md</x:v>
+      </x:c>
+      <x:c r="T16" s="23" t="str">
+        <x:v>Budget code and cancellation tests pass. Completion still requires one credentialed provider pilot with provider-reported token usage, measured elapsed time and execution-time pricing evidence.</x:v>
+      </x:c>
       <x:c r="U16" s="19" t="n">
         <x:f>IF(LEN(S16)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">
@@ -1357,7 +1361,7 @@
         <x:v>Freeze experiment protocol</x:v>
       </x:c>
       <x:c r="D17" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E17" s="19" t="str">
         <x:v>TB-002</x:v>
@@ -1367,7 +1371,7 @@
       </x:c>
       <x:c r="G17" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E17="",TRUE,COUNTIFS($A$12:$A$71,E17)=1),IF(F17="",TRUE,COUNTIFS($A$12:$A$71,F17)=1))),"Bad dependency",IF(NOT(AND(IF(E17="",TRUE,COUNTIFS($A$12:$A$71,E17,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F17="",TRUE,COUNTIFS($A$12:$A$71,F17,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D17="Completed","Check prerequisites","Waiting"),IF(D17="Completed",IF(S17="","Evidence needed","Done"),IF(D17="Blocked","Blocked",IF(D17="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H17" s="27" t="n">
         <x:v>4</x:v>
@@ -1396,11 +1400,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R17" s="19" t="str"/>
-      <x:c r="S17" s="23" t="str"/>
+      <x:c r="S17" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/protocol/preregister.md</x:v>
+      </x:c>
       <x:c r="T17" s="23" t="str"/>
       <x:c r="U17" s="19" t="n">
         <x:f>IF(LEN(S17)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
@@ -1422,7 +1428,7 @@
       <x:c r="F18" s="21" t="str"/>
       <x:c r="G18" s="21" t="str">
         <x:f>IF(NOT(AND(IF(E18="",TRUE,COUNTIFS($A$12:$A$71,E18)=1),IF(F18="",TRUE,COUNTIFS($A$12:$A$71,F18)=1))),"Bad dependency",IF(NOT(AND(IF(E18="",TRUE,COUNTIFS($A$12:$A$71,E18,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F18="",TRUE,COUNTIFS($A$12:$A$71,F18,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D18="Completed","Check prerequisites","Waiting"),IF(D18="Completed",IF(S18="","Evidence needed","Done"),IF(D18="Blocked","Blocked",IF(D18="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H18" s="26" t="n">
         <x:v>3</x:v>
@@ -4590,15 +4596,15 @@
       </x:c>
       <x:c r="C79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"Completed")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"In Progress")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"Blocked")</x:f>
@@ -4606,7 +4612,7 @@
       </x:c>
       <x:c r="G79" s="29" t="n">
         <x:f>IF(B79=0,0,C79/B79)</x:f>
-        <x:v>0.6666666666666666</x:v>
+        <x:v>0.8333333333333334</x:v>
       </x:c>
       <x:c r="H79" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A79)</x:f>
@@ -4614,11 +4620,11 @@
       </x:c>
       <x:c r="I79" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A79,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$G$12:$G$71,"Ready")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K79" s="2"/>
       <x:c r="L79" s="2"/>
@@ -4670,7 +4676,7 @@
       </x:c>
       <x:c r="J80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$G$12:$G$71,"Ready")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K80" s="2"/>
       <x:c r="L80" s="2"/>
@@ -7385,13 +7391,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red45e2414db5481b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9086f44fc7244ea0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a61c5a88d244452"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2df75fc6ec26439a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4608a25adfaf4732"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdddea8df32f54f2c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57e0341f189343c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bc2ee0c93b340b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f62413b1b864242"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cef43a355aa4973"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc6dce8846b4d05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6362250bdc8a47bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c7769dfe72b4751"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34fd9b02a52e4503"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Pin AgentDojo benchmark source and license
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R12269e845b8047a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R167e637ab2f84b99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.08333333333333333</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>266</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.09259259259259259</x:v>
+        <x:v>0.1111111111111111</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>17.833333333333332</x:v>
+        <x:v>17.583333333333332</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1420,7 +1420,7 @@
         <x:v>Acquire benchmark and permissions</x:v>
       </x:c>
       <x:c r="D18" s="22" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E18" s="21" t="str">
         <x:v>TB-006</x:v>
@@ -1428,7 +1428,7 @@
       <x:c r="F18" s="21" t="str"/>
       <x:c r="G18" s="21" t="str">
         <x:f>IF(NOT(AND(IF(E18="",TRUE,COUNTIFS($A$12:$A$71,E18)=1),IF(F18="",TRUE,COUNTIFS($A$12:$A$71,F18)=1))),"Bad dependency",IF(NOT(AND(IF(E18="",TRUE,COUNTIFS($A$12:$A$71,E18,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F18="",TRUE,COUNTIFS($A$12:$A$71,F18,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D18="Completed","Check prerequisites","Waiting"),IF(D18="Completed",IF(S18="","Evidence needed","Done"),IF(D18="Blocked","Blocked",IF(D18="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H18" s="26" t="n">
         <x:v>3</x:v>
@@ -1459,11 +1459,13 @@
       <x:c r="R18" s="21" t="str">
         <x:v>TB-S1</x:v>
       </x:c>
-      <x:c r="S18" s="22" t="str"/>
+      <x:c r="S18" s="22" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/data/manifest.json</x:v>
+      </x:c>
       <x:c r="T18" s="22" t="str"/>
       <x:c r="U18" s="19" t="n">
         <x:f>IF(LEN(S18)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
@@ -1485,7 +1487,7 @@
       <x:c r="F19" s="19" t="str"/>
       <x:c r="G19" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E19="",TRUE,COUNTIFS($A$12:$A$71,E19)=1),IF(F19="",TRUE,COUNTIFS($A$12:$A$71,F19)=1))),"Bad dependency",IF(NOT(AND(IF(E19="",TRUE,COUNTIFS($A$12:$A$71,E19,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F19="",TRUE,COUNTIFS($A$12:$A$71,F19,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D19="Completed","Check prerequisites","Waiting"),IF(D19="Completed",IF(S19="","Evidence needed","Done"),IF(D19="Blocked","Blocked",IF(D19="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H19" s="27" t="n">
         <x:v>5</x:v>
@@ -4648,11 +4650,11 @@
       </x:c>
       <x:c r="C80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Completed")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"In Progress")</x:f>
@@ -4664,7 +4666,7 @@
       </x:c>
       <x:c r="G80" s="30" t="n">
         <x:f>IF(B80=0,0,C80/B80)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.16666666666666666</x:v>
       </x:c>
       <x:c r="H80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80)</x:f>
@@ -4672,7 +4674,7 @@
       </x:c>
       <x:c r="I80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>24</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="J80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$G$12:$G$71,"Ready")</x:f>
@@ -7391,13 +7393,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bc2ee0c93b340b7"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f62413b1b864242"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cef43a355aa4973"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc6dce8846b4d05"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6362250bdc8a47bc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c7769dfe72b4751"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34fd9b02a52e4503"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cdaf4ca7ff14135"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f4cceae79f24087"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fffe64fafcd4351"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re40421a793614290"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bb462aaf8bc42df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3698d28898b54e94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5de6c9439ab9482a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete provider-backed budget pilot
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R167e637ab2f84b99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="Rf4f2eacf1b1d436a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.11666666666666667</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.1111111111111111</x:v>
+        <x:v>0.12962962962962962</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>17.583333333333332</x:v>
+        <x:v>17.416666666666668</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1302,7 +1302,7 @@
         <x:v>Set compute and spend limits</x:v>
       </x:c>
       <x:c r="D16" s="23" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E16" s="20" t="str">
         <x:v>TB-003</x:v>
@@ -1310,7 +1310,7 @@
       <x:c r="F16" s="20" t="str"/>
       <x:c r="G16" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E16="",TRUE,COUNTIFS($A$12:$A$71,E16)=1),IF(F16="",TRUE,COUNTIFS($A$12:$A$71,F16)=1))),"Bad dependency",IF(NOT(AND(IF(E16="",TRUE,COUNTIFS($A$12:$A$71,E16,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F16="",TRUE,COUNTIFS($A$12:$A$71,F16,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D16="Completed","Check prerequisites","Waiting"),IF(D16="Completed",IF(S16="","Evidence needed","Done"),IF(D16="Blocked","Blocked",IF(D16="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H16" s="27" t="n">
         <x:v>2</x:v>
@@ -1340,11 +1340,9 @@
       </x:c>
       <x:c r="R16" s="20" t="str"/>
       <x:c r="S16" s="23" t="str">
-        <x:v>/Volumes/MHRJ/TrustBench-AI/docs/budget-policy.md</x:v>
-      </x:c>
-      <x:c r="T16" s="23" t="str">
-        <x:v>Budget code and cancellation tests pass. Completion still requires one credentialed provider pilot with provider-reported token usage, measured elapsed time and execution-time pricing evidence.</x:v>
-      </x:c>
+        <x:v>/Volumes/MHRJ/TrustBench-AI/configs/budget.yaml</x:v>
+      </x:c>
+      <x:c r="T16" s="23"/>
       <x:c r="U16" s="19" t="n">
         <x:f>IF(LEN(S16)&gt;0,1,0)</x:f>
         <x:v>1</x:v>
@@ -4598,7 +4596,7 @@
       </x:c>
       <x:c r="C79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"Completed")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"Not Started")</x:f>
@@ -4606,7 +4604,7 @@
       </x:c>
       <x:c r="E79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"In Progress")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$D$12:$D$71,"Blocked")</x:f>
@@ -4614,7 +4612,7 @@
       </x:c>
       <x:c r="G79" s="29" t="n">
         <x:f>IF(B79=0,0,C79/B79)</x:f>
-        <x:v>0.8333333333333334</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H79" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A79)</x:f>
@@ -4622,7 +4620,7 @@
       </x:c>
       <x:c r="I79" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A79,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J79" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A79,$G$12:$G$71,"Ready")</x:f>
@@ -7393,13 +7391,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cdaf4ca7ff14135"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f4cceae79f24087"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fffe64fafcd4351"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re40421a793614290"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bb462aaf8bc42df"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3698d28898b54e94"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5de6c9439ab9482a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0e8cf75ca5e49c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365bd0dc69094f9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd437f457a0b47a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea6e58da315c409c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R868ef628a74242be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53487a1a802d4ff6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaf099f615c04b6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add synthetic benign task fixtures
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="Rf4f2eacf1b1d436a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R0bf8ae28b8cf49ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.11666666666666667</x:v>
+        <x:v>0.13333333333333333</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>261</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.12962962962962962</x:v>
+        <x:v>0.14814814814814814</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>17.416666666666668</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1477,7 +1477,7 @@
         <x:v>Create local benign task set</x:v>
       </x:c>
       <x:c r="D19" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E19" s="19" t="str">
         <x:v>TB-007</x:v>
@@ -1485,7 +1485,7 @@
       <x:c r="F19" s="19" t="str"/>
       <x:c r="G19" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E19="",TRUE,COUNTIFS($A$12:$A$71,E19)=1),IF(F19="",TRUE,COUNTIFS($A$12:$A$71,F19)=1))),"Bad dependency",IF(NOT(AND(IF(E19="",TRUE,COUNTIFS($A$12:$A$71,E19,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F19="",TRUE,COUNTIFS($A$12:$A$71,F19,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D19="Completed","Check prerequisites","Waiting"),IF(D19="Completed",IF(S19="","Evidence needed","Done"),IF(D19="Blocked","Blocked",IF(D19="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H19" s="27" t="n">
         <x:v>5</x:v>
@@ -1514,11 +1514,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R19" s="19" t="str"/>
-      <x:c r="S19" s="23" t="str"/>
-      <x:c r="T19" s="23" t="str"/>
+      <x:c r="S19" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/data/benign.jsonl</x:v>
+      </x:c>
+      <x:c r="T19" s="23"/>
       <x:c r="U19" s="19" t="n">
         <x:f>IF(LEN(S19)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="64" customHeight="1">
@@ -1542,7 +1544,7 @@
       </x:c>
       <x:c r="G20" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E20="",TRUE,COUNTIFS($A$12:$A$71,E20)=1),IF(F20="",TRUE,COUNTIFS($A$12:$A$71,F20)=1))),"Bad dependency",IF(NOT(AND(IF(E20="",TRUE,COUNTIFS($A$12:$A$71,E20,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F20="",TRUE,COUNTIFS($A$12:$A$71,F20,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D20="Completed","Check prerequisites","Waiting"),IF(D20="Completed",IF(S20="","Evidence needed","Done"),IF(D20="Blocked","Blocked",IF(D20="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H20" s="27" t="n">
         <x:v>5</x:v>
@@ -4648,11 +4650,11 @@
       </x:c>
       <x:c r="C80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Completed")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"In Progress")</x:f>
@@ -4664,7 +4666,7 @@
       </x:c>
       <x:c r="G80" s="30" t="n">
         <x:f>IF(B80=0,0,C80/B80)</x:f>
-        <x:v>0.16666666666666666</x:v>
+        <x:v>0.3333333333333333</x:v>
       </x:c>
       <x:c r="H80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80)</x:f>
@@ -4672,7 +4674,7 @@
       </x:c>
       <x:c r="I80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>21</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$G$12:$G$71,"Ready")</x:f>
@@ -7391,13 +7393,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0e8cf75ca5e49c4"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365bd0dc69094f9c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd437f457a0b47a0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea6e58da315c409c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R868ef628a74242be"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53487a1a802d4ff6"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaf099f615c04b6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88909aa2cc8949b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ec3ec7826334d3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd162a523246a437b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7934f52de527402e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b573d9f7d2943a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cd794a4987e468d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8524b5f700204d16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add attack fixtures and locked evaluation split
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R0bf8ae28b8cf49ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R7dd6f0e5233f41eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.13333333333333333</x:v>
+        <x:v>0.16666666666666666</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>256</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.14814814814814814</x:v>
+        <x:v>0.18518518518518517</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>17</x:v>
+        <x:v>16.25</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1534,7 +1534,7 @@
         <x:v>Build controlled injection fixtures</x:v>
       </x:c>
       <x:c r="D20" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E20" s="20" t="str">
         <x:v>TB-002</x:v>
@@ -1544,7 +1544,7 @@
       </x:c>
       <x:c r="G20" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E20="",TRUE,COUNTIFS($A$12:$A$71,E20)=1),IF(F20="",TRUE,COUNTIFS($A$12:$A$71,F20)=1))),"Bad dependency",IF(NOT(AND(IF(E20="",TRUE,COUNTIFS($A$12:$A$71,E20,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F20="",TRUE,COUNTIFS($A$12:$A$71,F20,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D20="Completed","Check prerequisites","Waiting"),IF(D20="Completed",IF(S20="","Evidence needed","Done"),IF(D20="Blocked","Blocked",IF(D20="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H20" s="27" t="n">
         <x:v>5</x:v>
@@ -1573,11 +1573,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R20" s="20" t="str"/>
-      <x:c r="S20" s="23" t="str"/>
-      <x:c r="T20" s="23" t="str"/>
+      <x:c r="S20" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/data/attacks.jsonl</x:v>
+      </x:c>
+      <x:c r="T20" s="23"/>
       <x:c r="U20" s="19" t="n">
         <x:f>IF(LEN(S20)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="64" customHeight="1">
@@ -1591,7 +1593,7 @@
         <x:v>Separate tuning and holdout families</x:v>
       </x:c>
       <x:c r="D21" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E21" s="19" t="str">
         <x:v>TB-009</x:v>
@@ -1599,7 +1601,7 @@
       <x:c r="F21" s="19" t="str"/>
       <x:c r="G21" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E21="",TRUE,COUNTIFS($A$12:$A$71,E21)=1),IF(F21="",TRUE,COUNTIFS($A$12:$A$71,F21)=1))),"Bad dependency",IF(NOT(AND(IF(E21="",TRUE,COUNTIFS($A$12:$A$71,E21,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F21="",TRUE,COUNTIFS($A$12:$A$71,F21,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D21="Completed","Check prerequisites","Waiting"),IF(D21="Completed",IF(S21="","Evidence needed","Done"),IF(D21="Blocked","Blocked",IF(D21="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H21" s="27" t="n">
         <x:v>4</x:v>
@@ -1628,11 +1630,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R21" s="19" t="str"/>
-      <x:c r="S21" s="23" t="str"/>
-      <x:c r="T21" s="23" t="str"/>
+      <x:c r="S21" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/data/splits.json</x:v>
+      </x:c>
+      <x:c r="T21" s="23"/>
       <x:c r="U21" s="19" t="n">
         <x:f>IF(LEN(S21)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="64" customHeight="1">
@@ -1654,7 +1658,7 @@
       <x:c r="F22" s="20" t="str"/>
       <x:c r="G22" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E22="",TRUE,COUNTIFS($A$12:$A$71,E22)=1),IF(F22="",TRUE,COUNTIFS($A$12:$A$71,F22)=1))),"Bad dependency",IF(NOT(AND(IF(E22="",TRUE,COUNTIFS($A$12:$A$71,E22,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F22="",TRUE,COUNTIFS($A$12:$A$71,F22,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D22="Completed","Check prerequisites","Waiting"),IF(D22="Completed",IF(S22="","Evidence needed","Done"),IF(D22="Blocked","Blocked",IF(D22="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H22" s="27" t="n">
         <x:v>4</x:v>
@@ -4650,11 +4654,11 @@
       </x:c>
       <x:c r="C80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Completed")</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"In Progress")</x:f>
@@ -4666,7 +4670,7 @@
       </x:c>
       <x:c r="G80" s="30" t="n">
         <x:f>IF(B80=0,0,C80/B80)</x:f>
-        <x:v>0.3333333333333333</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="H80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80)</x:f>
@@ -4674,7 +4678,7 @@
       </x:c>
       <x:c r="I80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>16</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="J80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$G$12:$G$71,"Ready")</x:f>
@@ -7393,13 +7397,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88909aa2cc8949b6"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ec3ec7826334d3b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd162a523246a437b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7934f52de527402e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b573d9f7d2943a5"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cd794a4987e468d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8524b5f700204d16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R779b6277e60d46d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28606ed737dd4290"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd755c0a152e94077"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53e6fa4f565346af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3598cd6740f94c6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd7b11167a1a43db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc91ca78adad74425"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify dataset labels and episode resets
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R7dd6f0e5233f41eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R0ce9e7f58c0a4166"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.16666666666666666</x:v>
+        <x:v>0.18333333333333332</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>247</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.18518518518518517</x:v>
+        <x:v>0.2037037037037037</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>16.25</x:v>
+        <x:v>15.916666666666666</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1650,7 +1650,7 @@
         <x:v>Validate dataset and reset semantics</x:v>
       </x:c>
       <x:c r="D22" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E22" s="20" t="str">
         <x:v>TB-010</x:v>
@@ -1658,7 +1658,7 @@
       <x:c r="F22" s="20" t="str"/>
       <x:c r="G22" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E22="",TRUE,COUNTIFS($A$12:$A$71,E22)=1),IF(F22="",TRUE,COUNTIFS($A$12:$A$71,F22)=1))),"Bad dependency",IF(NOT(AND(IF(E22="",TRUE,COUNTIFS($A$12:$A$71,E22,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F22="",TRUE,COUNTIFS($A$12:$A$71,F22,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D22="Completed","Check prerequisites","Waiting"),IF(D22="Completed",IF(S22="","Evidence needed","Done"),IF(D22="Blocked","Blocked",IF(D22="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H22" s="27" t="n">
         <x:v>4</x:v>
@@ -1687,11 +1687,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R22" s="20" t="str"/>
-      <x:c r="S22" s="23" t="str"/>
-      <x:c r="T22" s="23" t="str"/>
+      <x:c r="S22" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/reports/data-validation.json</x:v>
+      </x:c>
+      <x:c r="T22" s="23"/>
       <x:c r="U22" s="19" t="n">
         <x:f>IF(LEN(S22)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="64" customHeight="1">
@@ -1713,7 +1715,7 @@
       <x:c r="F23" s="19" t="str"/>
       <x:c r="G23" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E23="",TRUE,COUNTIFS($A$12:$A$71,E23)=1),IF(F23="",TRUE,COUNTIFS($A$12:$A$71,F23)=1))),"Bad dependency",IF(NOT(AND(IF(E23="",TRUE,COUNTIFS($A$12:$A$71,E23,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F23="",TRUE,COUNTIFS($A$12:$A$71,F23,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D23="Completed","Check prerequisites","Waiting"),IF(D23="Completed",IF(S23="","Evidence needed","Done"),IF(D23="Blocked","Blocked",IF(D23="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H23" s="27" t="n">
         <x:v>3</x:v>
@@ -4654,11 +4656,11 @@
       </x:c>
       <x:c r="C80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Completed")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"In Progress")</x:f>
@@ -4670,7 +4672,7 @@
       </x:c>
       <x:c r="G80" s="30" t="n">
         <x:f>IF(B80=0,0,C80/B80)</x:f>
-        <x:v>0.6666666666666666</x:v>
+        <x:v>0.8333333333333334</x:v>
       </x:c>
       <x:c r="H80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80)</x:f>
@@ -4678,7 +4680,7 @@
       </x:c>
       <x:c r="I80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$G$12:$G$71,"Ready")</x:f>
@@ -7397,13 +7399,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R779b6277e60d46d3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28606ed737dd4290"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd755c0a152e94077"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53e6fa4f565346af"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3598cd6740f94c6e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd7b11167a1a43db"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc91ca78adad74425"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9df34653f81d4d21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dcc246d22c64cd8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5dfc374b3d14d84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f96adf74be945cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f587023e17d40a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2d4aa6258614135"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90c78df4f76b41be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add offline end-to-end smoke suite
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R0ce9e7f58c0a4166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R4f5b2c90e457421e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.18333333333333332</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>243</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.2037037037037037</x:v>
+        <x:v>0.2222222222222222</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>15.916666666666666</x:v>
+        <x:v>15.666666666666666</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1707,7 +1707,7 @@
         <x:v>Create small end-to-end smoke suite</x:v>
       </x:c>
       <x:c r="D23" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E23" s="19" t="str">
         <x:v>TB-011</x:v>
@@ -1715,7 +1715,7 @@
       <x:c r="F23" s="19" t="str"/>
       <x:c r="G23" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E23="",TRUE,COUNTIFS($A$12:$A$71,E23)=1),IF(F23="",TRUE,COUNTIFS($A$12:$A$71,F23)=1))),"Bad dependency",IF(NOT(AND(IF(E23="",TRUE,COUNTIFS($A$12:$A$71,E23,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F23="",TRUE,COUNTIFS($A$12:$A$71,F23,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D23="Completed","Check prerequisites","Waiting"),IF(D23="Completed",IF(S23="","Evidence needed","Done"),IF(D23="Blocked","Blocked",IF(D23="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H23" s="27" t="n">
         <x:v>3</x:v>
@@ -1744,11 +1744,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R23" s="19" t="str"/>
-      <x:c r="S23" s="23" t="str"/>
-      <x:c r="T23" s="23" t="str"/>
+      <x:c r="S23" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/tests/smoke/report.json</x:v>
+      </x:c>
+      <x:c r="T23" s="23"/>
       <x:c r="U23" s="19" t="n">
         <x:f>IF(LEN(S23)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="64" customHeight="1">
@@ -1770,7 +1772,7 @@
       <x:c r="F24" s="21" t="str"/>
       <x:c r="G24" s="21" t="str">
         <x:f>IF(NOT(AND(IF(E24="",TRUE,COUNTIFS($A$12:$A$71,E24)=1),IF(F24="",TRUE,COUNTIFS($A$12:$A$71,F24)=1))),"Bad dependency",IF(NOT(AND(IF(E24="",TRUE,COUNTIFS($A$12:$A$71,E24,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F24="",TRUE,COUNTIFS($A$12:$A$71,F24,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D24="Completed","Check prerequisites","Waiting"),IF(D24="Completed",IF(S24="","Evidence needed","Done"),IF(D24="Blocked","Blocked",IF(D24="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H24" s="26" t="n">
         <x:v>4</x:v>
@@ -4656,11 +4658,11 @@
       </x:c>
       <x:c r="C80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Completed")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$D$12:$D$71,"In Progress")</x:f>
@@ -4672,7 +4674,7 @@
       </x:c>
       <x:c r="G80" s="30" t="n">
         <x:f>IF(B80=0,0,C80/B80)</x:f>
-        <x:v>0.8333333333333334</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80)</x:f>
@@ -4680,11 +4682,11 @@
       </x:c>
       <x:c r="I80" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A80,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J80" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A80,$G$12:$G$71,"Ready")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K80" s="2"/>
       <x:c r="L80" s="2"/>
@@ -4736,7 +4738,7 @@
       </x:c>
       <x:c r="J81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$G$12:$G$71,"Ready")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K81" s="2"/>
       <x:c r="L81" s="2"/>
@@ -7399,13 +7401,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9df34653f81d4d21"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dcc246d22c64cd8"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5dfc374b3d14d84"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f96adf74be945cb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f587023e17d40a7"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2d4aa6258614135"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90c78df4f76b41be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78f4185b5b8448fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb884a7ddb68a4413"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae22ea264a34e9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da3f48df53f4bba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5caf5b2b47744a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree393a0458c24c4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R468c82279fd74f57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add provider-neutral model adapter
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R4f5b2c90e457421e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="Rd843e72864c84ad7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.2</x:v>
+        <x:v>0.21666666666666667</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>240</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.2222222222222222</x:v>
+        <x:v>0.24074074074074073</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>15.666666666666666</x:v>
+        <x:v>15.333333333333334</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1764,7 +1764,7 @@
         <x:v>Implement provider-neutral model adapter</x:v>
       </x:c>
       <x:c r="D24" s="22" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E24" s="21" t="str">
         <x:v>TB-012</x:v>
@@ -1772,7 +1772,7 @@
       <x:c r="F24" s="21" t="str"/>
       <x:c r="G24" s="21" t="str">
         <x:f>IF(NOT(AND(IF(E24="",TRUE,COUNTIFS($A$12:$A$71,E24)=1),IF(F24="",TRUE,COUNTIFS($A$12:$A$71,F24)=1))),"Bad dependency",IF(NOT(AND(IF(E24="",TRUE,COUNTIFS($A$12:$A$71,E24,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F24="",TRUE,COUNTIFS($A$12:$A$71,F24,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D24="Completed","Check prerequisites","Waiting"),IF(D24="Completed",IF(S24="","Evidence needed","Done"),IF(D24="Blocked","Blocked",IF(D24="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H24" s="26" t="n">
         <x:v>4</x:v>
@@ -1801,11 +1801,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R24" s="21" t="str"/>
-      <x:c r="S24" s="22" t="str"/>
-      <x:c r="T24" s="22" t="str"/>
+      <x:c r="S24" s="22" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/artifacts/verification/tb013-model-adapter.json</x:v>
+      </x:c>
+      <x:c r="T24" s="22"/>
       <x:c r="U24" s="19" t="n">
         <x:f>IF(LEN(S24)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="64" customHeight="1">
@@ -1827,7 +1829,7 @@
       <x:c r="F25" s="19" t="str"/>
       <x:c r="G25" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E25="",TRUE,COUNTIFS($A$12:$A$71,E25)=1),IF(F25="",TRUE,COUNTIFS($A$12:$A$71,F25)=1))),"Bad dependency",IF(NOT(AND(IF(E25="",TRUE,COUNTIFS($A$12:$A$71,E25,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F25="",TRUE,COUNTIFS($A$12:$A$71,F25,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D25="Completed","Check prerequisites","Waiting"),IF(D25="Completed",IF(S25="","Evidence needed","Done"),IF(D25="Blocked","Blocked",IF(D25="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H25" s="27" t="n">
         <x:v>6</x:v>
@@ -4710,11 +4712,11 @@
       </x:c>
       <x:c r="C81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Completed")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"In Progress")</x:f>
@@ -4726,7 +4728,7 @@
       </x:c>
       <x:c r="G81" s="29" t="n">
         <x:f>IF(B81=0,0,C81/B81)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.16666666666666666</x:v>
       </x:c>
       <x:c r="H81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81)</x:f>
@@ -4734,7 +4736,7 @@
       </x:c>
       <x:c r="I81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="J81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$G$12:$G$71,"Ready")</x:f>
@@ -7401,13 +7403,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78f4185b5b8448fd"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb884a7ddb68a4413"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae22ea264a34e9e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da3f48df53f4bba"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5caf5b2b47744a6"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree393a0458c24c4a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R468c82279fd74f57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R343ffeb7dd4d4f7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44e089ee344f4572"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79a66ccc8e65453c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0abb8b5111c4914"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d63cf36c99e44fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R621c473085194f8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2c8c911817344ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add isolated synthetic tool services
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="Rd843e72864c84ad7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R46e7b9077392405d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.21666666666666667</x:v>
+        <x:v>0.23333333333333334</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>236</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.24074074074074073</x:v>
+        <x:v>0.25925925925925924</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>15.333333333333334</x:v>
+        <x:v>14.833333333333334</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1821,7 +1821,7 @@
         <x:v>Implement isolated tool services</x:v>
       </x:c>
       <x:c r="D25" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E25" s="19" t="str">
         <x:v>TB-013</x:v>
@@ -1829,7 +1829,7 @@
       <x:c r="F25" s="19" t="str"/>
       <x:c r="G25" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E25="",TRUE,COUNTIFS($A$12:$A$71,E25)=1),IF(F25="",TRUE,COUNTIFS($A$12:$A$71,F25)=1))),"Bad dependency",IF(NOT(AND(IF(E25="",TRUE,COUNTIFS($A$12:$A$71,E25,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F25="",TRUE,COUNTIFS($A$12:$A$71,F25,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D25="Completed","Check prerequisites","Waiting"),IF(D25="Completed",IF(S25="","Evidence needed","Done"),IF(D25="Blocked","Blocked",IF(D25="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H25" s="27" t="n">
         <x:v>6</x:v>
@@ -1858,11 +1858,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R25" s="19" t="str"/>
-      <x:c r="S25" s="23" t="str"/>
-      <x:c r="T25" s="23" t="str"/>
+      <x:c r="S25" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/evidence/tb014-tool-service-report.json; /Volumes/MHRJ/TrustBench-AI/src/tools/; /Volumes/MHRJ/TrustBench-AI/agent/sandbox.ts; /Volumes/MHRJ/TrustBench-AI/agent/sandbox/Dockerfile</x:v>
+      </x:c>
+      <x:c r="T25" s="23"/>
       <x:c r="U25" s="19" t="n">
         <x:f>IF(LEN(S25)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="64" customHeight="1">
@@ -1884,7 +1886,7 @@
       <x:c r="F26" s="20" t="str"/>
       <x:c r="G26" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E26="",TRUE,COUNTIFS($A$12:$A$71,E26)=1),IF(F26="",TRUE,COUNTIFS($A$12:$A$71,F26)=1))),"Bad dependency",IF(NOT(AND(IF(E26="",TRUE,COUNTIFS($A$12:$A$71,E26,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F26="",TRUE,COUNTIFS($A$12:$A$71,F26,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D26="Completed","Check prerequisites","Waiting"),IF(D26="Completed",IF(S26="","Evidence needed","Done"),IF(D26="Blocked","Blocked",IF(D26="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H26" s="27" t="n">
         <x:v>5</x:v>
@@ -4712,11 +4714,11 @@
       </x:c>
       <x:c r="C81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Completed")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"In Progress")</x:f>
@@ -4728,7 +4730,7 @@
       </x:c>
       <x:c r="G81" s="29" t="n">
         <x:f>IF(B81=0,0,C81/B81)</x:f>
-        <x:v>0.16666666666666666</x:v>
+        <x:v>0.3333333333333333</x:v>
       </x:c>
       <x:c r="H81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81)</x:f>
@@ -4736,7 +4738,7 @@
       </x:c>
       <x:c r="I81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>23</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="J81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$G$12:$G$71,"Ready")</x:f>
@@ -7403,13 +7405,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R343ffeb7dd4d4f7a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44e089ee344f4572"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79a66ccc8e65453c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0abb8b5111c4914"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d63cf36c99e44fc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R621c473085194f8f"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2c8c911817344ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f97c66f2bcc4dda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f8ebee3c6664412"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f3d43fe58994833"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcd94d7a6a484588"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4102b70d6e1347c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10e14d536d4b4e60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re04fa8a51d5540ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add bounded baseline agent state machine
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R46e7b9077392405d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R1376721797ad4b7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.23333333333333334</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>230</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.25925925925925924</x:v>
+        <x:v>0.2777777777777778</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>14.833333333333334</x:v>
+        <x:v>14.416666666666666</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1878,7 +1878,7 @@
         <x:v>Build bounded baseline agent</x:v>
       </x:c>
       <x:c r="D26" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E26" s="20" t="str">
         <x:v>TB-014</x:v>
@@ -1886,7 +1886,7 @@
       <x:c r="F26" s="20" t="str"/>
       <x:c r="G26" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E26="",TRUE,COUNTIFS($A$12:$A$71,E26)=1),IF(F26="",TRUE,COUNTIFS($A$12:$A$71,F26)=1))),"Bad dependency",IF(NOT(AND(IF(E26="",TRUE,COUNTIFS($A$12:$A$71,E26,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F26="",TRUE,COUNTIFS($A$12:$A$71,F26,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D26="Completed","Check prerequisites","Waiting"),IF(D26="Completed",IF(S26="","Evidence needed","Done"),IF(D26="Blocked","Blocked",IF(D26="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H26" s="27" t="n">
         <x:v>5</x:v>
@@ -1917,11 +1917,13 @@
       <x:c r="R26" s="20" t="str">
         <x:v>TB-S3</x:v>
       </x:c>
-      <x:c r="S26" s="23" t="str"/>
-      <x:c r="T26" s="23" t="str"/>
+      <x:c r="S26" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/evidence/tb015-baseline-agent-report.json; /Volumes/MHRJ/TrustBench-AI/src/agent/</x:v>
+      </x:c>
+      <x:c r="T26" s="23"/>
       <x:c r="U26" s="19" t="n">
         <x:f>IF(LEN(S26)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="64" customHeight="1">
@@ -1943,7 +1945,7 @@
       <x:c r="F27" s="19" t="str"/>
       <x:c r="G27" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E27="",TRUE,COUNTIFS($A$12:$A$71,E27)=1),IF(F27="",TRUE,COUNTIFS($A$12:$A$71,F27)=1))),"Bad dependency",IF(NOT(AND(IF(E27="",TRUE,COUNTIFS($A$12:$A$71,E27,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F27="",TRUE,COUNTIFS($A$12:$A$71,F27,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D27="Completed","Check prerequisites","Waiting"),IF(D27="Completed",IF(S27="","Evidence needed","Done"),IF(D27="Blocked","Blocked",IF(D27="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H27" s="27" t="n">
         <x:v>5</x:v>
@@ -4714,11 +4716,11 @@
       </x:c>
       <x:c r="C81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Completed")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"In Progress")</x:f>
@@ -4730,7 +4732,7 @@
       </x:c>
       <x:c r="G81" s="29" t="n">
         <x:f>IF(B81=0,0,C81/B81)</x:f>
-        <x:v>0.3333333333333333</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="H81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81)</x:f>
@@ -4738,7 +4740,7 @@
       </x:c>
       <x:c r="I81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>17</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="J81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$G$12:$G$71,"Ready")</x:f>
@@ -7405,13 +7407,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f97c66f2bcc4dda"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f8ebee3c6664412"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f3d43fe58994833"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcd94d7a6a484588"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4102b70d6e1347c2"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10e14d536d4b4e60"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re04fa8a51d5540ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f07270a883e45ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7255cae530364a53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeadbf4027e3456b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc7d521b85cf432d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15b27ce50ccb42a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c358095d36e44b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R627567534e224ee0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add independent outcome evaluators
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R1376721797ad4b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R1481ff0a8b844d62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.26666666666666666</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>225</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.2777777777777778</x:v>
+        <x:v>0.2962962962962963</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>14.416666666666666</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1937,7 +1937,7 @@
         <x:v>Add independent outcome evaluators</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E27" s="19" t="str">
         <x:v>TB-015</x:v>
@@ -1945,7 +1945,7 @@
       <x:c r="F27" s="19" t="str"/>
       <x:c r="G27" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E27="",TRUE,COUNTIFS($A$12:$A$71,E27)=1),IF(F27="",TRUE,COUNTIFS($A$12:$A$71,F27)=1))),"Bad dependency",IF(NOT(AND(IF(E27="",TRUE,COUNTIFS($A$12:$A$71,E27,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F27="",TRUE,COUNTIFS($A$12:$A$71,F27,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D27="Completed","Check prerequisites","Waiting"),IF(D27="Completed",IF(S27="","Evidence needed","Done"),IF(D27="Blocked","Blocked",IF(D27="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H27" s="27" t="n">
         <x:v>5</x:v>
@@ -1974,11 +1974,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R27" s="19" t="str"/>
-      <x:c r="S27" s="23" t="str"/>
-      <x:c r="T27" s="23" t="str"/>
+      <x:c r="S27" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/evidence/tb016-evaluator-report.json; /Volumes/MHRJ/TrustBench-AI/src/evaluators/; /Volumes/MHRJ/TrustBench-AI/tests/evaluators/</x:v>
+      </x:c>
+      <x:c r="T27" s="23"/>
       <x:c r="U27" s="19" t="n">
         <x:f>IF(LEN(S27)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="64" customHeight="1">
@@ -2002,7 +2004,7 @@
       </x:c>
       <x:c r="G28" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E28="",TRUE,COUNTIFS($A$12:$A$71,E28)=1),IF(F28="",TRUE,COUNTIFS($A$12:$A$71,F28)=1))),"Bad dependency",IF(NOT(AND(IF(E28="",TRUE,COUNTIFS($A$12:$A$71,E28,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F28="",TRUE,COUNTIFS($A$12:$A$71,F28,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D28="Completed","Check prerequisites","Waiting"),IF(D28="Completed",IF(S28="","Evidence needed","Done"),IF(D28="Blocked","Blocked",IF(D28="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H28" s="27" t="n">
         <x:v>4</x:v>
@@ -4716,11 +4718,11 @@
       </x:c>
       <x:c r="C81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Completed")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"In Progress")</x:f>
@@ -4732,7 +4734,7 @@
       </x:c>
       <x:c r="G81" s="29" t="n">
         <x:f>IF(B81=0,0,C81/B81)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="H81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81)</x:f>
@@ -4740,7 +4742,7 @@
       </x:c>
       <x:c r="I81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>12</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="J81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$G$12:$G$71,"Ready")</x:f>
@@ -7407,13 +7409,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f07270a883e45ca"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7255cae530364a53"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeadbf4027e3456b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc7d521b85cf432d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15b27ce50ccb42a0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c358095d36e44b4"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R627567534e224ee0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9de72e209bbd4f33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cae7b805c854282"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re373972882394892"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25260fbcac0449e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cd04cb7061944d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ff8b7548262446b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4b0d49849f447b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Run provider-backed baseline pilot
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R1481ff0a8b844d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R9e4e24bb5ae245c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.26666666666666666</x:v>
+        <x:v>0.2833333333333333</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>220</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.2962962962962963</x:v>
+        <x:v>0.3148148148148148</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>14</x:v>
+        <x:v>13.666666666666666</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -1994,7 +1994,7 @@
         <x:v>Run and store baseline pilot</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E28" s="20" t="str">
         <x:v>TB-016</x:v>
@@ -2004,7 +2004,7 @@
       </x:c>
       <x:c r="G28" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E28="",TRUE,COUNTIFS($A$12:$A$71,E28)=1),IF(F28="",TRUE,COUNTIFS($A$12:$A$71,F28)=1))),"Bad dependency",IF(NOT(AND(IF(E28="",TRUE,COUNTIFS($A$12:$A$71,E28,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F28="",TRUE,COUNTIFS($A$12:$A$71,F28,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D28="Completed","Check prerequisites","Waiting"),IF(D28="Completed",IF(S28="","Evidence needed","Done"),IF(D28="Blocked","Blocked",IF(D28="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H28" s="27" t="n">
         <x:v>4</x:v>
@@ -2033,11 +2033,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R28" s="20" t="str"/>
-      <x:c r="S28" s="23" t="str"/>
-      <x:c r="T28" s="23" t="str"/>
+      <x:c r="S28" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/runs/baseline-pilot/</x:v>
+      </x:c>
+      <x:c r="T28" s="23"/>
       <x:c r="U28" s="19" t="n">
         <x:f>IF(LEN(S28)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="64" customHeight="1">
@@ -2059,7 +2061,7 @@
       <x:c r="F29" s="19" t="str"/>
       <x:c r="G29" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E29="",TRUE,COUNTIFS($A$12:$A$71,E29)=1),IF(F29="",TRUE,COUNTIFS($A$12:$A$71,F29)=1))),"Bad dependency",IF(NOT(AND(IF(E29="",TRUE,COUNTIFS($A$12:$A$71,E29,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F29="",TRUE,COUNTIFS($A$12:$A$71,F29,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D29="Completed","Check prerequisites","Waiting"),IF(D29="Completed",IF(S29="","Evidence needed","Done"),IF(D29="Blocked","Blocked",IF(D29="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H29" s="27" t="n">
         <x:v>3</x:v>
@@ -4718,11 +4720,11 @@
       </x:c>
       <x:c r="C81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Completed")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"In Progress")</x:f>
@@ -4734,7 +4736,7 @@
       </x:c>
       <x:c r="G81" s="29" t="n">
         <x:f>IF(B81=0,0,C81/B81)</x:f>
-        <x:v>0.6666666666666666</x:v>
+        <x:v>0.8333333333333334</x:v>
       </x:c>
       <x:c r="H81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81)</x:f>
@@ -4742,7 +4744,7 @@
       </x:c>
       <x:c r="I81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$G$12:$G$71,"Ready")</x:f>
@@ -7409,13 +7411,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9de72e209bbd4f33"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cae7b805c854282"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re373972882394892"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25260fbcac0449e4"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cd04cb7061944d0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ff8b7548262446b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4b0d49849f447b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2965005f7ae44ba4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9412a037148349f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f510be1879e4fc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebbf1d4a123f4bc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R692fb2a21eb84840"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ef0c3b5bee04d17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f88c3b26e264c0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Review pilot failures and add gateway provenance boundary
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R9e4e24bb5ae245c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TrustBench-AI" sheetId="1" r:id="R52b7b39f0f8045f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,11 +811,11 @@
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Completed")</x:f>
-        <x:v>17</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>IF(A5=0,0,B5/A5)</x:f>
-        <x:v>0.2833333333333333</x:v>
+        <x:v>0.3333333333333333</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:f>COUNTIFS($D$12:$D$71,"Blocked")</x:f>
@@ -827,15 +827,15 @@
       </x:c>
       <x:c r="F5" s="12" t="n">
         <x:f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>216</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
         <x:f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</x:f>
-        <x:v>0.3148148148148148</x:v>
+        <x:v>0.37037037037037035</x:v>
       </x:c>
       <x:c r="H5" s="14" t="n">
         <x:f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</x:f>
-        <x:v>13.666666666666666</x:v>
+        <x:v>12.416666666666666</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
         <x:f>COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</x:f>
@@ -2053,7 +2053,7 @@
         <x:v>Review failure taxonomy</x:v>
       </x:c>
       <x:c r="D29" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E29" s="19" t="str">
         <x:v>TB-017</x:v>
@@ -2061,7 +2061,7 @@
       <x:c r="F29" s="19" t="str"/>
       <x:c r="G29" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E29="",TRUE,COUNTIFS($A$12:$A$71,E29)=1),IF(F29="",TRUE,COUNTIFS($A$12:$A$71,F29)=1))),"Bad dependency",IF(NOT(AND(IF(E29="",TRUE,COUNTIFS($A$12:$A$71,E29,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F29="",TRUE,COUNTIFS($A$12:$A$71,F29,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D29="Completed","Check prerequisites","Waiting"),IF(D29="Completed",IF(S29="","Evidence needed","Done"),IF(D29="Blocked","Blocked",IF(D29="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H29" s="27" t="n">
         <x:v>3</x:v>
@@ -2090,11 +2090,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R29" s="19" t="str"/>
-      <x:c r="S29" s="23" t="str"/>
-      <x:c r="T29" s="23" t="str"/>
+      <x:c r="S29" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/reports/failure-taxonomy.csv; /Volumes/MHRJ/TrustBench-AI/reports/failure-review.ipynb; /Volumes/MHRJ/TrustBench-AI/reports/tb018-review-summary.json</x:v>
+      </x:c>
+      <x:c r="T29" s="23"/>
       <x:c r="U29" s="19" t="n">
         <x:f>IF(LEN(S29)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="64" customHeight="1">
@@ -2108,7 +2110,7 @@
         <x:v>Implement centralized tool interception</x:v>
       </x:c>
       <x:c r="D30" s="22" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E30" s="21" t="str">
         <x:v>TB-018</x:v>
@@ -2116,7 +2118,7 @@
       <x:c r="F30" s="21" t="str"/>
       <x:c r="G30" s="21" t="str">
         <x:f>IF(NOT(AND(IF(E30="",TRUE,COUNTIFS($A$12:$A$71,E30)=1),IF(F30="",TRUE,COUNTIFS($A$12:$A$71,F30)=1))),"Bad dependency",IF(NOT(AND(IF(E30="",TRUE,COUNTIFS($A$12:$A$71,E30,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F30="",TRUE,COUNTIFS($A$12:$A$71,F30,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D30="Completed","Check prerequisites","Waiting"),IF(D30="Completed",IF(S30="","Evidence needed","Done"),IF(D30="Blocked","Blocked",IF(D30="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H30" s="26" t="n">
         <x:v>6</x:v>
@@ -2145,11 +2147,13 @@
         <x:v>Core</x:v>
       </x:c>
       <x:c r="R30" s="21" t="str"/>
-      <x:c r="S30" s="22" t="str"/>
-      <x:c r="T30" s="22" t="str"/>
+      <x:c r="S30" s="22" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/src/gateway/; /Volumes/MHRJ/TrustBench-AI/reports/tb019-gateway-tests.xml</x:v>
+      </x:c>
+      <x:c r="T30" s="22"/>
       <x:c r="U30" s="19" t="n">
         <x:f>IF(LEN(S30)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="64" customHeight="1">
@@ -2163,7 +2167,7 @@
         <x:v>Track provenance through tool outputs</x:v>
       </x:c>
       <x:c r="D31" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E31" s="19" t="str">
         <x:v>TB-019</x:v>
@@ -2171,7 +2175,7 @@
       <x:c r="F31" s="19" t="str"/>
       <x:c r="G31" s="19" t="str">
         <x:f>IF(NOT(AND(IF(E31="",TRUE,COUNTIFS($A$12:$A$71,E31)=1),IF(F31="",TRUE,COUNTIFS($A$12:$A$71,F31)=1))),"Bad dependency",IF(NOT(AND(IF(E31="",TRUE,COUNTIFS($A$12:$A$71,E31,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F31="",TRUE,COUNTIFS($A$12:$A$71,F31,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D31="Completed","Check prerequisites","Waiting"),IF(D31="Completed",IF(S31="","Evidence needed","Done"),IF(D31="Blocked","Blocked",IF(D31="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H31" s="27" t="n">
         <x:v>6</x:v>
@@ -2202,11 +2206,13 @@
       <x:c r="R31" s="19" t="str">
         <x:v>TB-S2</x:v>
       </x:c>
-      <x:c r="S31" s="23" t="str"/>
-      <x:c r="T31" s="23" t="str"/>
+      <x:c r="S31" s="23" t="str">
+        <x:v>/Volumes/MHRJ/TrustBench-AI/tests/provenance/; /Volumes/MHRJ/TrustBench-AI/reports/tb020-provenance-tests.xml</x:v>
+      </x:c>
+      <x:c r="T31" s="23"/>
       <x:c r="U31" s="19" t="n">
         <x:f>IF(LEN(S31)&gt;0,1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="64" customHeight="1">
@@ -2228,7 +2234,7 @@
       <x:c r="F32" s="20" t="str"/>
       <x:c r="G32" s="20" t="str">
         <x:f>IF(NOT(AND(IF(E32="",TRUE,COUNTIFS($A$12:$A$71,E32)=1),IF(F32="",TRUE,COUNTIFS($A$12:$A$71,F32)=1))),"Bad dependency",IF(NOT(AND(IF(E32="",TRUE,COUNTIFS($A$12:$A$71,E32,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F32="",TRUE,COUNTIFS($A$12:$A$71,F32,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D32="Completed","Check prerequisites","Waiting"),IF(D32="Completed",IF(S32="","Evidence needed","Done"),IF(D32="Blocked","Blocked",IF(D32="In Progress","In Progress","Ready")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H32" s="27" t="n">
         <x:v>7</x:v>
@@ -4720,11 +4726,11 @@
       </x:c>
       <x:c r="C81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Completed")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$D$12:$D$71,"In Progress")</x:f>
@@ -4736,7 +4742,7 @@
       </x:c>
       <x:c r="G81" s="29" t="n">
         <x:f>IF(B81=0,0,C81/B81)</x:f>
-        <x:v>0.8333333333333334</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81)</x:f>
@@ -4744,11 +4750,11 @@
       </x:c>
       <x:c r="I81" s="20" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A81,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J81" s="20" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A81,$G$12:$G$71,"Ready")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K81" s="2"/>
       <x:c r="L81" s="2"/>
@@ -4772,11 +4778,11 @@
       </x:c>
       <x:c r="C82" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A82,$D$12:$D$71,"Completed")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D82" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A82,$D$12:$D$71,"Not Started")</x:f>
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E82" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A82,$D$12:$D$71,"In Progress")</x:f>
@@ -4788,7 +4794,7 @@
       </x:c>
       <x:c r="G82" s="30" t="n">
         <x:f>IF(B82=0,0,C82/B82)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.3333333333333333</x:v>
       </x:c>
       <x:c r="H82" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A82)</x:f>
@@ -4796,11 +4802,11 @@
       </x:c>
       <x:c r="I82" s="19" t="n">
         <x:f>SUMIFS($H$12:$H$71,$B$12:$B$71,A82,$D$12:$D$71,"&lt;&gt;Completed")</x:f>
-        <x:v>33</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="J82" s="19" t="n">
         <x:f>COUNTIFS($B$12:$B$71,A82,$G$12:$G$71,"Ready")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K82" s="2"/>
       <x:c r="L82" s="2"/>
@@ -7411,13 +7417,13 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="7">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2965005f7ae44ba4"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9412a037148349f6"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f510be1879e4fc7"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebbf1d4a123f4bc7"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R692fb2a21eb84840"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ef0c3b5bee04d17"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f88c3b26e264c0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8876e76dd80f4d5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R291f22ba41c045c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e3b294008ac4d7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87f931c549844edc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07c534a6c64c42c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55f3a757102e4a62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb448d688fb0040b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Test policy boundary and normalization failures (TB-023)
Declare eight security invariants with collection-time positive/negative
coverage, add adversarial fixtures and Hypothesis property tests, and make
the gateway fail closed on malformed tool output.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -3138,7 +3138,7 @@
       </c>
       <c r="D34" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E34" s="20" t="inlineStr">
@@ -3192,8 +3192,16 @@
         </is>
       </c>
       <c r="R34" s="20" t="str"/>
-      <c r="S34" s="23" t="str"/>
-      <c r="T34" s="23" t="str"/>
+      <c r="S34" s="23" t="inlineStr">
+        <is>
+          <t>/Volumes/MHRJ/TrustBench-AI/reports/policy-tests.xml; /Volumes/MHRJ/TrustBench-AI/reports/policy-invariant-coverage.json; /Volumes/MHRJ/TrustBench-AI/tests/policy/test_invariants.py; /Volumes/MHRJ/TrustBench-AI/fixtures/policy/invariants.json; /Volumes/MHRJ/TrustBench-AI/fixtures/policy/adversarial.json</t>
+        </is>
+      </c>
+      <c r="T34" s="23" t="inlineStr">
+        <is>
+          <t>8 invariants, each with positive+negative tests enforced at collection (89 tests, 3 consecutive passes, Hypothesis included). Gateway hardened to fail closed on malformed tool output. Synthetic fixtures only; not proof against all attacks.</t>
+        </is>
+      </c>
       <c r="U34" s="19">
         <f>IF(LEN(S34)&gt;0,1,0)</f>
         <v/>

</xml_diff>

<commit_message>
Wire defended agent arm through the gateway (TB-024)
Add baseline/defended arm configs, a shared arm builder, gateway policy
decision traces, a LangGraph approval CLI and a 7-case parity smoke run.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -3225,7 +3225,7 @@
       </c>
       <c r="D35" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
@@ -3283,8 +3283,16 @@
         </is>
       </c>
       <c r="R35" s="19" t="str"/>
-      <c r="S35" s="23" t="str"/>
-      <c r="T35" s="23" t="str"/>
+      <c r="S35" s="23" t="inlineStr">
+        <is>
+          <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tb024-policy-decision-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log</t>
+        </is>
+      </c>
+      <c r="T35" s="23" t="inlineStr">
+        <is>
+          <t>Wired via same runner; 7 scripted smoke cases (3 benign, 4 attack) show identical config/prompts/state and gateway-only divergence. Scripted mock model: checks wiring/parity, NOT attack success rates. Baseline backend keeps its own contract checks; runner stops on first failed tool call (recovery is T-E3).</t>
+        </is>
+      </c>
       <c r="U35" s="19">
         <f>IF(LEN(S35)&gt;0,1,0)</f>
         <v/>

</xml_diff>

<commit_message>
Correct arm design flaws and contain holdout exposure (TB-024)
Make the baseline backend permissive per the protocol, expose all tools to both
arms, return tool errors to the model, add answer-format rules, a versioned v2
evaluator, attack renderings, repetitions and summary rates. Exclude locked
holdout fixtures from all runs and record amendments A-001 to A-006.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -2596,7 +2596,11 @@
           <t>/Volumes/MHRJ/TrustBench-AI/evidence/tb016-evaluator-report.json; /Volumes/MHRJ/TrustBench-AI/src/evaluators/; /Volumes/MHRJ/TrustBench-AI/tests/evaluators/</t>
         </is>
       </c>
-      <c r="T27" s="23" t="n"/>
+      <c r="T27" s="23" t="inlineStr">
+        <is>
+          <t>Frozen v1 (tb016.1.0.0) kept for the TB-017 pilot hash. Post-pilot fixes live in src/evaluators/outcomes_v2.py (tb016.1.1.0): abstention judging, answer normalization, HTTP argument names, decoy-record handling. See protocol/amendments.md A-002.</t>
+        </is>
+      </c>
       <c r="U27" s="19">
         <f>IF(LEN(S27)&gt;0,1,0)</f>
         <v/>
@@ -3285,12 +3289,12 @@
       <c r="R35" s="19" t="str"/>
       <c r="S35" s="23" t="inlineStr">
         <is>
-          <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tb024-policy-decision-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log</t>
+          <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tb024-policy-decision-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log; /Volumes/MHRJ/TrustBench-AI/protocol/amendments.md; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-holdout-mechanics-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-arm-corrections.log</t>
         </is>
       </c>
       <c r="T35" s="23" t="inlineStr">
         <is>
-          <t>Wired via same runner; 7 scripted smoke cases (3 benign, 4 attack) show identical config/prompts/state and gateway-only divergence. Scripted mock model: checks wiring/parity, NOT attack success rates. Baseline backend keeps its own contract checks; runner stops on first failed tool call (recovery is T-E3).</t>
+          <t>Corrected 2026-10-15 (protocol/amendments.md A-001..A-006): baseline now permissive per protocol; all tools visible in both arms; on_tool_error=continue; live pilots on NVIDIA/Qwen/Gemini (dev split, pilot-sized, not confirmatory). OPEN: the update-workflow holdout (TB-BEN/ATT-UPDATE-001) was exposed during wiring (A-005); a replacement sealed holdout and protocol version bump are needed before any confirmatory run. Residual gap: gateway does not inspect free-text body content inside authorized actions.</t>
         </is>
       </c>
       <c r="U35" s="19">

</xml_diff>

<commit_message>
Record harder-attack live matrix results and prompt-profile findings (TB-024)
Generated results from the finished passes (plain and hardened profiles, published
AgentDojo templates, positive control), amendment A-008, refreshed evidence and a
full verify log. Unfinished matrix cells are listed, not counted.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -3289,12 +3289,12 @@
       <c r="R35" s="19" t="str"/>
       <c r="S35" s="23" t="inlineStr">
         <is>
-          <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tb024-policy-decision-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log; /Volumes/MHRJ/TrustBench-AI/protocol/amendments.md; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-holdout-mechanics-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-arm-corrections.log</t>
+          <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tb024-policy-decision-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log; /Volumes/MHRJ/TrustBench-AI/protocol/amendments.md; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-holdout-mechanics-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-arm-corrections.log; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/data/attack-renderings.json; /Volumes/MHRJ/TrustBench-AI/configs/live-matrix.yaml; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-harder-attacks.log</t>
         </is>
       </c>
       <c r="T35" s="23" t="inlineStr">
         <is>
-          <t>Corrected 2026-10-15 (protocol/amendments.md A-001..A-006): baseline now permissive per protocol; all tools visible in both arms; on_tool_error=continue; live pilots on NVIDIA/Qwen/Gemini (dev split, pilot-sized, not confirmatory). OPEN: the update-workflow holdout (TB-BEN/ATT-UPDATE-001) was exposed during wiring (A-005); a replacement sealed holdout and protocol version bump are needed before any confirmatory run. Residual gap: gateway does not inspect free-text body content inside authorized actions.</t>
+          <t>Updated 2026-10-15 (protocol 1.1.0, amendments A-001..A-008): replacement sealed holdout created and never run; prompt profiles plain/hardened; published AgentDojo attack templates; positive control; run validity/exposure accounting. Live pilot (plain prompt, AgentDojo important_instructions): baseline attacker goal 8/20 (gpt-oss-20b) and 6/12 (qwen3.5:9b) vs 0 defended; generated tables in docs/pilot-results-tb024.md. Unfinished: several registered matrix cells (listed in that doc), Gemini quota exhausted. Residual gap: gateway does not inspect free-text content inside authorized actions. Pilot-sized, not confirmatory.</t>
         </is>
       </c>
       <c r="U35" s="19">

</xml_diff>

<commit_message>
Add bounded retries and write-safe recovery (TB-025)
Retry transient read failures and retryable model errors inside the registered retry
budget; never retry writes automatically, report unknown outcomes and suppress exact
duplicate writes. Applied to both arms. Tests with HTTP fault injection against the real
tool service, a naive-retry negative control and seeded fault-injection evidence.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -3320,7 +3320,7 @@
       </c>
       <c r="D36" s="22" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E36" s="21" t="inlineStr">
@@ -3374,8 +3374,16 @@
         </is>
       </c>
       <c r="R36" s="21" t="str"/>
-      <c r="S36" s="22" t="str"/>
-      <c r="T36" s="22" t="str"/>
+      <c r="S36" s="22" t="inlineStr">
+        <is>
+          <t>/Volumes/MHRJ/TrustBench-AI/tests/recovery/; /Volumes/MHRJ/TrustBench-AI/reports/tb025-recovery-tests.xml; /Volumes/MHRJ/TrustBench-AI/evidence/tb025-recovery-report.json; /Volumes/MHRJ/TrustBench-AI/src/agent/recovery.ts; /Volumes/MHRJ/TrustBench-AI/configs/recovery.yaml; /Volumes/MHRJ/TrustBench-AI/docs/recovery.md; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb025.log</t>
+        </is>
+      </c>
+      <c r="T36" s="22" t="inlineStr">
+        <is>
+          <t>Explicit retry logic (no Tenacity): reads retried with seeded backoff inside the registered retry budget; writes get exactly one attempt, unknown outcomes are reported and exact repeats suppressed. 29 tests incl. real-service HTTP fault injection and a naive-retry negative control; seven mutation checks. Seeded trials (synthetic faults, scripted model) show 0 duplicate writes and retries never above budget; success and the extra attempts/backoff cost are in evidence/tb025-recovery-report.json. Limit: LLM behavior after failed/unknown-outcome calls is not measured; durable restart handling is TB-026.</t>
+        </is>
+      </c>
       <c r="U36" s="19">
         <f>IF(LEN(S36)&gt;0,1,0)</f>
         <v/>

</xml_diff>

<commit_message>
Add provenance-aware flow check, remove hardcoding, record known issues
Gateway rules, providers, prompts, tool descriptions, run settings and attack
oracles move to config/data; a guard test fails on hardcoded fixture IDs,
endpoints, key names, models or seeds in runtime code. The defended arm gains a
provenance-aware flow check (default variant, capability-only kept as ablation),
measured in scripted and live runs. Evaluator oracles are data-driven and match
all frozen verdicts. Adds a gateway overhead benchmark and docs/known-issues.md.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -3289,12 +3289,12 @@
       <c r="R35" s="19" t="str"/>
       <c r="S35" s="23" t="inlineStr">
         <is>
-          <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tb024-policy-decision-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log; /Volumes/MHRJ/TrustBench-AI/protocol/amendments.md; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-holdout-mechanics-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-arm-corrections.log; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/data/attack-renderings.json; /Volumes/MHRJ/TrustBench-AI/configs/live-matrix.yaml; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-harder-attacks.log</t>
+          <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tb024-policy-decision-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log; /Volumes/MHRJ/TrustBench-AI/protocol/amendments.md; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/evidence/tb024-defended-arm-holdout-mechanics-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-arm-corrections.log; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/data/attack-renderings.json; /Volumes/MHRJ/TrustBench-AI/configs/live-matrix.yaml; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-harder-attacks.log; /Volumes/MHRJ/TrustBench-AI/docs/known-issues.md; /Volumes/MHRJ/TrustBench-AI/docs/flow-check.md; /Volumes/MHRJ/TrustBench-AI/configs/policy.yaml; /Volumes/MHRJ/TrustBench-AI/evidence/gateway-overhead-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-flow-check.log</t>
         </is>
       </c>
       <c r="T35" s="23" t="inlineStr">
         <is>
-          <t>Updated 2026-10-15 (protocol 1.1.0, amendments A-001..A-008): replacement sealed holdout created and never run; prompt profiles plain/hardened; published AgentDojo attack templates; positive control; run validity/exposure accounting. Live pilot (plain prompt, AgentDojo important_instructions): baseline attacker goal 8/20 (gpt-oss-20b) and 6/12 (qwen3.5:9b) vs 0 defended; generated tables in docs/pilot-results-tb024.md. Unfinished: several registered matrix cells (listed in that doc), Gemini quota exhausted. Residual gap: gateway does not inspect free-text content inside authorized actions. Pilot-sized, not confirmatory.</t>
+          <t>Updated 2026-10-15 (protocol 1.1.0, amendments A-001..A-008): replacement sealed holdout created and never run; prompt profiles plain/hardened; published AgentDojo attack templates; positive control; run validity/exposure accounting. Live pilot (plain prompt, AgentDojo important_instructions): baseline attacker goal 8/20 (gpt-oss-20b) and 6/12 (qwen3.5:9b) vs 0 defended; generated tables in docs/pilot-results-tb024.md. Unfinished: several registered matrix cells (listed in that doc), Gemini quota exhausted. Residual gap: gateway does not inspect free-text content inside authorized actions. Pilot-sized, not confirmatory. | 2026-10-15 later: provenance-aware flow check added as default defended variant (capability_only kept as ablation; A-010); open items tracked in docs/known-issues.md.</t>
         </is>
       </c>
       <c r="U35" s="19">

</xml_diff>

<commit_message>
Add durable runs, cancellation and durable gateway sessions (TB-026)
SQLite run store with checkpoints, write-ahead intent log, cancellation markers and
one final outcome per run; interrupted writes are never repeated unless replay-safe
through approval receipts. Gateway sessions persist with hashed tokens and a TTL.
Process-kill restart tests cover read, write and approval phases.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -3407,7 +3407,7 @@
       </c>
       <c r="D37" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
@@ -3461,8 +3461,16 @@
         </is>
       </c>
       <c r="R37" s="19" t="str"/>
-      <c r="S37" s="23" t="str"/>
-      <c r="T37" s="23" t="str"/>
+      <c r="S37" s="23" t="inlineStr">
+        <is>
+          <t>/Volumes/MHRJ/TrustBench-AI/tests/restart/; /Volumes/MHRJ/TrustBench-AI/reports/tb026-restart-tests.xml; /Volumes/MHRJ/TrustBench-AI/src/agent/run-store.ts; /Volumes/MHRJ/TrustBench-AI/tests/gateway/test_durable_sessions.py; /Volumes/MHRJ/TrustBench-AI/configs/durability.yaml; /Volumes/MHRJ/TrustBench-AI/docs/durability.md; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb026.log</t>
+        </is>
+      </c>
+      <c r="T37" s="23" t="inlineStr">
+        <is>
+          <t>SQLite run store with checkpoints, write-ahead intent log, cancellation markers and a single final outcome per run; durable gateway sessions (hashed tokens, TTL, owner-only file). Restart tests SIGKILL the real agent during read, after a committed write, and at the approval pause (gateway restarted too), plus cancellation; two mutation checks caught. Limits: per-run wall-clock timeout restarts after resume; restored flow-check memory starts empty; retention runs on store open.</t>
+        </is>
+      </c>
       <c r="U37" s="19">
         <f>IF(LEN(S37)&gt;0,1,0)</f>
         <v/>

</xml_diff>

<commit_message>
Live CaMeL and directive_flow v2-v4 results, new models, matrix cells
- CaMeL-style baseline compared on four models; directive_flow v2/v3/v4
  pre-registered (A-014, A-016, A-017) and scored per prediction.
- Llama-3.2-11B and Gemma 4 added; pre-registered pooled analysis reported
  with the A-019 parser-bug confound and its correction (not separated).
- Exposure line per model (Llama models never read injections).
- Shared JSON extractor fixes inline-reasoning parses (A-019); token-aware
  pacing for free-tier limits (A-018); missing matrix cells filled.
- Docs, known issues and workbook updated; full verify passed.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A03340E-F813-8240-8419-D1B5CA07E311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A8C471-16E8-F149-A90E-6BDF5089FDC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -850,10 +850,10 @@
     <t>Avoid confounding security changes with stronger model prompts.</t>
   </si>
   <si>
-    <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/reports/tests/tb024-scripted-as_authored-plain-gateway_capability-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tests/tb024-scripted-as_authored-plain-gateway_capability-policy-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log; /Volumes/MHRJ/TrustBench-AI/protocol/amendments.md; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/reports/tests/tb024-scripted-as_authored-plain-gateway_capability-suite-holdout-guard-suite-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-arm-corrections.log; /Volumes/MHRJ/TrustBench-AI/data/attack-renderings.json; /Volumes/MHRJ/TrustBench-AI/configs/live-matrix.yaml; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-harder-attacks.log; /Volumes/MHRJ/TrustBench-AI/docs/known-issues.md; /Volumes/MHRJ/TrustBench-AI/docs/flow-check.md; /Volumes/MHRJ/TrustBench-AI/configs/policy.yaml; /Volumes/MHRJ/TrustBench-AI/evidence/gateway-overhead-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-flow-check.log; /Volumes/MHRJ/TrustBench-AI/docs/defense-comparison.md; /Volumes/MHRJ/TrustBench-AI/scripts/summarize-defense-comparison.mjs; /Volumes/MHRJ/TrustBench-AI/configs/defense-comparison.yaml; /Volumes/MHRJ/TrustBench-AI/configs/defenses.yaml; /Volumes/MHRJ/TrustBench-AI/src/agent/defenses.ts; /Volumes/MHRJ/TrustBench-AI/tests/arms/stress-cases.json</t>
-  </si>
-  <si>
-    <t>Updated 2026-10-15 (protocol 1.1.0, amendments A-001..A-008): replacement sealed holdout created and never run; prompt profiles plain/hardened; published AgentDojo attack templates; positive control; run validity/exposure accounting. Live pilot (plain prompt, AgentDojo important_instructions): baseline attacker goal 8/20 (gpt-oss-20b) and 6/12 (qwen3.5:9b) vs 0 defended; generated tables in docs/pilot-results-tb024.md. Unfinished: several registered matrix cells (listed in that doc), Gemini quota exhausted. Residual gap: gateway does not inspect free-text content inside authorized actions. Pilot-sized, not confirmatory. | 2026-10-15 later: provenance-aware flow check added as default defended variant (capability_only kept as ablation; A-010); open items tracked in docs/known-issues.md. | Updated 2026-10-15 (A-011..A-013): plain registered as primary profile; signed provenance envelopes; registered live defense comparison (configs/defense-comparison.yaml, gpt-oss-20b and qwen3.5:9b, 2 reps, important_instructions) against re-implemented spotlighting, sandwich, tool_filter and MELON, generated with Newcombe intervals in docs/defense-comparison.md (all registered cells finished). Candidate gateway_directive_flow is lower than every published baseline and no defense on gpt-oss, but not separated from the capability gateway alone at this sample size; it uniquely stops the answer-poisoning and link cases. Stress fixture TB-ATT-DOC-005 shows its measured blind spot (declarative-only poisoning passes). Contract-backend ablation: gateway benefit assumes a permissive tool backend. All development split; exploratory, not confirmatory. | Evidence paths corrected 2026-10-16: the single scripted report and traces were renamed per run in commit 0d7cc53 (scripted runs are tests, under reports/tests/); the holdout-mechanics report is now the holdout-guard suite report written by npm run test:arms.</t>
+    <t>/Volumes/MHRJ/TrustBench-AI/configs/defended.yaml; /Volumes/MHRJ/TrustBench-AI/configs/baseline.yaml; /Volumes/MHRJ/TrustBench-AI/src/arms/; /Volumes/MHRJ/TrustBench-AI/reports/tests/tb024-scripted-as_authored-plain-gateway_capability-report.json; /Volumes/MHRJ/TrustBench-AI/reports/tests/tb024-scripted-as_authored-plain-gateway_capability-policy-traces.jsonl; /Volumes/MHRJ/TrustBench-AI/tests/arms.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/approval/test_approved_call.py; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb024.log; /Volumes/MHRJ/TrustBench-AI/protocol/amendments.md; /Volumes/MHRJ/TrustBench-AI/docs/pilot-results-tb024.md; /Volumes/MHRJ/TrustBench-AI/reports/tests/tb024-scripted-as_authored-plain-gateway_capability-suite-holdout-guard-suite-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-arm-corrections.log; /Volumes/MHRJ/TrustBench-AI/data/attack-renderings.json; /Volumes/MHRJ/TrustBench-AI/configs/live-matrix.yaml; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-harder-attacks.log; /Volumes/MHRJ/TrustBench-AI/docs/known-issues.md; /Volumes/MHRJ/TrustBench-AI/docs/flow-check.md; /Volumes/MHRJ/TrustBench-AI/configs/policy.yaml; /Volumes/MHRJ/TrustBench-AI/evidence/gateway-overhead-report.json; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-flow-check.log; /Volumes/MHRJ/TrustBench-AI/docs/defense-comparison.md; /Volumes/MHRJ/TrustBench-AI/scripts/summarize-defense-comparison.mjs; /Volumes/MHRJ/TrustBench-AI/configs/defense-comparison.yaml; /Volumes/MHRJ/TrustBench-AI/configs/defenses.yaml; /Volumes/MHRJ/TrustBench-AI/src/agent/defenses.ts; /Volumes/MHRJ/TrustBench-AI/tests/arms/stress-cases.json; /Volumes/MHRJ/TrustBench-AI/docs/camel.md; /Volumes/MHRJ/TrustBench-AI/src/agent/camel.ts; /Volumes/MHRJ/TrustBench-AI/tests/camel.test.ts; /Volumes/MHRJ/TrustBench-AI/src/agent/json-extract.ts; /Volumes/MHRJ/TrustBench-AI/tests/json-extract.test.ts; /Volumes/MHRJ/TrustBench-AI/tests/arms/stress-v2-cases.json; /Volumes/MHRJ/TrustBench-AI/tests/arms/stress-v3-cases.json</t>
+  </si>
+  <si>
+    <t>Updated 2026-10-15 (protocol 1.1.0, amendments A-001..A-008): replacement sealed holdout created and never run; prompt profiles plain/hardened; published AgentDojo attack templates; positive control; run validity/exposure accounting. Live pilot (plain prompt, AgentDojo important_instructions): baseline attacker goal 8/20 (gpt-oss-20b) and 6/12 (qwen3.5:9b) vs 0 defended; generated tables in docs/pilot-results-tb024.md. Unfinished: several registered matrix cells (listed in that doc), Gemini quota exhausted. Residual gap: gateway does not inspect free-text content inside authorized actions. Pilot-sized, not confirmatory. | 2026-10-15 later: provenance-aware flow check added as default defended variant (capability_only kept as ablation; A-010); open items tracked in docs/known-issues.md. | Updated 2026-10-15 (A-011..A-013): plain registered as primary profile; signed provenance envelopes; registered live defense comparison (configs/defense-comparison.yaml, gpt-oss-20b and qwen3.5:9b, 2 reps, important_instructions) against re-implemented spotlighting, sandwich, tool_filter and MELON, generated with Newcombe intervals in docs/defense-comparison.md (all registered cells finished). Candidate gateway_directive_flow is lower than every published baseline and no defense on gpt-oss, but not separated from the capability gateway alone at this sample size; it uniquely stops the answer-poisoning and link cases. Stress fixture TB-ATT-DOC-005 shows its measured blind spot (declarative-only poisoning passes). Contract-backend ablation: gateway benefit assumes a permissive tool backend. All development split; exploratory, not confirmatory. | Evidence paths corrected 2026-10-16: the single scripted report and traces were renamed per run in commit 0d7cc53 (scripted runs are tests, under reports/tests/); the holdout-mechanics report is now the holdout-guard suite report written by npm run test:arms. | Updated 2026-10-16 (A-014..A-019): CaMeL-style baseline re-implemented and compared; directive_flow v2/v3/v4 each pre-registered before its runs, scored per prediction in docs/defense-comparison.md (v3/v4 fresh-fixture predictions supported with non-vacuous classifier calls; pure statement-of-fact poisoning still passes). Added Llama-3.2-11B and Gemma 4; pre-registered pooled analysis (directive_flow vs capability gateway on the new models) not separated, reported with the A-019 parser-bug confound and its correction. Llama models never read injections (no defense effect measurable). Live matrix cells filled (A-014/A-015/A-018). Development split only; exploratory.</t>
   </si>
   <si>
     <t>TB-025</t>

</xml_diff>

<commit_message>
Mark TB-027 Completed; ignore Office lock files
Full verify passed after the TB-027 merge (reports/full-verify-after-tb027.log).
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A8C471-16E8-F149-A90E-6BDF5089FDC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57DC5F0F-6E3E-7141-A467-431DA57F89E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="764">
   <si>
     <t>TrustBench-AI — implementation plan</t>
   </si>
@@ -2318,6 +2318,12 @@
   </si>
   <si>
     <t>Top: A1</t>
+  </si>
+  <si>
+    <t>/Volumes/MHRJ/TrustBench-AI/observability/README.md; /Volumes/MHRJ/TrustBench-AI/observability/tb027-report.json; /Volumes/MHRJ/TrustBench-AI/observability/traces/; /Volumes/MHRJ/TrustBench-AI/src/observability/tracing.ts; /Volumes/MHRJ/TrustBench-AI/src/observability/run-spans.ts; /Volumes/MHRJ/TrustBench-AI/src/observability/check.ts; /Volumes/MHRJ/TrustBench-AI/scripts/verify-observability.mjs; /Volumes/MHRJ/TrustBench-AI/tests/observability.test.ts; /Volumes/MHRJ/TrustBench-AI/configs/observability.yaml; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb027.log</t>
+  </si>
+  <si>
+    <t>Completed 2026-10-16. OpenTelemetry spans (api + sdk-trace-base), JSON-lines export: one trace per arm run with agent.run root; model.call (queue.ms = pacing wait, so latency includes queueing), tool.call (retrieval-tagged, per attempt, argument SHA-256 only), policy.decision (gateway-timed audit). Every span carries run.id. Export drops non-allowlisted attributes and redacts seeded fixture secrets derived from the data files (holdout excluded). verify:observability passes on scripted and live exports (gpt-oss-20b, Gemma 4); in both live runs the undefended agent read the canary yet no span contains it. Limit: spans cover the TrustBench harness and gateway, not eve's own pilot agent runtime.</t>
   </si>
 </sst>
 </file>
@@ -3094,11 +3100,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$71,"Completed")</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.43333333333333335</v>
+        <v>0.45</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$71,"Blocked")</f>
@@ -3110,15 +3116,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</f>
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</f>
-        <v>0.48148148148148145</v>
+        <v>0.5</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>9.9166666666666661</v>
+        <v>9.5833333333333339</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</f>
@@ -4871,7 +4877,7 @@
         <v>296</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>297</v>
+        <v>2</v>
       </c>
       <c r="E38" s="11" t="s">
         <v>285</v>
@@ -4879,7 +4885,7 @@
       <c r="F38" s="11"/>
       <c r="G38" s="11" t="str">
         <f t="shared" si="0"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H38" s="18">
         <v>4</v>
@@ -4908,11 +4914,15 @@
         <v>52</v>
       </c>
       <c r="R38" s="11"/>
-      <c r="S38" s="14"/>
-      <c r="T38" s="14"/>
+      <c r="S38" s="14" t="s">
+        <v>762</v>
+      </c>
+      <c r="T38" s="14" t="s">
+        <v>763</v>
+      </c>
       <c r="U38" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:21" ht="64" customHeight="1">
@@ -4934,7 +4944,7 @@
       <c r="F39" s="10"/>
       <c r="G39" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H39" s="18">
         <v>5</v>
@@ -5212,7 +5222,7 @@
       </c>
       <c r="F44" s="11"/>
       <c r="G44" s="11" t="str">
-        <f t="shared" ref="G44:G75" si="2">IF(NOT(AND(IF(E44="",TRUE,COUNTIFS($A$12:$A$71,E44)=1),IF(F44="",TRUE,COUNTIFS($A$12:$A$71,F44)=1))),"Bad dependency",IF(NOT(AND(IF(E44="",TRUE,COUNTIFS($A$12:$A$71,E44,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F44="",TRUE,COUNTIFS($A$12:$A$71,F44,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D44="Completed","Check prerequisites","Waiting"),IF(D44="Completed",IF(S44="","Evidence needed","Done"),IF(D44="Blocked","Blocked",IF(D44="In Progress","In Progress","Ready")))))</f>
+        <f t="shared" ref="G44:G71" si="2">IF(NOT(AND(IF(E44="",TRUE,COUNTIFS($A$12:$A$71,E44)=1),IF(F44="",TRUE,COUNTIFS($A$12:$A$71,F44)=1))),"Bad dependency",IF(NOT(AND(IF(E44="",TRUE,COUNTIFS($A$12:$A$71,E44,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1),IF(F44="",TRUE,COUNTIFS($A$12:$A$71,F44,$D$12:$D$71,"Completed",$U$12:$U$71,1)=1))),IF(D44="Completed","Check prerequisites","Waiting"),IF(D44="Completed",IF(S44="","Evidence needed","Done"),IF(D44="Blocked","Blocked",IF(D44="In Progress","In Progress","Ready")))))</f>
         <v>Waiting</v>
       </c>
       <c r="H44" s="18">
@@ -7141,11 +7151,11 @@
       </c>
       <c r="C83" s="11">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D83" s="11">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E83" s="11">
         <f t="shared" si="7"/>
@@ -7157,7 +7167,7 @@
       </c>
       <c r="G83" s="20">
         <f t="shared" si="9"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="H83" s="11">
         <f t="shared" si="10"/>
@@ -7165,7 +7175,7 @@
       </c>
       <c r="I83" s="11">
         <f t="shared" si="11"/>
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J83" s="11">
         <f t="shared" si="12"/>

</xml_diff>

<commit_message>
Add repeated-run evaluator with fixed task-seed schedules (TB-028)
Python + NumPy: per-cluster success frequency, all-repeats success,
cluster bootstrap and intra-cluster correlation; runner executes schedules
exactly. Same units in two orders give identical pairing, denominators and
results. Live 80-unit schedule on gpt-oss-20b; 38 existing repeated-run
reports evaluated. Locked tools env gains numpy and the previously
undeclared openpyxl. TB-028 marked Completed; full verify passed.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57DC5F0F-6E3E-7141-A467-431DA57F89E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62696910-1E14-7048-838E-A113207D9196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="766">
   <si>
     <t>TrustBench-AI — implementation plan</t>
   </si>
@@ -2324,6 +2324,12 @@
   </si>
   <si>
     <t>Completed 2026-10-16. OpenTelemetry spans (api + sdk-trace-base), JSON-lines export: one trace per arm run with agent.run root; model.call (queue.ms = pacing wait, so latency includes queueing), tool.call (retrieval-tagged, per attempt, argument SHA-256 only), policy.decision (gateway-timed audit). Every span carries run.id. Export drops non-allowlisted attributes and redacts seeded fixture secrets derived from the data files (holdout excluded). verify:observability passes on scripted and live exports (gpt-oss-20b, Gemma 4); in both live runs the undefended agent read the canary yet no span contains it. Limit: spans cover the TrustBench harness and gateway, not eve's own pilot agent runtime.</t>
+  </si>
+  <si>
+    <t>/Volumes/MHRJ/TrustBench-AI/src/evaluation/repeats.py; /Volumes/MHRJ/TrustBench-AI/src/evaluation/README.md; /Volumes/MHRJ/TrustBench-AI/tests/evaluation/test_repeats.py; /Volumes/MHRJ/TrustBench-AI/scripts/verify-repeats.py; /Volumes/MHRJ/TrustBench-AI/evidence/tb028-order-invariance-report.json; /Volumes/MHRJ/TrustBench-AI/observability/schedules/tb028-dev-suite.json; /Volumes/MHRJ/TrustBench-AI/evidence/tb028/; /Volumes/MHRJ/TrustBench-AI/docs/repeated-runs.md; /Volumes/MHRJ/TrustBench-AI/reports/full-verify-after-tb028.log</t>
+  </si>
+  <si>
+    <t>Completed 2026-10-16. Python + NumPy evaluator: fixed task-seed schedules (unit = task x attack variant x repetition, registered seeds, seeded order; content and order hashed separately); runner executes a schedule exactly and refuses seed mismatches. Per-cluster success frequency, all-repeats and any-repeat success, cluster-bootstrap CIs, paired defended-baseline difference by cluster, intra-cluster correlation; pooled rate shown only as contrast. Acceptance: same units executed in two orders through the real harness give identical pairing, denominators and results (evidence/tb028-order-invariance-report.json); shuffled-input and mutation tests. Live: 80/80 scheduled units on gpt-oss-20b (v4 vs baseline, 5 reps) plus 38 existing repeated-run reports in docs/repeated-runs.md. Baseline ICC 0.5-0.7 shows repeats are strongly correlated. Development split only.</t>
   </si>
 </sst>
 </file>
@@ -3100,11 +3106,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$71,"Completed")</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.45</v>
+        <v>0.46666666666666667</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$71,"Blocked")</f>
@@ -3116,15 +3122,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$71,$D$12:$D$71,"&lt;&gt;Completed")</f>
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$71,"Core",$D$12:$D$71,"Completed")/COUNTIFS($Q$12:$Q$71,"Core")</f>
-        <v>0.5</v>
+        <v>0.51851851851851849</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$71,$Q$12:$Q$71,"Core",$D$12:$D$71,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>9.5833333333333339</v>
+        <v>9.1666666666666661</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$71,"&gt;0",$J$12:$J$71,"&lt;"&amp;TODAY(),$D$12:$D$71,"&lt;&gt;Completed")</f>
@@ -4936,7 +4942,7 @@
         <v>305</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>297</v>
+        <v>2</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>295</v>
@@ -4944,7 +4950,7 @@
       <c r="F39" s="10"/>
       <c r="G39" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H39" s="18">
         <v>5</v>
@@ -4973,11 +4979,15 @@
         <v>52</v>
       </c>
       <c r="R39" s="10"/>
-      <c r="S39" s="14"/>
-      <c r="T39" s="14"/>
+      <c r="S39" s="14" t="s">
+        <v>764</v>
+      </c>
+      <c r="T39" s="14" t="s">
+        <v>765</v>
+      </c>
       <c r="U39" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:21" ht="64" customHeight="1">
@@ -4999,7 +5009,7 @@
       <c r="F40" s="11"/>
       <c r="G40" s="11" t="str">
         <f t="shared" si="0"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H40" s="18">
         <v>6</v>
@@ -7151,11 +7161,11 @@
       </c>
       <c r="C83" s="11">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D83" s="11">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E83" s="11">
         <f t="shared" si="7"/>
@@ -7167,7 +7177,7 @@
       </c>
       <c r="G83" s="20">
         <f t="shared" si="9"/>
-        <v>0.5</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H83" s="11">
         <f t="shared" si="10"/>
@@ -7175,7 +7185,7 @@
       </c>
       <c r="I83" s="11">
         <f t="shared" si="11"/>
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J83" s="11">
         <f t="shared" si="12"/>

</xml_diff>

<commit_message>
Add failure localizer, attribution report and human review UI (TB-029)
Deterministic first-violated-contract rules (configs/localization.yaml)
over 2,464 failed live runs (reports/attribution.csv), constructed ground
truth 56/56, local review UI with a seeded 43-case sample. TB-029 is
Blocked until a human reviews the sample; accuracy is then computed by
npm run attribution:build.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62696910-1E14-7048-838E-A113207D9196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB87CCEE-EA33-434F-9CF0-2A9F71B4CC77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="768">
   <si>
     <t>TrustBench-AI — implementation plan</t>
   </si>
@@ -2330,6 +2330,12 @@
   </si>
   <si>
     <t>Completed 2026-10-16. Python + NumPy evaluator: fixed task-seed schedules (unit = task x attack variant x repetition, registered seeds, seeded order; content and order hashed separately); runner executes a schedule exactly and refuses seed mismatches. Per-cluster success frequency, all-repeats and any-repeat success, cluster-bootstrap CIs, paired defended-baseline difference by cluster, intra-cluster correlation; pooled rate shown only as contrast. Acceptance: same units executed in two orders through the real harness give identical pairing, denominators and results (evidence/tb028-order-invariance-report.json); shuffled-input and mutation tests. Live: 80/80 scheduled units on gpt-oss-20b (v4 vs baseline, 5 reps) plus 38 existing repeated-run reports in docs/repeated-runs.md. Baseline ICC 0.5-0.7 shows repeats are strongly correlated. Development split only.</t>
+  </si>
+  <si>
+    <t>/Volumes/MHRJ/TrustBench-AI/reports/attribution.csv; /Volumes/MHRJ/TrustBench-AI/src/analysis/localize.py; /Volumes/MHRJ/TrustBench-AI/src/analysis/constructed.py; /Volumes/MHRJ/TrustBench-AI/configs/localization.yaml; /Volumes/MHRJ/TrustBench-AI/src/review/app.py; /Volumes/MHRJ/TrustBench-AI/reports/attribution-review-sample.json; /Volumes/MHRJ/TrustBench-AI/evidence/tb029-attribution-accuracy.json; /Volumes/MHRJ/TrustBench-AI/docs/attribution.md; /Volumes/MHRJ/TrustBench-AI/tests/analysis/</t>
+  </si>
+  <si>
+    <t>BLOCKED on human review (acceptance needs accuracy against reviewed cases). Done: deterministic first-violated-contract localizer (7 rules, config-driven) over 2,464 failed live runs -&gt; reports/attribution.csv; constructed ground truth 56/56; review UI (npm run review:attribution, http://127.0.0.1:8765) with a seeded stratified sample of 43 cases, labels bound to the exact prediction. Next: a human labels the 43 cases, then npm run attribution:build computes accuracy. Judge labels not used until that calibration exists.</t>
   </si>
 </sst>
 </file>
@@ -3114,7 +3120,7 @@
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$71,"Blocked")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="5">
         <f>SUM($H$12:$H$71)</f>
@@ -5001,7 +5007,7 @@
         <v>313</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>297</v>
+        <v>4</v>
       </c>
       <c r="E40" s="11" t="s">
         <v>304</v>
@@ -5009,7 +5015,7 @@
       <c r="F40" s="11"/>
       <c r="G40" s="11" t="str">
         <f t="shared" si="0"/>
-        <v>Ready</v>
+        <v>Blocked</v>
       </c>
       <c r="H40" s="18">
         <v>6</v>
@@ -5038,11 +5044,15 @@
         <v>52</v>
       </c>
       <c r="R40" s="11"/>
-      <c r="S40" s="14"/>
-      <c r="T40" s="14"/>
+      <c r="S40" s="14" t="s">
+        <v>766</v>
+      </c>
+      <c r="T40" s="14" t="s">
+        <v>767</v>
+      </c>
       <c r="U40" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:21" ht="64" customHeight="1">
@@ -7165,7 +7175,7 @@
       </c>
       <c r="D83" s="11">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E83" s="11">
         <f t="shared" si="7"/>
@@ -7173,7 +7183,7 @@
       </c>
       <c r="F83" s="11">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G83" s="20">
         <f t="shared" si="9"/>
@@ -7189,7 +7199,7 @@
       </c>
       <c r="J83" s="11">
         <f t="shared" si="12"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K83" s="1"/>
       <c r="L83" s="1"/>

</xml_diff>

<commit_message>
Audit failure attribution in two rounds; fix localizer defects (TB-029)
AI audit (an AI model, labelled as AI, not human) of 43 + 50 cases, per failed
check. Round 1 found six localizer defects (malformed writes, string
booleans, outcome-unknown writes, grounding misfires, termination, proposal
attacker values), fixed in localizer 1.1.0; round 2 on fresh cases scores
61/65 checks. Every case and verdict in docs/attribution-audit.md; review
UI now judges each failed check. TB-029 stays Blocked on human calibration.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB87CCEE-EA33-434F-9CF0-2A9F71B4CC77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A11ABF4A-D699-274F-A335-5B12B8A2AD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2332,10 +2332,10 @@
     <t>Completed 2026-10-16. Python + NumPy evaluator: fixed task-seed schedules (unit = task x attack variant x repetition, registered seeds, seeded order; content and order hashed separately); runner executes a schedule exactly and refuses seed mismatches. Per-cluster success frequency, all-repeats and any-repeat success, cluster-bootstrap CIs, paired defended-baseline difference by cluster, intra-cluster correlation; pooled rate shown only as contrast. Acceptance: same units executed in two orders through the real harness give identical pairing, denominators and results (evidence/tb028-order-invariance-report.json); shuffled-input and mutation tests. Live: 80/80 scheduled units on gpt-oss-20b (v4 vs baseline, 5 reps) plus 38 existing repeated-run reports in docs/repeated-runs.md. Baseline ICC 0.5-0.7 shows repeats are strongly correlated. Development split only.</t>
   </si>
   <si>
-    <t>/Volumes/MHRJ/TrustBench-AI/reports/attribution.csv; /Volumes/MHRJ/TrustBench-AI/src/analysis/localize.py; /Volumes/MHRJ/TrustBench-AI/src/analysis/constructed.py; /Volumes/MHRJ/TrustBench-AI/configs/localization.yaml; /Volumes/MHRJ/TrustBench-AI/src/review/app.py; /Volumes/MHRJ/TrustBench-AI/reports/attribution-review-sample.json; /Volumes/MHRJ/TrustBench-AI/evidence/tb029-attribution-accuracy.json; /Volumes/MHRJ/TrustBench-AI/docs/attribution.md; /Volumes/MHRJ/TrustBench-AI/tests/analysis/</t>
-  </si>
-  <si>
-    <t>BLOCKED on human review (acceptance needs accuracy against reviewed cases). Done: deterministic first-violated-contract localizer (7 rules, config-driven) over 2,464 failed live runs -&gt; reports/attribution.csv; constructed ground truth 56/56; review UI (npm run review:attribution, http://127.0.0.1:8765) with a seeded stratified sample of 43 cases, labels bound to the exact prediction. Next: a human labels the 43 cases, then npm run attribution:build computes accuracy. Judge labels not used until that calibration exists.</t>
+    <t>/Volumes/MHRJ/TrustBench-AI/reports/attribution.csv; /Volumes/MHRJ/TrustBench-AI/src/analysis/localize.py; /Volumes/MHRJ/TrustBench-AI/src/analysis/constructed.py; /Volumes/MHRJ/TrustBench-AI/configs/localization.yaml; /Volumes/MHRJ/TrustBench-AI/src/review/app.py; /Volumes/MHRJ/TrustBench-AI/reports/attribution-audit/; /Volumes/MHRJ/TrustBench-AI/data/reviews/attribution-ai-audit.jsonl; /Volumes/MHRJ/TrustBench-AI/evidence/tb029-attribution-accuracy.json; /Volumes/MHRJ/TrustBench-AI/docs/attribution.md; /Volumes/MHRJ/TrustBench-AI/docs/attribution-audit.md; /Volumes/MHRJ/TrustBench-AI/tests/analysis/</t>
+  </si>
+  <si>
+    <t>BLOCKED on human calibration. Done: localizer 1.1.0 over 2,464 failed live runs (reports/attribution.csv); constructed ground truth 86/86; AI audit (Claude, labelled as AI, not human) round 1 = 48/59 checks on localizer 1.0 (drove 6 fixes), round 2 on 50 fresh cases = 61/65 checks (utility 37/41, security 24/24); every case in docs/attribution-audit.md; 4 open localizer defects listed there. Next: a human reviews the 50 round-2 cases (npm run review:attribution) so the AI audit can be calibrated; then npm run attribution:build.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Renumber task IDs in row order: phase 10 is TB-055..TB-066, extensions TB-067..TB-072
Dependencies and in-text references were remapped together in one pass;
no other file in the repository referenced these IDs.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A9A795-E33C-FB4E-AE7A-2D4AE1D0FBDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6714F291-2E45-4E4E-8D83-9737E37E8022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2389,9 +2389,6 @@
     <t>Agent SDK or MCP, src/gateway, TypeScript or Python adapter</t>
   </si>
   <si>
-    <t>Integration contract (TB-062); gateway and tool services</t>
-  </si>
-  <si>
     <t>Adapter tests show every TrustBench tool callable from the agent, traces validating against the TB-004 schema, and a diff proving no change to the agent's source.</t>
   </si>
   <si>
@@ -2494,9 +2491,6 @@
     <t>protocol/amendments.md (external validation entry); data/external-splits.json</t>
   </si>
   <si>
-    <t>Too few unused fixture families for a fresh split: author new families first (TB-068) and register them before use.</t>
-  </si>
-  <si>
     <t>TB-068</t>
   </si>
   <si>
@@ -2557,9 +2551,6 @@
     <t>Batch runner, TB-028 schedules, free models</t>
   </si>
   <si>
-    <t>External validation split (TB-067), frozen gateway configuration (configs/frozen/)</t>
-  </si>
-  <si>
     <t>Paired reports for every scheduled unit or a recorded reason for each missing one; the provider revision is recorded and constant, or the comparison is labelled invalid.</t>
   </si>
   <si>
@@ -2605,9 +2596,6 @@
     <t>docs/, web/</t>
   </si>
   <si>
-    <t>TB-071 results; TB-062 threat model</t>
-  </si>
-  <si>
     <t>Limitations section lists every uncovered entry point and failed check; the guide is followed once on a clean checkout; claims stay within the measured scope.</t>
   </si>
   <si>
@@ -2645,6 +2633,18 @@
   </si>
   <si>
     <t>Work through phases 01–09 for Core. Phase 10 (External agent validation, Scope = Validation) follows the core roadmap and starts only after TB-054; phase 11 is optional. Dependencies refer to task IDs in this sheet; independent projects need no other project to be finished.</t>
+  </si>
+  <si>
+    <t>Integration contract (TB-056); gateway and tool services</t>
+  </si>
+  <si>
+    <t>Too few unused fixture families for a fresh split: author new families first (TB-062) and register them before use.</t>
+  </si>
+  <si>
+    <t>External validation split (TB-061), frozen gateway configuration (configs/frozen/)</t>
+  </si>
+  <si>
+    <t>TB-065 results; TB-056 threat model</t>
   </si>
 </sst>
 </file>
@@ -3521,28 +3521,28 @@
     </row>
     <row r="8" spans="1:21" ht="32" customHeight="1">
       <c r="A8" s="9" t="s">
+        <v>858</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>859</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>860</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>861</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>862</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="F8" s="9" t="s">
         <v>863</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="G8" s="9" t="s">
         <v>864</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="H8" s="9" t="s">
         <v>865</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>866</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>867</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>868</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>869</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -6757,7 +6757,7 @@
     </row>
     <row r="66" spans="1:21" ht="64" customHeight="1">
       <c r="A66" s="10" t="s">
-        <v>762</v>
+        <v>515</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>763</v>
@@ -6814,7 +6814,7 @@
     </row>
     <row r="67" spans="1:21" ht="64" customHeight="1">
       <c r="A67" s="10" t="s">
-        <v>772</v>
+        <v>524</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>763</v>
@@ -6826,7 +6826,7 @@
         <v>288</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>762</v>
+        <v>515</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>45</v>
@@ -6873,7 +6873,7 @@
     </row>
     <row r="68" spans="1:21" ht="64" customHeight="1">
       <c r="A68" s="10" t="s">
-        <v>781</v>
+        <v>532</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>763</v>
@@ -6885,7 +6885,7 @@
         <v>288</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>772</v>
+        <v>524</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>255</v>
@@ -6906,16 +6906,16 @@
         <v>784</v>
       </c>
       <c r="M68" s="10" t="s">
+        <v>867</v>
+      </c>
+      <c r="N68" s="10" t="s">
         <v>785</v>
       </c>
-      <c r="N68" s="10" t="s">
+      <c r="O68" s="10" t="s">
         <v>786</v>
       </c>
-      <c r="O68" s="10" t="s">
+      <c r="P68" s="10" t="s">
         <v>787</v>
-      </c>
-      <c r="P68" s="10" t="s">
-        <v>788</v>
       </c>
       <c r="Q68" s="10" t="s">
         <v>771</v>
@@ -6932,19 +6932,19 @@
     </row>
     <row r="69" spans="1:21" ht="64" customHeight="1">
       <c r="A69" s="10" t="s">
-        <v>789</v>
+        <v>540</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="D69" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>781</v>
+        <v>532</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>225</v>
@@ -6959,22 +6959,22 @@
       <c r="I69" s="14"/>
       <c r="J69" s="16"/>
       <c r="K69" s="10" t="s">
+        <v>790</v>
+      </c>
+      <c r="L69" s="10" t="s">
         <v>791</v>
       </c>
-      <c r="L69" s="10" t="s">
+      <c r="M69" s="10" t="s">
         <v>792</v>
       </c>
-      <c r="M69" s="10" t="s">
+      <c r="N69" s="10" t="s">
         <v>793</v>
       </c>
-      <c r="N69" s="10" t="s">
+      <c r="O69" s="10" t="s">
         <v>794</v>
       </c>
-      <c r="O69" s="10" t="s">
+      <c r="P69" s="10" t="s">
         <v>795</v>
-      </c>
-      <c r="P69" s="10" t="s">
-        <v>796</v>
       </c>
       <c r="Q69" s="10" t="s">
         <v>771</v>
@@ -6991,19 +6991,19 @@
     </row>
     <row r="70" spans="1:21" ht="64" customHeight="1">
       <c r="A70" s="10" t="s">
-        <v>797</v>
+        <v>548</v>
       </c>
       <c r="B70" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="D70" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>781</v>
+        <v>532</v>
       </c>
       <c r="F70" s="10" t="s">
         <v>138</v>
@@ -7018,22 +7018,22 @@
       <c r="I70" s="14"/>
       <c r="J70" s="16"/>
       <c r="K70" s="10" t="s">
+        <v>798</v>
+      </c>
+      <c r="L70" s="10" t="s">
         <v>799</v>
       </c>
-      <c r="L70" s="10" t="s">
+      <c r="M70" s="10" t="s">
         <v>800</v>
       </c>
-      <c r="M70" s="10" t="s">
+      <c r="N70" s="10" t="s">
         <v>801</v>
       </c>
-      <c r="N70" s="10" t="s">
+      <c r="O70" s="10" t="s">
         <v>802</v>
       </c>
-      <c r="O70" s="10" t="s">
+      <c r="P70" s="10" t="s">
         <v>803</v>
-      </c>
-      <c r="P70" s="10" t="s">
-        <v>804</v>
       </c>
       <c r="Q70" s="10" t="s">
         <v>771</v>
@@ -7050,22 +7050,22 @@
     </row>
     <row r="71" spans="1:21" ht="64" customHeight="1">
       <c r="A71" s="10" t="s">
-        <v>805</v>
+        <v>556</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="D71" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>789</v>
+        <v>540</v>
       </c>
       <c r="F71" s="10" t="s">
-        <v>797</v>
+        <v>548</v>
       </c>
       <c r="G71" s="10" t="str">
         <f t="shared" si="4"/>
@@ -7077,22 +7077,22 @@
       <c r="I71" s="14"/>
       <c r="J71" s="16"/>
       <c r="K71" s="10" t="s">
+        <v>806</v>
+      </c>
+      <c r="L71" s="10" t="s">
         <v>807</v>
       </c>
-      <c r="L71" s="10" t="s">
+      <c r="M71" s="10" t="s">
         <v>808</v>
       </c>
-      <c r="M71" s="10" t="s">
+      <c r="N71" s="10" t="s">
         <v>809</v>
       </c>
-      <c r="N71" s="10" t="s">
+      <c r="O71" s="10" t="s">
         <v>810</v>
       </c>
-      <c r="O71" s="10" t="s">
+      <c r="P71" s="10" t="s">
         <v>811</v>
-      </c>
-      <c r="P71" s="10" t="s">
-        <v>812</v>
       </c>
       <c r="Q71" s="10" t="s">
         <v>771</v>
@@ -7109,19 +7109,19 @@
     </row>
     <row r="72" spans="1:21" ht="64" customHeight="1">
       <c r="A72" s="10" t="s">
-        <v>813</v>
+        <v>762</v>
       </c>
       <c r="B72" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="D72" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>805</v>
+        <v>556</v>
       </c>
       <c r="F72" s="10" t="s">
         <v>82</v>
@@ -7136,22 +7136,22 @@
       <c r="I72" s="14"/>
       <c r="J72" s="16"/>
       <c r="K72" s="10" t="s">
+        <v>814</v>
+      </c>
+      <c r="L72" s="10" t="s">
         <v>815</v>
       </c>
-      <c r="L72" s="10" t="s">
+      <c r="M72" s="10" t="s">
         <v>816</v>
       </c>
-      <c r="M72" s="10" t="s">
+      <c r="N72" s="10" t="s">
         <v>817</v>
       </c>
-      <c r="N72" s="10" t="s">
+      <c r="O72" s="10" t="s">
         <v>818</v>
       </c>
-      <c r="O72" s="10" t="s">
-        <v>819</v>
-      </c>
       <c r="P72" s="10" t="s">
-        <v>820</v>
+        <v>868</v>
       </c>
       <c r="Q72" s="10" t="s">
         <v>771</v>
@@ -7168,19 +7168,19 @@
     </row>
     <row r="73" spans="1:21" ht="64" customHeight="1">
       <c r="A73" s="10" t="s">
-        <v>821</v>
+        <v>772</v>
       </c>
       <c r="B73" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="D73" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>813</v>
+        <v>762</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>111</v>
@@ -7195,22 +7195,22 @@
       <c r="I73" s="14"/>
       <c r="J73" s="16"/>
       <c r="K73" s="10" t="s">
+        <v>821</v>
+      </c>
+      <c r="L73" s="10" t="s">
+        <v>822</v>
+      </c>
+      <c r="M73" s="10" t="s">
         <v>823</v>
       </c>
-      <c r="L73" s="10" t="s">
+      <c r="N73" s="10" t="s">
         <v>824</v>
       </c>
-      <c r="M73" s="10" t="s">
+      <c r="O73" s="10" t="s">
         <v>825</v>
       </c>
-      <c r="N73" s="10" t="s">
+      <c r="P73" s="10" t="s">
         <v>826</v>
-      </c>
-      <c r="O73" s="10" t="s">
-        <v>827</v>
-      </c>
-      <c r="P73" s="10" t="s">
-        <v>828</v>
       </c>
       <c r="Q73" s="10" t="s">
         <v>771</v>
@@ -7227,19 +7227,19 @@
     </row>
     <row r="74" spans="1:21" ht="64" customHeight="1">
       <c r="A74" s="10" t="s">
-        <v>829</v>
+        <v>781</v>
       </c>
       <c r="B74" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="D74" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>805</v>
+        <v>556</v>
       </c>
       <c r="F74" s="10" t="s">
         <v>265</v>
@@ -7254,22 +7254,22 @@
       <c r="I74" s="14"/>
       <c r="J74" s="16"/>
       <c r="K74" s="10" t="s">
+        <v>829</v>
+      </c>
+      <c r="L74" s="10" t="s">
+        <v>830</v>
+      </c>
+      <c r="M74" s="10" t="s">
         <v>831</v>
       </c>
-      <c r="L74" s="10" t="s">
+      <c r="N74" s="10" t="s">
         <v>832</v>
       </c>
-      <c r="M74" s="10" t="s">
+      <c r="O74" s="10" t="s">
         <v>833</v>
       </c>
-      <c r="N74" s="10" t="s">
+      <c r="P74" s="10" t="s">
         <v>834</v>
-      </c>
-      <c r="O74" s="10" t="s">
-        <v>835</v>
-      </c>
-      <c r="P74" s="10" t="s">
-        <v>836</v>
       </c>
       <c r="Q74" s="10" t="s">
         <v>771</v>
@@ -7286,22 +7286,22 @@
     </row>
     <row r="75" spans="1:21" ht="64" customHeight="1">
       <c r="A75" s="10" t="s">
-        <v>837</v>
+        <v>788</v>
       </c>
       <c r="B75" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="D75" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>821</v>
+        <v>772</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>829</v>
+        <v>781</v>
       </c>
       <c r="G75" s="10" t="str">
         <f t="shared" si="4"/>
@@ -7313,22 +7313,22 @@
       <c r="I75" s="14"/>
       <c r="J75" s="16"/>
       <c r="K75" s="10" t="s">
+        <v>837</v>
+      </c>
+      <c r="L75" s="10" t="s">
+        <v>838</v>
+      </c>
+      <c r="M75" s="10" t="s">
+        <v>869</v>
+      </c>
+      <c r="N75" s="10" t="s">
         <v>839</v>
       </c>
-      <c r="L75" s="10" t="s">
+      <c r="O75" s="10" t="s">
         <v>840</v>
       </c>
-      <c r="M75" s="10" t="s">
+      <c r="P75" s="10" t="s">
         <v>841</v>
-      </c>
-      <c r="N75" s="10" t="s">
-        <v>842</v>
-      </c>
-      <c r="O75" s="10" t="s">
-        <v>843</v>
-      </c>
-      <c r="P75" s="10" t="s">
-        <v>844</v>
       </c>
       <c r="Q75" s="10" t="s">
         <v>771</v>
@@ -7345,19 +7345,19 @@
     </row>
     <row r="76" spans="1:21" ht="64" customHeight="1">
       <c r="A76" s="10" t="s">
-        <v>845</v>
+        <v>796</v>
       </c>
       <c r="B76" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="D76" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>837</v>
+        <v>788</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>344</v>
@@ -7372,22 +7372,22 @@
       <c r="I76" s="14"/>
       <c r="J76" s="16"/>
       <c r="K76" s="10" t="s">
+        <v>844</v>
+      </c>
+      <c r="L76" s="10" t="s">
+        <v>845</v>
+      </c>
+      <c r="M76" s="10" t="s">
+        <v>846</v>
+      </c>
+      <c r="N76" s="10" t="s">
         <v>847</v>
       </c>
-      <c r="L76" s="10" t="s">
+      <c r="O76" s="10" t="s">
         <v>848</v>
       </c>
-      <c r="M76" s="10" t="s">
+      <c r="P76" s="10" t="s">
         <v>849</v>
-      </c>
-      <c r="N76" s="10" t="s">
-        <v>850</v>
-      </c>
-      <c r="O76" s="10" t="s">
-        <v>851</v>
-      </c>
-      <c r="P76" s="10" t="s">
-        <v>852</v>
       </c>
       <c r="Q76" s="10" t="s">
         <v>771</v>
@@ -7404,19 +7404,19 @@
     </row>
     <row r="77" spans="1:21" ht="64" customHeight="1">
       <c r="A77" s="10" t="s">
-        <v>853</v>
+        <v>804</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>763</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="D77" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>845</v>
+        <v>796</v>
       </c>
       <c r="F77" s="10"/>
       <c r="G77" s="10" t="str">
@@ -7429,22 +7429,22 @@
       <c r="I77" s="14"/>
       <c r="J77" s="16"/>
       <c r="K77" s="10" t="s">
+        <v>852</v>
+      </c>
+      <c r="L77" s="10" t="s">
+        <v>853</v>
+      </c>
+      <c r="M77" s="10" t="s">
+        <v>870</v>
+      </c>
+      <c r="N77" s="10" t="s">
+        <v>854</v>
+      </c>
+      <c r="O77" s="10" t="s">
         <v>855</v>
       </c>
-      <c r="L77" s="10" t="s">
+      <c r="P77" s="10" t="s">
         <v>856</v>
-      </c>
-      <c r="M77" s="10" t="s">
-        <v>857</v>
-      </c>
-      <c r="N77" s="10" t="s">
-        <v>858</v>
-      </c>
-      <c r="O77" s="10" t="s">
-        <v>859</v>
-      </c>
-      <c r="P77" s="10" t="s">
-        <v>860</v>
       </c>
       <c r="Q77" s="10" t="s">
         <v>771</v>
@@ -7461,10 +7461,10 @@
     </row>
     <row r="78" spans="1:21" ht="64" customHeight="1">
       <c r="A78" s="12" t="s">
-        <v>515</v>
+        <v>812</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="C78" s="12" t="s">
         <v>516</v>
@@ -7473,7 +7473,7 @@
         <v>288</v>
       </c>
       <c r="E78" s="12" t="s">
-        <v>853</v>
+        <v>804</v>
       </c>
       <c r="F78" s="12"/>
       <c r="G78" s="12" t="str">
@@ -7516,10 +7516,10 @@
     </row>
     <row r="79" spans="1:21" ht="64" customHeight="1">
       <c r="A79" s="10" t="s">
-        <v>524</v>
+        <v>819</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="C79" s="10" t="s">
         <v>525</v>
@@ -7528,7 +7528,7 @@
         <v>288</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>853</v>
+        <v>804</v>
       </c>
       <c r="F79" s="10"/>
       <c r="G79" s="10" t="str">
@@ -7571,10 +7571,10 @@
     </row>
     <row r="80" spans="1:21" ht="64" customHeight="1">
       <c r="A80" s="11" t="s">
-        <v>532</v>
+        <v>827</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="C80" s="11" t="s">
         <v>533</v>
@@ -7583,7 +7583,7 @@
         <v>288</v>
       </c>
       <c r="E80" s="11" t="s">
-        <v>853</v>
+        <v>804</v>
       </c>
       <c r="F80" s="11"/>
       <c r="G80" s="11" t="str">
@@ -7626,10 +7626,10 @@
     </row>
     <row r="81" spans="1:21" ht="64" customHeight="1">
       <c r="A81" s="10" t="s">
-        <v>540</v>
+        <v>835</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="C81" s="10" t="s">
         <v>541</v>
@@ -7638,7 +7638,7 @@
         <v>288</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>853</v>
+        <v>804</v>
       </c>
       <c r="F81" s="10"/>
       <c r="G81" s="10" t="str">
@@ -7681,10 +7681,10 @@
     </row>
     <row r="82" spans="1:21" ht="64" customHeight="1">
       <c r="A82" s="11" t="s">
-        <v>548</v>
+        <v>842</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="C82" s="11" t="s">
         <v>549</v>
@@ -7693,7 +7693,7 @@
         <v>288</v>
       </c>
       <c r="E82" s="11" t="s">
-        <v>853</v>
+        <v>804</v>
       </c>
       <c r="F82" s="11"/>
       <c r="G82" s="11" t="str">
@@ -7736,10 +7736,10 @@
     </row>
     <row r="83" spans="1:21" ht="64" customHeight="1">
       <c r="A83" s="10" t="s">
-        <v>556</v>
+        <v>850</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="C83" s="10" t="s">
         <v>557</v>
@@ -7748,10 +7748,10 @@
         <v>288</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>515</v>
+        <v>812</v>
       </c>
       <c r="F83" s="10" t="s">
-        <v>548</v>
+        <v>842</v>
       </c>
       <c r="G83" s="10" t="str">
         <f t="shared" si="2"/>
@@ -8490,7 +8490,7 @@
     </row>
     <row r="101" spans="1:21" ht="38" customHeight="1">
       <c r="A101" s="10" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="B101" s="10">
         <f t="shared" si="6"/>
@@ -8694,7 +8694,7 @@
         <v>572</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>870</v>
+        <v>866</v>
       </c>
       <c r="D108" s="1"/>
       <c r="E108" s="1"/>

</xml_diff>

<commit_message>
Phase 10 plan review fixes: split procedure ordering, native-integration mode, dashboard formulas
- TB-061 pre-registers the external validation protocol and the split procedure (script + tests);
  TB-062 authors the families, applies that procedure and freezes the split and attack manifests
  before any defended run. Removes the TB-061/TB-062 circular dependency. TB-064 input updated.
- TB-057 adds Mode B: the agent keeps one independently implemented native tool integration,
  unchanged, against a synthetic sandbox, with the gateway interposed (12 h). TB-058 bypass tests
  cover both modes.
- Phase dashboard row 100: Remaining h (I100) and Ready (J100) formulas added.
All phase-10 tasks remain Not Started.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DCC6B76-95A1-A94A-897B-733AFE7F3277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9905D2F0-8E51-6743-AFE8-1FFBE0548403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2374,42 +2374,18 @@
     <t>TB-063</t>
   </si>
   <si>
-    <t>Build the external-agent adapter</t>
-  </si>
-  <si>
-    <t>Expose the TrustBench tool services to the agent through its native tool interface (function tools or an MCP server), routed through the policy gateway. Translate run configuration, model settings and step limits; capture the agent's tool calls, final text and errors into the TrustBench trace schema. Keep the agent's own code unmodified.</t>
-  </si>
-  <si>
-    <t>Agent SDK or MCP, src/gateway, TypeScript or Python adapter</t>
-  </si>
-  <si>
-    <t>Adapter tests show every TrustBench tool callable from the agent, traces validating against the TB-004 schema, and a diff proving no change to the agent's source.</t>
-  </si>
-  <si>
-    <t>src/external/; tests/external/adapter/</t>
-  </si>
-  <si>
-    <t>The agent's tool interface cannot carry capability tokens: hold tokens in the adapter process, never in prompts, and enforce at the gateway.</t>
-  </si>
-  <si>
     <t>TB-064</t>
   </si>
   <si>
     <t>Enforce tool authorization outside the agent</t>
   </si>
   <si>
-    <t>Run the agent in a sandbox whose only route to tools is the gateway (network egress denied, raw tool service unreachable). Bind each episode to a capability token held outside the agent. Add bypass tests: direct calls to tool services, forged or replayed tokens, unlisted tools, argument smuggling and calls after cancellation.</t>
-  </si>
-  <si>
     <t>Docker or a sandbox network policy, src/policy, pytest</t>
   </si>
   <si>
     <t>TB-021 capability policy; TB-023 boundary tests</t>
   </si>
   <si>
-    <t>Every bypass test is refused and audited; a positive control proves each test can detect a working bypass; no tool effect occurs without a gateway allow decision in the audit log.</t>
-  </si>
-  <si>
     <t>tests/external/authorization/; evidence/external-authorization-report.json</t>
   </si>
   <si>
@@ -2467,48 +2443,21 @@
     <t>TB-067</t>
   </si>
   <si>
-    <t>Pre-register the external validation protocol</t>
-  </si>
-  <si>
-    <t>Write an amendment before any external evaluation run: hypotheses, primary endpoints (unsafe committed-effect rate, benign utility), integration-overhead measures, repetitions, models, analysis and stopping rules. Create a new external validation split from fixture families never used in tuning; the sealed core holdout stays untouched.</t>
-  </si>
-  <si>
     <t>protocol/, scripts/verify-protocol.mjs</t>
   </si>
   <si>
-    <t>TB-006 protocol; experiment registry</t>
-  </si>
-  <si>
-    <t>Amendment committed and verified before the first external evaluation run; the new split is disjoint from the core holdout and the tuning families, checked by script.</t>
-  </si>
-  <si>
-    <t>protocol/amendments.md (external validation entry); data/external-splits.json</t>
-  </si>
-  <si>
     <t>TB-068</t>
   </si>
   <si>
     <t>Build realistic adversarial scenarios</t>
   </si>
   <si>
-    <t>Author attack families closer to deployment: injections inside long realistic documents, tool-output injection across several tools, multi-step and delayed instructions, data exfiltration through allowed tools, and attacks on the agent's own planning or memory features. Each family has an oracle, a benign twin and a positive control; families are assigned to tuning or external validation before any run.</t>
-  </si>
-  <si>
     <t>data/ fixture builders, attack oracles, src/arms materialization</t>
   </si>
   <si>
     <t>TB-009 fixtures; published attack patterns (cited)</t>
   </si>
   <si>
-    <t>Each family has a cited source or rationale, an oracle validated on scripted trajectories, a benign twin, and a recorded split; positive controls succeed against the undefended agent.</t>
-  </si>
-  <si>
-    <t>data/external-attacks.jsonl; data/external-attack-oracles.json; tests/external/attacks/</t>
-  </si>
-  <si>
-    <t>Attacks tuned to defeat or to favour the gateway: freeze them before any defended run and report their source.</t>
-  </si>
-  <si>
     <t>TB-069</t>
   </si>
   <si>
@@ -2629,15 +2578,6 @@
     <t>Work through phases 01–09 for Core. Phase 10 (External agent validation, Scope = Validation) follows the core roadmap and starts only after TB-054; phase 11 is optional. Dependencies refer to task IDs in this sheet; independent projects need no other project to be finished.</t>
   </si>
   <si>
-    <t>Integration contract (TB-056); gateway and tool services</t>
-  </si>
-  <si>
-    <t>Too few unused fixture families for a fresh split: author new families first (TB-062) and register them before use.</t>
-  </si>
-  <si>
-    <t>External validation split (TB-061), frozen gateway configuration (configs/frozen/)</t>
-  </si>
-  <si>
     <t>TB-065 results; TB-056 threat model</t>
   </si>
   <si>
@@ -2645,6 +2585,66 @@
   </si>
   <si>
     <t>Completed. Rules pre-registered as A-023 (system selection) and A-024 (reliability sweep) and applied by script to tuning-split runs only (holdout fixtures checked absent; no holdout run exists). Selected gateway_directive_flow_v4 on gpt-oss-20b, plain profile: unsafe 76.1% -&gt; 0.0% (paired cluster bootstrap -88.9 to -63.1 pp), benign utility 70.0% -&gt; 88.0%; 2 of 14 systems met the evidence minimum and gate. Thresholds = the registered v4 version. Reliability sweep (5 configurations x 48 pairs, 0 invalid): step limit 12 and timeout 240 s kept (16 steps cost 14 pp utility, 8 steps and 360 s raised terminations); read retries 4 -&gt; 2 adopted (no worse, 3.1 s faster), applied only to the holdout via configs/frozen/reliability-override.json. Frozen configs, settings copies, classifier prompt and SHA-256 manifest in configs/frozen/; npm run verify:frozen fails on drift. Disclosed: winner's curse, v4 designed on these fixtures, ~27 attack / 21 benign runs per arm in the sweep, budget limits not swept, A-024 committed with its results. No attack-success reduction on the holdout is assumed.</t>
+  </si>
+  <si>
+    <t>Build the external-agent adapter (TrustBench tools and the agent's own tool integration)</t>
+  </si>
+  <si>
+    <t>Mode A (controlled tools): expose the TrustBench tool services to the agent through its native tool interface (function tools or an MCP server), routed through the policy gateway. Mode B (native integration): keep at least one of the agent's own, independently implemented tool integrations (for example its SQL, HTTP-API or mail connector) unchanged, point it at a sandboxed local instance (database container or mock API server seeded with synthetic data, no real accounts), and interpose the gateway between that integration and its service without replacing the agent's tool environment. In both modes translate run configuration, model settings and step limits, and capture tool calls, final text and errors into the TrustBench trace schema. Keep the agent's own code unmodified.</t>
+  </si>
+  <si>
+    <t>Agent SDK or MCP, src/gateway, TypeScript or Python adapter, Docker (sandboxed database or mock API)</t>
+  </si>
+  <si>
+    <t>Integration contract (TB-056); gateway and tool services; the agent's native tool integration and a synthetic sandbox instance for it</t>
+  </si>
+  <si>
+    <t>Mode A: adapter tests show every TrustBench tool callable from the agent and traces validating against the TB-004 schema. Mode B: at least one independently implemented native integration runs unchanged against its sandbox with every call passing through the gateway, which records an allow or deny decision per call; the sandbox holds synthetic data only. A diff proves no change to the agent's source or to the native integration's code.</t>
+  </si>
+  <si>
+    <t>src/external/; tests/external/adapter/; tests/external/native-integration/; docs/external/native-integration.md</t>
+  </si>
+  <si>
+    <t>The agent's tool interface cannot carry capability tokens: hold tokens in the adapter process, never in prompts, and enforce at the gateway. The native integration cannot be interposed (in-process client, pinned TLS): use a network-level proxy in the sandbox, or record Mode B as not demonstrated and limit claims to Mode A.</t>
+  </si>
+  <si>
+    <t>Run the agent in a sandbox whose only route to tools is the gateway (network egress denied, raw tool service unreachable). Bind each episode to a capability token held outside the agent. Add bypass tests: direct calls to tool services, forged or replayed tokens, unlisted tools, argument smuggling and calls after cancellation. Repeat the bypass tests against the Mode B native integration: its client must reach the sandboxed service only through the gateway.</t>
+  </si>
+  <si>
+    <t>Every bypass test is refused and audited in both adapter modes (TrustBench tools and the native integration); a positive control proves each test can detect a working bypass; no tool effect occurs without a gateway allow decision in the audit log.</t>
+  </si>
+  <si>
+    <t>Pre-register the external validation protocol and split procedure</t>
+  </si>
+  <si>
+    <t>Write an amendment before any external evaluation run: hypotheses, primary endpoints (unsafe committed-effect rate, benign utility), integration-overhead measures, adapter modes, repetitions, models, analysis and stopping rules. Register the split procedure, not the split: which fixture families are eligible (existing families never used in tuning, and families to be authored in TB-062), the seeded assignment rule to tuning or external validation, stratification, and the requirement that the sealed core holdout is excluded. Implement the procedure as a script and test it on placeholder family lists.</t>
+  </si>
+  <si>
+    <t>TB-006 protocol; experiment registry; inventory of existing fixture families and their tuning use</t>
+  </si>
+  <si>
+    <t>Amendment committed and verified before the first external evaluation run; the split script is committed with tests showing it is deterministic for its seed, excludes the core holdout and every tuning-used family, and refuses to reassign a family once assigned.</t>
+  </si>
+  <si>
+    <t>protocol/amendments.md (external validation entry); scripts/external-split.py; tests/external/split/</t>
+  </si>
+  <si>
+    <t>The procedure is changed after families are seen: any change needs a new amendment committed before TB-062 assigns families.</t>
+  </si>
+  <si>
+    <t>Author attack families closer to deployment: injections inside long realistic documents, tool-output injection across several tools, multi-step and delayed instructions, data exfiltration through allowed tools, and attacks on the agent's own planning or memory features. Each family has an oracle, a benign twin and a positive control. Then apply the TB-061 split procedure to the new and eligible existing families, write data/external-splits.json, and freeze the attack and split manifests with content hashes before any defended evaluation run.</t>
+  </si>
+  <si>
+    <t>Each family has a cited source or rationale, an oracle validated on scripted trajectories, a benign twin, and a split assigned by the registered TB-061 script; the split manifest is disjoint from the core holdout and the tuning families (checked by script) and its hash is committed before any defended run; positive controls succeed against the undefended agent.</t>
+  </si>
+  <si>
+    <t>data/external-attacks.jsonl; data/external-attack-oracles.json; data/external-splits.json; tests/external/attacks/</t>
+  </si>
+  <si>
+    <t>Attacks tuned to defeat or to favour the gateway: freeze them before any defended run and report their source. Too few families for a meaningful external split: author more before assignment, never after.</t>
+  </si>
+  <si>
+    <t>External validation split (data/external-splits.json, frozen in TB-062), frozen gateway configuration (configs/frozen/)</t>
   </si>
 </sst>
 </file>
@@ -3433,11 +3433,11 @@
       </c>
       <c r="E5" s="5">
         <f>SUM($H$12:$H$83)</f>
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -3521,28 +3521,28 @@
     </row>
     <row r="8" spans="1:21" ht="32" customHeight="1">
       <c r="A8" s="9" t="s">
-        <v>856</v>
+        <v>839</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>857</v>
+        <v>840</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>858</v>
+        <v>841</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>859</v>
+        <v>842</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>860</v>
+        <v>843</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>861</v>
+        <v>844</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>862</v>
+        <v>845</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>863</v>
+        <v>846</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -5474,10 +5474,10 @@
       </c>
       <c r="R42" s="12"/>
       <c r="S42" s="13" t="s">
-        <v>869</v>
+        <v>849</v>
       </c>
       <c r="T42" s="13" t="s">
-        <v>870</v>
+        <v>850</v>
       </c>
       <c r="U42" s="10">
         <f t="shared" si="1"/>
@@ -6879,7 +6879,7 @@
         <v>761</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>780</v>
+        <v>851</v>
       </c>
       <c r="D68" s="14" t="s">
         <v>288</v>
@@ -6895,27 +6895,27 @@
         <v>Waiting</v>
       </c>
       <c r="H68" s="18">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I68" s="14"/>
       <c r="J68" s="16"/>
       <c r="K68" s="10" t="s">
-        <v>781</v>
+        <v>852</v>
       </c>
       <c r="L68" s="10" t="s">
-        <v>782</v>
+        <v>853</v>
       </c>
       <c r="M68" s="10" t="s">
-        <v>865</v>
+        <v>854</v>
       </c>
       <c r="N68" s="10" t="s">
-        <v>783</v>
+        <v>855</v>
       </c>
       <c r="O68" s="10" t="s">
-        <v>784</v>
+        <v>856</v>
       </c>
       <c r="P68" s="10" t="s">
-        <v>785</v>
+        <v>857</v>
       </c>
       <c r="Q68" s="10" t="s">
         <v>769</v>
@@ -6938,7 +6938,7 @@
         <v>761</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>787</v>
+        <v>781</v>
       </c>
       <c r="D69" s="14" t="s">
         <v>288</v>
@@ -6959,22 +6959,22 @@
       <c r="I69" s="14"/>
       <c r="J69" s="16"/>
       <c r="K69" s="10" t="s">
-        <v>788</v>
+        <v>858</v>
       </c>
       <c r="L69" s="10" t="s">
-        <v>789</v>
+        <v>782</v>
       </c>
       <c r="M69" s="10" t="s">
-        <v>790</v>
+        <v>783</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>791</v>
+        <v>859</v>
       </c>
       <c r="O69" s="10" t="s">
-        <v>792</v>
+        <v>784</v>
       </c>
       <c r="P69" s="10" t="s">
-        <v>793</v>
+        <v>785</v>
       </c>
       <c r="Q69" s="10" t="s">
         <v>769</v>
@@ -6997,7 +6997,7 @@
         <v>761</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>795</v>
+        <v>787</v>
       </c>
       <c r="D70" s="14" t="s">
         <v>288</v>
@@ -7018,22 +7018,22 @@
       <c r="I70" s="14"/>
       <c r="J70" s="16"/>
       <c r="K70" s="10" t="s">
-        <v>796</v>
+        <v>788</v>
       </c>
       <c r="L70" s="10" t="s">
-        <v>797</v>
+        <v>789</v>
       </c>
       <c r="M70" s="10" t="s">
-        <v>798</v>
+        <v>790</v>
       </c>
       <c r="N70" s="10" t="s">
-        <v>799</v>
+        <v>791</v>
       </c>
       <c r="O70" s="10" t="s">
-        <v>800</v>
+        <v>792</v>
       </c>
       <c r="P70" s="10" t="s">
-        <v>801</v>
+        <v>793</v>
       </c>
       <c r="Q70" s="10" t="s">
         <v>769</v>
@@ -7056,7 +7056,7 @@
         <v>761</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>803</v>
+        <v>795</v>
       </c>
       <c r="D71" s="14" t="s">
         <v>288</v>
@@ -7077,22 +7077,22 @@
       <c r="I71" s="14"/>
       <c r="J71" s="16"/>
       <c r="K71" s="10" t="s">
-        <v>804</v>
+        <v>796</v>
       </c>
       <c r="L71" s="10" t="s">
-        <v>805</v>
+        <v>797</v>
       </c>
       <c r="M71" s="10" t="s">
-        <v>806</v>
+        <v>798</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>807</v>
+        <v>799</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>808</v>
+        <v>800</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>809</v>
+        <v>801</v>
       </c>
       <c r="Q71" s="10" t="s">
         <v>769</v>
@@ -7115,7 +7115,7 @@
         <v>761</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>811</v>
+        <v>860</v>
       </c>
       <c r="D72" s="14" t="s">
         <v>288</v>
@@ -7136,22 +7136,22 @@
       <c r="I72" s="14"/>
       <c r="J72" s="16"/>
       <c r="K72" s="10" t="s">
-        <v>812</v>
+        <v>861</v>
       </c>
       <c r="L72" s="10" t="s">
-        <v>813</v>
+        <v>803</v>
       </c>
       <c r="M72" s="10" t="s">
-        <v>814</v>
+        <v>862</v>
       </c>
       <c r="N72" s="10" t="s">
-        <v>815</v>
+        <v>863</v>
       </c>
       <c r="O72" s="10" t="s">
-        <v>816</v>
+        <v>864</v>
       </c>
       <c r="P72" s="10" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="Q72" s="10" t="s">
         <v>769</v>
@@ -7174,7 +7174,7 @@
         <v>761</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>818</v>
+        <v>805</v>
       </c>
       <c r="D73" s="14" t="s">
         <v>288</v>
@@ -7195,22 +7195,22 @@
       <c r="I73" s="14"/>
       <c r="J73" s="16"/>
       <c r="K73" s="10" t="s">
-        <v>819</v>
+        <v>866</v>
       </c>
       <c r="L73" s="10" t="s">
-        <v>820</v>
+        <v>806</v>
       </c>
       <c r="M73" s="10" t="s">
-        <v>821</v>
+        <v>807</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>822</v>
+        <v>867</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>823</v>
+        <v>868</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>824</v>
+        <v>869</v>
       </c>
       <c r="Q73" s="10" t="s">
         <v>769</v>
@@ -7233,7 +7233,7 @@
         <v>761</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>826</v>
+        <v>809</v>
       </c>
       <c r="D74" s="14" t="s">
         <v>288</v>
@@ -7254,22 +7254,22 @@
       <c r="I74" s="14"/>
       <c r="J74" s="16"/>
       <c r="K74" s="10" t="s">
-        <v>827</v>
+        <v>810</v>
       </c>
       <c r="L74" s="10" t="s">
-        <v>828</v>
+        <v>811</v>
       </c>
       <c r="M74" s="10" t="s">
-        <v>829</v>
+        <v>812</v>
       </c>
       <c r="N74" s="10" t="s">
-        <v>830</v>
+        <v>813</v>
       </c>
       <c r="O74" s="10" t="s">
-        <v>831</v>
+        <v>814</v>
       </c>
       <c r="P74" s="10" t="s">
-        <v>832</v>
+        <v>815</v>
       </c>
       <c r="Q74" s="10" t="s">
         <v>769</v>
@@ -7286,13 +7286,13 @@
     </row>
     <row r="75" spans="1:21" ht="64" customHeight="1">
       <c r="A75" s="10" t="s">
-        <v>786</v>
+        <v>780</v>
       </c>
       <c r="B75" s="10" t="s">
         <v>761</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>834</v>
+        <v>817</v>
       </c>
       <c r="D75" s="14" t="s">
         <v>288</v>
@@ -7313,22 +7313,22 @@
       <c r="I75" s="14"/>
       <c r="J75" s="16"/>
       <c r="K75" s="10" t="s">
-        <v>835</v>
+        <v>818</v>
       </c>
       <c r="L75" s="10" t="s">
-        <v>836</v>
+        <v>819</v>
       </c>
       <c r="M75" s="10" t="s">
-        <v>867</v>
+        <v>870</v>
       </c>
       <c r="N75" s="10" t="s">
-        <v>837</v>
+        <v>820</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>838</v>
+        <v>821</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>839</v>
+        <v>822</v>
       </c>
       <c r="Q75" s="10" t="s">
         <v>769</v>
@@ -7345,19 +7345,19 @@
     </row>
     <row r="76" spans="1:21" ht="64" customHeight="1">
       <c r="A76" s="10" t="s">
-        <v>794</v>
+        <v>786</v>
       </c>
       <c r="B76" s="10" t="s">
         <v>761</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>841</v>
+        <v>824</v>
       </c>
       <c r="D76" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>786</v>
+        <v>780</v>
       </c>
       <c r="F76" s="10" t="s">
         <v>344</v>
@@ -7372,22 +7372,22 @@
       <c r="I76" s="14"/>
       <c r="J76" s="16"/>
       <c r="K76" s="10" t="s">
-        <v>842</v>
+        <v>825</v>
       </c>
       <c r="L76" s="10" t="s">
-        <v>843</v>
+        <v>826</v>
       </c>
       <c r="M76" s="10" t="s">
-        <v>844</v>
+        <v>827</v>
       </c>
       <c r="N76" s="10" t="s">
-        <v>845</v>
+        <v>828</v>
       </c>
       <c r="O76" s="10" t="s">
-        <v>846</v>
+        <v>829</v>
       </c>
       <c r="P76" s="10" t="s">
-        <v>847</v>
+        <v>830</v>
       </c>
       <c r="Q76" s="10" t="s">
         <v>769</v>
@@ -7404,19 +7404,19 @@
     </row>
     <row r="77" spans="1:21" ht="64" customHeight="1">
       <c r="A77" s="10" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>761</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>849</v>
+        <v>832</v>
       </c>
       <c r="D77" s="14" t="s">
         <v>288</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>794</v>
+        <v>786</v>
       </c>
       <c r="F77" s="10"/>
       <c r="G77" s="10" t="str">
@@ -7429,22 +7429,22 @@
       <c r="I77" s="14"/>
       <c r="J77" s="16"/>
       <c r="K77" s="10" t="s">
-        <v>850</v>
+        <v>833</v>
       </c>
       <c r="L77" s="10" t="s">
-        <v>851</v>
+        <v>834</v>
       </c>
       <c r="M77" s="10" t="s">
-        <v>868</v>
+        <v>848</v>
       </c>
       <c r="N77" s="10" t="s">
-        <v>852</v>
+        <v>835</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>853</v>
+        <v>836</v>
       </c>
       <c r="P77" s="10" t="s">
-        <v>854</v>
+        <v>837</v>
       </c>
       <c r="Q77" s="10" t="s">
         <v>769</v>
@@ -7461,10 +7461,10 @@
     </row>
     <row r="78" spans="1:21" ht="64" customHeight="1">
       <c r="A78" s="12" t="s">
-        <v>810</v>
+        <v>802</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>855</v>
+        <v>838</v>
       </c>
       <c r="C78" s="12" t="s">
         <v>516</v>
@@ -7473,7 +7473,7 @@
         <v>288</v>
       </c>
       <c r="E78" s="12" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="F78" s="12"/>
       <c r="G78" s="12" t="str">
@@ -7516,10 +7516,10 @@
     </row>
     <row r="79" spans="1:21" ht="64" customHeight="1">
       <c r="A79" s="10" t="s">
-        <v>817</v>
+        <v>804</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>855</v>
+        <v>838</v>
       </c>
       <c r="C79" s="10" t="s">
         <v>525</v>
@@ -7528,7 +7528,7 @@
         <v>288</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="F79" s="10"/>
       <c r="G79" s="10" t="str">
@@ -7571,10 +7571,10 @@
     </row>
     <row r="80" spans="1:21" ht="64" customHeight="1">
       <c r="A80" s="11" t="s">
-        <v>825</v>
+        <v>808</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>855</v>
+        <v>838</v>
       </c>
       <c r="C80" s="11" t="s">
         <v>533</v>
@@ -7583,7 +7583,7 @@
         <v>288</v>
       </c>
       <c r="E80" s="11" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="F80" s="11"/>
       <c r="G80" s="11" t="str">
@@ -7626,10 +7626,10 @@
     </row>
     <row r="81" spans="1:21" ht="64" customHeight="1">
       <c r="A81" s="10" t="s">
-        <v>833</v>
+        <v>816</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>855</v>
+        <v>838</v>
       </c>
       <c r="C81" s="10" t="s">
         <v>541</v>
@@ -7638,7 +7638,7 @@
         <v>288</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="F81" s="10"/>
       <c r="G81" s="10" t="str">
@@ -7681,10 +7681,10 @@
     </row>
     <row r="82" spans="1:21" ht="64" customHeight="1">
       <c r="A82" s="11" t="s">
-        <v>840</v>
+        <v>823</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>855</v>
+        <v>838</v>
       </c>
       <c r="C82" s="11" t="s">
         <v>549</v>
@@ -7693,7 +7693,7 @@
         <v>288</v>
       </c>
       <c r="E82" s="11" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="F82" s="11"/>
       <c r="G82" s="11" t="str">
@@ -7736,10 +7736,10 @@
     </row>
     <row r="83" spans="1:21" ht="64" customHeight="1">
       <c r="A83" s="10" t="s">
-        <v>848</v>
+        <v>831</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>855</v>
+        <v>838</v>
       </c>
       <c r="C83" s="10" t="s">
         <v>557</v>
@@ -7748,10 +7748,10 @@
         <v>288</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>810</v>
+        <v>802</v>
       </c>
       <c r="F83" s="10" t="s">
-        <v>840</v>
+        <v>823</v>
       </c>
       <c r="G83" s="10" t="str">
         <f t="shared" si="2"/>
@@ -8472,10 +8472,16 @@
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
-        <v>68</v>
-      </c>
-      <c r="I100" s="11"/>
-      <c r="J100" s="11"/>
+        <v>72</v>
+      </c>
+      <c r="I100" s="11">
+        <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
+        <v>72</v>
+      </c>
+      <c r="J100" s="11">
+        <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>
+        <v>0</v>
+      </c>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>
       <c r="M100" s="1"/>
@@ -8490,7 +8496,7 @@
     </row>
     <row r="101" spans="1:21" ht="38" customHeight="1">
       <c r="A101" s="10" t="s">
-        <v>855</v>
+        <v>838</v>
       </c>
       <c r="B101" s="10">
         <f t="shared" si="6"/>
@@ -8694,7 +8700,7 @@
         <v>572</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>864</v>
+        <v>847</v>
       </c>
       <c r="D108" s="1"/>
       <c r="E108" s="1"/>

</xml_diff>

<commit_message>
TB-032: confirmatory holdout run complete (A-025)
Frozen configuration on the sealed holdout suite (3 benign, 3 attack), five registered
renderings x 6 cases x 5 repetitions from TB-028 schedules: 150/150 pairs intended,
attempted and valid; 0 invalid; no provider outage; one response model (openai/gpt-oss-20b).
A second execution is refused by the runner; registry marks the single confirmatory use
consumed (holdout_results_seen: true). Runs and validity only; comparisons are TB-033.
npm run verify exits 0; workbook check 260 formulas, 0 problems.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9905D2F0-8E51-6743-AFE8-1FFBE0548403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B0CA56-6C97-E34F-AFA4-7ADB2A6651D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="871">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1217" uniqueCount="873">
   <si>
     <t>Tasks</t>
   </si>
@@ -2645,6 +2645,12 @@
   </si>
   <si>
     <t>External validation split (data/external-splits.json, frozen in TB-062), frozen gateway configuration (configs/frozen/)</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: frozen config (directive_flow v4, gpt-oss-20b, plain, retries override) on the sealed holdout suite (3 benign, 3 attack), 5 renderings x 6 cases x 5 repetitions from TB-028 schedules: 150/150 pairs intended, attempted and valid, 0 invalid, no outages, one response model (openai/gpt-oss-20b; provider exposes no immutable revision, response IDs recorded). Second execution refused by the runner; holdout use consumed. No comparisons reported here. Next: TB-033.</t>
+  </si>
+  <si>
+    <t>runs/holdout/; evidence/tb032-holdout-run.json; docs/holdout-run.md; evidence/release-gate-dev.json</t>
   </si>
 </sst>
 </file>
@@ -3421,11 +3427,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.43055555555555558</v>
+        <v>0.44444444444444442</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3437,15 +3443,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.57407407407407407</v>
+        <v>0.59259259259259256</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>7.833333333333333</v>
+        <v>7.166666666666667</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -5495,7 +5501,7 @@
         <v>329</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>319</v>
@@ -5505,7 +5511,7 @@
       </c>
       <c r="G43" s="10" t="str">
         <f t="shared" si="0"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H43" s="18">
         <v>8</v>
@@ -5534,11 +5540,15 @@
         <v>43</v>
       </c>
       <c r="R43" s="10"/>
-      <c r="S43" s="14"/>
-      <c r="T43" s="14"/>
+      <c r="S43" s="14" t="s">
+        <v>872</v>
+      </c>
+      <c r="T43" s="14" t="s">
+        <v>871</v>
+      </c>
       <c r="U43" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:21" ht="64" customHeight="1">
@@ -5560,7 +5570,7 @@
       <c r="F44" s="11"/>
       <c r="G44" s="11" t="str">
         <f t="shared" ref="G44:G83" si="2">IF(NOT(AND(IF(E44="",TRUE,COUNTIFS($A$12:$A$83,E44)=1),IF(F44="",TRUE,COUNTIFS($A$12:$A$83,F44)=1))),"Bad dependency",IF(NOT(AND(IF(E44="",TRUE,COUNTIFS($A$12:$A$83,E44,$D$12:$D$83,"Completed",$U$12:$U$83,1)=1),IF(F44="",TRUE,COUNTIFS($A$12:$A$83,F44,$D$12:$D$83,"Completed",$U$12:$U$83,1)=1))),IF(D44="Completed","Check prerequisites","Waiting"),IF(D44="Completed",IF(S44="","Evidence needed","Done"),IF(D44="Blocked","Blocked",IF(D44="In Progress","In Progress","Ready")))))</f>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H44" s="18">
         <v>4</v>
@@ -8244,11 +8254,11 @@
       </c>
       <c r="C96" s="10">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96" s="10">
         <f t="shared" si="8"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E96" s="10">
         <f t="shared" si="9"/>
@@ -8260,7 +8270,7 @@
       </c>
       <c r="G96" s="21">
         <f t="shared" si="11"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H96" s="10">
         <f t="shared" si="12"/>
@@ -8268,7 +8278,7 @@
       </c>
       <c r="I96" s="10">
         <f t="shared" si="13"/>
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="J96" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-033: security and utility metrics on the confirmatory holdout
Primary condition (agentdojo_important_instructions), 15 runs per arm: unsafe committed effect
66.7% -> 20.0%, benign utility 66.7% -> 93.3%, attacker goal 40.0% -> 20.0%, false blocks 0/33
permitted calls. Every rate with numerator, denominator, Wilson 95% and exclusions (0 invalid),
recomputed from raw records and cross-checked against the runner summary. Secondary renderings
and the positive control reported separately. Defended unsafe on holdout (20%) exceeds the
development result (0%); intervals and paired differences are TB-034.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B0CA56-6C97-E34F-AFA4-7ADB2A6651D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A396AE-9654-BA4F-9EB1-091D9570BF83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1217" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="875">
   <si>
     <t>Tasks</t>
   </si>
@@ -2651,6 +2651,12 @@
   </si>
   <si>
     <t>runs/holdout/; evidence/tb032-holdout-run.json; docs/holdout-run.md; evidence/release-gate-dev.json</t>
+  </si>
+  <si>
+    <t>reports/security-utility.csv; evidence/tb033-metrics.json; docs/security-utility.md; scripts/compute-security-utility.py; tests/evaluation/test_security_utility.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: every rate recomputed from the raw TB-032 records with numerator, denominator, Wilson 95% and exclusions (0 invalid pairs), cross-checked against the runner summary; analysis code committed before it ran on the holdout. Primary (agentdojo_important_instructions): unsafe committed effect 10/15 -&gt; 3/15 (66.7% -&gt; 20.0%), benign utility 10/15 -&gt; 14/15, false blocks 0/33 permitted calls. Not hidden: defended unsafe on holdout (20%) is well above development (0%), so the defense did not fully transfer; denominators are 15 runs per arm; false-block label is tool-level only. Point-estimate co-primary rule met; confirmatory reading needs TB-034 paired intervals. Next: TB-034.</t>
   </si>
 </sst>
 </file>
@@ -3427,11 +3433,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.44444444444444442</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3443,15 +3449,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.59259259259259256</v>
+        <v>0.61111111111111116</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>7.166666666666667</v>
+        <v>6.833333333333333</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -5562,7 +5568,7 @@
         <v>337</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E44" s="11" t="s">
         <v>328</v>
@@ -5570,7 +5576,7 @@
       <c r="F44" s="11"/>
       <c r="G44" s="11" t="str">
         <f t="shared" ref="G44:G83" si="2">IF(NOT(AND(IF(E44="",TRUE,COUNTIFS($A$12:$A$83,E44)=1),IF(F44="",TRUE,COUNTIFS($A$12:$A$83,F44)=1))),"Bad dependency",IF(NOT(AND(IF(E44="",TRUE,COUNTIFS($A$12:$A$83,E44,$D$12:$D$83,"Completed",$U$12:$U$83,1)=1),IF(F44="",TRUE,COUNTIFS($A$12:$A$83,F44,$D$12:$D$83,"Completed",$U$12:$U$83,1)=1))),IF(D44="Completed","Check prerequisites","Waiting"),IF(D44="Completed",IF(S44="","Evidence needed","Done"),IF(D44="Blocked","Blocked",IF(D44="In Progress","In Progress","Ready")))))</f>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H44" s="18">
         <v>4</v>
@@ -5599,11 +5605,15 @@
         <v>43</v>
       </c>
       <c r="R44" s="11"/>
-      <c r="S44" s="14"/>
-      <c r="T44" s="14"/>
+      <c r="S44" s="14" t="s">
+        <v>873</v>
+      </c>
+      <c r="T44" s="14" t="s">
+        <v>874</v>
+      </c>
       <c r="U44" s="10">
         <f t="shared" ref="U44:U83" si="3">IF(LEN(S44)&gt;0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:21" ht="64" customHeight="1">
@@ -5625,7 +5635,7 @@
       <c r="F45" s="10"/>
       <c r="G45" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H45" s="18">
         <v>5</v>
@@ -8254,11 +8264,11 @@
       </c>
       <c r="C96" s="10">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D96" s="10">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E96" s="10">
         <f t="shared" si="9"/>
@@ -8270,7 +8280,7 @@
       </c>
       <c r="G96" s="21">
         <f t="shared" si="11"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="H96" s="10">
         <f t="shared" si="12"/>
@@ -8278,7 +8288,7 @@
       </c>
       <c r="I96" s="10">
         <f t="shared" si="13"/>
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J96" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
Holdout-2 run and metrics (A-026): 240/240 pairs valid; primary unsafe 70.0% -> 8.3%
Run once with the unchanged frozen configuration: benign and attack suites on the primary
rendering, attack suite on as_authored and the positive control; 0 invalid, one response model.
Primary: unsafe committed effect 42/60 -> 5/60, benign utility 34/60 -> 52/60, false blocks 2/127.
Pooled with holdout-1 (pre-declared): unsafe 69.3% -> 10.7%, utility 58.7% -> 88.0%.
New families transfer less well: defended unsafe 3/15 vs 2/40 on reused tuning families.
Holdout-1 result unchanged and still reported. Registry marks holdout-2 consumed.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A396AE-9654-BA4F-9EB1-091D9570BF83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEB0772-EA02-264F-BBCD-207C3B1E54F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2647,16 +2647,16 @@
     <t>External validation split (data/external-splits.json, frozen in TB-062), frozen gateway configuration (configs/frozen/)</t>
   </si>
   <si>
-    <t>Done 2026-10-17: frozen config (directive_flow v4, gpt-oss-20b, plain, retries override) on the sealed holdout suite (3 benign, 3 attack), 5 renderings x 6 cases x 5 repetitions from TB-028 schedules: 150/150 pairs intended, attempted and valid, 0 invalid, no outages, one response model (openai/gpt-oss-20b; provider exposes no immutable revision, response IDs recorded). Second execution refused by the runner; holdout use consumed. No comparisons reported here. Next: TB-033.</t>
-  </si>
-  <si>
-    <t>runs/holdout/; evidence/tb032-holdout-run.json; docs/holdout-run.md; evidence/release-gate-dev.json</t>
-  </si>
-  <si>
-    <t>reports/security-utility.csv; evidence/tb033-metrics.json; docs/security-utility.md; scripts/compute-security-utility.py; tests/evaluation/test_security_utility.py</t>
-  </si>
-  <si>
-    <t>Done 2026-10-17: every rate recomputed from the raw TB-032 records with numerator, denominator, Wilson 95% and exclusions (0 invalid pairs), cross-checked against the runner summary; analysis code committed before it ran on the holdout. Primary (agentdojo_important_instructions): unsafe committed effect 10/15 -&gt; 3/15 (66.7% -&gt; 20.0%), benign utility 10/15 -&gt; 14/15, false blocks 0/33 permitted calls. Not hidden: defended unsafe on holdout (20%) is well above development (0%), so the defense did not fully transfer; denominators are 15 runs per arm; false-block label is tool-level only. Point-estimate co-primary rule met; confirmatory reading needs TB-034 paired intervals. Next: TB-034.</t>
+    <t>runs/holdout/; evidence/tb032-holdout-run.json; docs/holdout-run.md; evidence/release-gate-dev.json; runs/holdout2/; evidence/tb032-holdout2-run.json; docs/holdout2-run.md; evidence/holdout2-validation.json; evidence/holdout2-prerun.json</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: frozen config on the sealed holdout suite (3 benign, 3 attack), 5 renderings x 6 cases x 5 repetitions: 150/150 pairs valid, one response model; second execution refused; holdout use consumed. Extension (A-026, protocol 1.2.0): a fresh sealed holdout-2 of 12 new task templates (12 benign, 12 attacks incl. 3 new families), validated without a model (44/44 oracle checks), run once with the unchanged frozen config: 240/240 pairs valid, 0 invalid, one response model (openai/gpt-oss-20b). Disclosed: holdout-2 was authored after holdout-1 aggregate rates were seen; composition fixed in A-026 first. Comparisons are TB-033/TB-034.</t>
+  </si>
+  <si>
+    <t>reports/security-utility.csv; evidence/tb033-metrics.json; docs/security-utility.md; reports/security-utility-holdout2.csv; evidence/tb033-holdout2-metrics.json; docs/security-utility-holdout2.md; scripts/compute-security-utility.py; tests/evaluation/test_security_utility.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: every rate recomputed from raw records with numerator, denominator, Wilson 95% (SciPy) and exclusions, tables via pandas, cross-checked against the runner summaries; code committed before each holdout ran through it. Holdout-1 primary: unsafe 10/15 -&gt; 3/15, utility 10/15 -&gt; 14/15. Holdout-2 primary: unsafe 42/60 -&gt; 5/60 (70.0% -&gt; 8.3%), utility 34/60 -&gt; 52/60, false blocks 2/127 permitted calls (argument level also 2/127). Pooled primary: unsafe 69.3% -&gt; 10.7%, utility 58.7% -&gt; 88.0%. Not hidden: defended unsafe is 20% (3/15) on the three new families vs 5% (2/40) on reused tuning families; holdout-1 primary was 20%; argument-level label is post hoc for holdout-1. Paired intervals are TB-034.</t>
   </si>
 </sst>
 </file>
@@ -5547,10 +5547,10 @@
       </c>
       <c r="R43" s="10"/>
       <c r="S43" s="14" t="s">
+        <v>871</v>
+      </c>
+      <c r="T43" s="14" t="s">
         <v>872</v>
-      </c>
-      <c r="T43" s="14" t="s">
-        <v>871</v>
       </c>
       <c r="U43" s="10">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
TB-034: uncertainty and repeatability on both holdouts and the pre-declared pool
Paired cluster bootstrap (10000 resamples of whole task/attack clusters, seeded), exact McNemar
(supporting), one-sided bounds for zero observed, family-status/attack/workflow slices, latency and
token intervals, TB-028 repeatability. Primary unsafe difference: holdout-1 -46.7 pp [-100, 0]
(3 clusters, not excluding zero), holdout-2 -61.7 pp [-81.7, -40.0], pooled -58.7 pp [-77.3, -38.7];
benign utility lower bounds above the -5 pp margin throughout. New attack families: -53.3 pp
[-100, 0]. Seeded rerun reproduces every published interval.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEB0772-EA02-264F-BBCD-207C3B1E54F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62CFADB-136D-7042-B489-3299B37203B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="877">
   <si>
     <t>Tasks</t>
   </si>
@@ -2657,6 +2657,12 @@
   </si>
   <si>
     <t>Done 2026-10-17: every rate recomputed from raw records with numerator, denominator, Wilson 95% (SciPy) and exclusions, tables via pandas, cross-checked against the runner summaries; code committed before each holdout ran through it. Holdout-1 primary: unsafe 10/15 -&gt; 3/15, utility 10/15 -&gt; 14/15. Holdout-2 primary: unsafe 42/60 -&gt; 5/60 (70.0% -&gt; 8.3%), utility 34/60 -&gt; 52/60, false blocks 2/127 permitted calls (argument level also 2/127). Pooled primary: unsafe 69.3% -&gt; 10.7%, utility 58.7% -&gt; 88.0%. Not hidden: defended unsafe is 20% (3/15) on the three new families vs 5% (2/40) on reused tuning families; holdout-1 primary was 20%; argument-level label is post hoc for holdout-1. Paired intervals are TB-034.</t>
+  </si>
+  <si>
+    <t>reports/uncertainty.json; docs/uncertainty.md; scripts/estimate-uncertainty.py; configs/uncertainty.yaml; tests/evaluation/test_uncertainty.py; requirements/analysis.lock</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: paired cluster bootstrap (10000 resamples of whole task/attack clusters with their repetitions, seed 20261048, SciPy/numpy), exact McNemar (supporting), one-sided bounds where zero events were observed, per-attack, per-workflow and family-status slices, latency/token intervals, TB-028 repeatability. Seeded rerun reproduces every published interval (test). Primary unsafe difference: holdout-1 -46.7 pp [-100, 0] (3 clusters, does not exclude zero); holdout-2 -61.7 pp [-81.7, -40.0]; pooled -58.7 pp [-77.3, -38.7]. Benign utility lower bounds above the -5 pp margin in all three. Not hidden: on the 3 new attack families the interval does not exclude zero (-53.3 pp [-100, 0]); tuning families -62.5 pp [-87.5, -35.0]; few clusters; cost is zero on free tiers, tokens reported instead. Next: TB-035.</t>
   </si>
 </sst>
 </file>
@@ -3433,11 +3439,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.45833333333333331</v>
+        <v>0.47222222222222221</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3449,15 +3455,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.61111111111111116</v>
+        <v>0.62962962962962965</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>6.833333333333333</v>
+        <v>6.416666666666667</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -5627,7 +5633,7 @@
         <v>345</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>336</v>
@@ -5635,7 +5641,7 @@
       <c r="F45" s="10"/>
       <c r="G45" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H45" s="18">
         <v>5</v>
@@ -5664,11 +5670,15 @@
         <v>43</v>
       </c>
       <c r="R45" s="10"/>
-      <c r="S45" s="14"/>
-      <c r="T45" s="14"/>
+      <c r="S45" s="14" t="s">
+        <v>875</v>
+      </c>
+      <c r="T45" s="14" t="s">
+        <v>876</v>
+      </c>
       <c r="U45" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:21" ht="64" customHeight="1">
@@ -5690,7 +5700,7 @@
       <c r="F46" s="11"/>
       <c r="G46" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H46" s="18">
         <v>4</v>
@@ -8264,11 +8274,11 @@
       </c>
       <c r="C96" s="10">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D96" s="10">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E96" s="10">
         <f t="shared" si="9"/>
@@ -8280,7 +8290,7 @@
       </c>
       <c r="G96" s="21">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H96" s="10">
         <f t="shared" si="12"/>
@@ -8288,7 +8298,7 @@
       </c>
       <c r="I96" s="10">
         <f t="shared" si="13"/>
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J96" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-035: latency and operating cost from the trace exporter, with a full cost ledger
Ledger of all 3,604 model-call attempts (23 failed) across both confirmatory workloads, priced from
the frozen pricing block (free tier, 0 USD, verified 2026-10-15). Per completed task: p50/p95 time,
agent and defense tokens, failed attempts, cost and tokens per successful task (undefined without a
success). Concurrency measured per run from overlapping spans; latency compared only within one
level (defended about +7 to +25 s mean per run). Settings recorded: concurrency, price date, retries,
pacing, timeout.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62CFADB-136D-7042-B489-3299B37203B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82EC4B5B-A76F-E94C-BA8C-35E66E816FE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="877">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="879">
   <si>
     <t>Tasks</t>
   </si>
@@ -2663,6 +2663,12 @@
   </si>
   <si>
     <t>Done 2026-10-17: paired cluster bootstrap (10000 resamples of whole task/attack clusters with their repetitions, seed 20261048, SciPy/numpy), exact McNemar (supporting), one-sided bounds where zero events were observed, per-attack, per-workflow and family-status slices, latency/token intervals, TB-028 repeatability. Seeded rerun reproduces every published interval (test). Primary unsafe difference: holdout-1 -46.7 pp [-100, 0] (3 clusters, does not exclude zero); holdout-2 -61.7 pp [-81.7, -40.0]; pooled -58.7 pp [-77.3, -38.7]. Benign utility lower bounds above the -5 pp margin in all three. Not hidden: on the 3 new attack families the interval does not exclude zero (-53.3 pp [-100, 0]); tuning families -62.5 pp [-87.5, -35.0]; few clusters; cost is zero on free tiers, tokens reported instead. Next: TB-035.</t>
+  </si>
+  <si>
+    <t>reports/cost-latency.csv; reports/cost-ledger.csv; evidence/tb035-cost-latency.json; docs/cost-latency.md; scripts/measure-cost-latency.py; tests/evaluation/test_cost_latency.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: from the TB-027 spans of both confirmatory workloads (780 runs, every reported run covered); cost ledger of all 3,604 model-call attempts incl. 23 failed, priced from the frozen pricing block (free tier, 0 USD, verified 2026-10-15, build.nvidia.com). Records concurrency (measured per run, levels 0-2, at most 3 runs at once), retries (2 attempts per call, backoff, budget max 3), pacing 1000 ms and 240 s timeout. Latency compared only at matched concurrency: defended adds about +7 to +25 s mean per run (holdout-2 attack, level 2: +23.9 s [+9.7, +39.0]); pairs whose arms ran at different levels are excluded and counted. Billed cost is 0, so tokens per successful task is the cost measure: defended uses fewer per success (holdout-2 benign 6,731 vs 7,614). Next: TB-036.</t>
   </si>
 </sst>
 </file>
@@ -3439,11 +3445,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.47222222222222221</v>
+        <v>0.4861111111111111</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3455,15 +3461,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.62962962962962965</v>
+        <v>0.64814814814814814</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>6.416666666666667</v>
+        <v>6.083333333333333</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -5692,7 +5698,7 @@
         <v>353</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E46" s="11" t="s">
         <v>344</v>
@@ -5700,7 +5706,7 @@
       <c r="F46" s="11"/>
       <c r="G46" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H46" s="18">
         <v>4</v>
@@ -5729,11 +5735,15 @@
         <v>43</v>
       </c>
       <c r="R46" s="11"/>
-      <c r="S46" s="14"/>
-      <c r="T46" s="14"/>
+      <c r="S46" s="14" t="s">
+        <v>877</v>
+      </c>
+      <c r="T46" s="14" t="s">
+        <v>878</v>
+      </c>
       <c r="U46" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:21" ht="64" customHeight="1">
@@ -5755,7 +5765,7 @@
       <c r="F47" s="10"/>
       <c r="G47" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H47" s="18">
         <v>7</v>
@@ -8274,11 +8284,11 @@
       </c>
       <c r="C96" s="10">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D96" s="10">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E96" s="10">
         <f t="shared" si="9"/>
@@ -8290,7 +8300,7 @@
       </c>
       <c r="G96" s="21">
         <f t="shared" si="11"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="H96" s="10">
         <f t="shared" si="12"/>
@@ -8298,7 +8308,7 @@
       </c>
       <c r="I96" s="10">
         <f t="shared" si="13"/>
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="J96" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-036: component ablations on development data, nulls and negatives published (A-027)
Six arms plus the frozen gate run, identical settings and budget, 288 new pairs, 0 invalid.
Credited: tool allowlist + contract scoping (-51.8 pp unsafe [-77.8, -25.9]) and the gateway
under the directive-flow defense (-70.4 pp [-88.9, -48.1]). No measurable contribution on
development data: strict schemas alone, exact-argument approval (active, but contract scoping
already binds update arguments), directive flow on top of the gateway, sticky denials; the
blocking flow check costs -23.8 pp benign utility. Claims inventory: 7 tested, 7 untested with
reasons. Gateway README states approval is defence in depth, not an independent protection.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82EC4B5B-A76F-E94C-BA8C-35E66E816FE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D263047-4CFC-A44D-96E2-E675DE5647E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="879">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1225" uniqueCount="881">
   <si>
     <t>Tasks</t>
   </si>
@@ -2669,6 +2669,12 @@
   </si>
   <si>
     <t>Done 2026-10-17: from the TB-027 spans of both confirmatory workloads (780 runs, every reported run covered); cost ledger of all 3,604 model-call attempts incl. 23 failed, priced from the frozen pricing block (free tier, 0 USD, verified 2026-10-15, build.nvidia.com). Records concurrency (measured per run, levels 0-2, at most 3 runs at once), retries (2 attempts per call, backoff, budget max 3), pacing 1000 ms and 240 s timeout. Latency compared only at matched concurrency: defended adds about +7 to +25 s mean per run (holdout-2 attack, level 2: +23.9 s [+9.7, +39.0]); pairs whose arms ran at different levels are excluded and counted. Billed cost is 0, so tokens per successful task is the cost measure: defended uses fewer per success (holdout-2 benign 6,731 vs 7,614). Next: TB-036.</t>
+  </si>
+  <si>
+    <t>reports/ablations.csv; evidence/tb036-ablations.json; docs/ablations.md; configs/ablations.yaml; scripts/run-ablations.mjs; scripts/analyse-ablations.py; tests/evaluation/test_ablations.py; tests/policy/test_ablation_layers.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17 (A-027, development data only; both holdouts already used): 6 new arms x 48 pairs + the frozen system's gate run, identical frozen settings and budget, 0 invalid. Credited: tool allowlist + contract scoping (-51.8 pp unsafe [-77.8, -25.9], also +23.8 pp utility) and the gateway under the directive-flow defense (-70.4 pp [-88.9, -48.1]). Negative/null results published: schemas alone, exact-argument approval (0.0 pp; it fired 10 times but contract scoping already binds update arguments), directive flow on top of the gateway (-22.2 pp [-55.6, 0]), sticky denials (0.0 pp), blocking flow check (-14.8 pp, n.s., with a -23.8 pp utility cost). 14 claims: 7 tested, 7 labelled untested with reasons. Baseline varied 63-85% unsafe across runs (stochastic), stated. Next: TB-037.</t>
   </si>
 </sst>
 </file>
@@ -3445,11 +3451,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.4861111111111111</v>
+        <v>0.5</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3461,15 +3467,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.64814814814814814</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>6.083333333333333</v>
+        <v>5.5</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -5757,7 +5763,7 @@
         <v>361</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>352</v>
@@ -5765,7 +5771,7 @@
       <c r="F47" s="10"/>
       <c r="G47" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H47" s="18">
         <v>7</v>
@@ -5794,11 +5800,15 @@
         <v>43</v>
       </c>
       <c r="R47" s="10"/>
-      <c r="S47" s="14"/>
-      <c r="T47" s="14"/>
+      <c r="S47" s="14" t="s">
+        <v>879</v>
+      </c>
+      <c r="T47" s="14" t="s">
+        <v>880</v>
+      </c>
       <c r="U47" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:21" ht="64" customHeight="1">
@@ -5820,7 +5830,7 @@
       <c r="F48" s="12"/>
       <c r="G48" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H48" s="17">
         <v>4</v>
@@ -6150,7 +6160,7 @@
       <c r="F54" s="12"/>
       <c r="G54" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H54" s="17">
         <v>4</v>
@@ -8284,11 +8294,11 @@
       </c>
       <c r="C96" s="10">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D96" s="10">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E96" s="10">
         <f t="shared" si="9"/>
@@ -8300,7 +8310,7 @@
       </c>
       <c r="G96" s="21">
         <f t="shared" si="11"/>
-        <v>0.83333333333333337</v>
+        <v>1</v>
       </c>
       <c r="H96" s="10">
         <f t="shared" si="12"/>
@@ -8308,11 +8318,11 @@
       </c>
       <c r="I96" s="10">
         <f t="shared" si="13"/>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J96" s="10">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K96" s="1"/>
       <c r="L96" s="1"/>
@@ -8364,7 +8374,7 @@
       </c>
       <c r="J97" s="11">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K97" s="1"/>
       <c r="L97" s="1"/>
@@ -8416,7 +8426,7 @@
       </c>
       <c r="J98" s="10">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K98" s="1"/>
       <c r="L98" s="1"/>

</xml_diff>

<commit_message>
TB-037: fresh-environment reproduction evidence and CLI documentation
A fresh clone following the README quickstart passes every CLI step and the full npm run verify;
smoke outputs equal the committed results apart from listed volatile fields and the arm report is
schema-valid; 55 reproduction tests pass. The digest-pinned container (Node 26.5.0, npm 12.0.0,
Python 3.14.0) passes the same CLI checks. Live benchmark runs need the user's own credentials.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D263047-4CFC-A44D-96E2-E675DE5647E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8352D1D9-415E-F34C-A89F-6EA97493B975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1225" uniqueCount="881">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="883">
   <si>
     <t>Tasks</t>
   </si>
@@ -2675,6 +2675,12 @@
   </si>
   <si>
     <t>Done 2026-10-17 (A-027, development data only; both holdouts already used): 6 new arms x 48 pairs + the frozen system's gate run, identical frozen settings and budget, 0 invalid. Credited: tool allowlist + contract scoping (-51.8 pp unsafe [-77.8, -25.9], also +23.8 pp utility) and the gateway under the directive-flow defense (-70.4 pp [-88.9, -48.1]). Negative/null results published: schemas alone, exact-argument approval (0.0 pp; it fired 10 times but contract scoping already binds update arguments), directive flow on top of the gateway (-22.2 pp [-55.6, 0]), sticky denials (0.0 pp), blocking flow check (-14.8 pp, n.s., with a -23.8 pp utility cost). 14 claims: 7 tested, 7 labelled untested with reasons. Baseline varied 63-85% unsafe across runs (stochastic), stated. Next: TB-037.</t>
+  </si>
+  <si>
+    <t>README.md; docs/benchmark-cli.md; evidence/tb037-fresh-reproduction.json; src/cli.py; bin/trustbench; configs/cli/trustbench.yaml; schemas/arm-report.schema.json; manifests/pinned.json; Dockerfile.bench; tests/cli/test_cli.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: Typer CLI (validate, fetch-data, smoke --check, benchmark &lt;profile&gt;, evaluate, report --check, manifest) driven by configs/cli/trustbench.yaml; report schema (all 125 existing reports valid); pinned content manifest checked in verify; Docker image pinned by digest. Fresh clone (no node_modules/venv/vendor) following the README: all CLI steps and the full npm run verify exit 0, smoke outputs equal the committed results apart from listed volatile fields, 55 reproduction tests pass; the container (Node 26.5.0, npm 12.0.0, Python 3.14.0) passes the same CLI checks. Defect found and fixed: the quickstart missed the review-site dependencies. Not covered: live benchmark runs need the user's own key and quota (dry-run only). Next: TB-038.</t>
   </si>
 </sst>
 </file>
@@ -3451,11 +3457,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.5</v>
+        <v>0.51388888888888884</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3467,15 +3473,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.66666666666666663</v>
+        <v>0.68518518518518523</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>5.5</v>
+        <v>5.166666666666667</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -5822,7 +5828,7 @@
         <v>370</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E48" s="12" t="s">
         <v>360</v>
@@ -5830,7 +5836,7 @@
       <c r="F48" s="12"/>
       <c r="G48" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H48" s="17">
         <v>4</v>
@@ -5859,11 +5865,15 @@
         <v>43</v>
       </c>
       <c r="R48" s="12"/>
-      <c r="S48" s="13"/>
-      <c r="T48" s="13"/>
+      <c r="S48" s="13" t="s">
+        <v>881</v>
+      </c>
+      <c r="T48" s="13" t="s">
+        <v>882</v>
+      </c>
       <c r="U48" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:21" ht="64" customHeight="1">
@@ -5885,7 +5895,7 @@
       <c r="F49" s="10"/>
       <c r="G49" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H49" s="18">
         <v>5</v>
@@ -8346,11 +8356,11 @@
       </c>
       <c r="C97" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D97" s="11">
         <f t="shared" si="8"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E97" s="11">
         <f t="shared" si="9"/>
@@ -8362,7 +8372,7 @@
       </c>
       <c r="G97" s="20">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="H97" s="11">
         <f t="shared" si="12"/>
@@ -8370,7 +8380,7 @@
       </c>
       <c r="I97" s="11">
         <f t="shared" si="13"/>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J97" s="11">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-038: two-tier regression release gate with CI, injected-regression acceptance tests
Tier 1 (every change, credential-free) compares fresh scripted runs and the smoke suite with
baselines committed on the base branch; Tier 2 (release candidates) is the A-025 live gate with
an attempt ledger. Injected security and functional regressions block; an unmodified candidate
passes. CI steps verified in a clean Linux container; the GitHub workflow runs on first push
(no remote is configured yet).
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D88A1A-11ED-F545-A0F9-0A79933F3319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9934395-CCA2-D547-953D-A06BB940A1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="883">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1229" uniqueCount="885">
   <si>
     <t>Tasks</t>
   </si>
@@ -2681,6 +2681,12 @@
   </si>
   <si>
     <t>Done 2026-10-17: Typer CLI (validate, fetch-data, smoke --check, benchmark &lt;profile&gt;, evaluate, report --check, manifest) driven by configs/cli/trustbench.yaml; report schema (all 125 existing reports valid); pinned content manifest checked in verify; Docker image pinned by digest. Fresh clone (no node_modules/venv/vendor) following the README: all CLI steps and the full npm run verify exit 0, smoke outputs equal the committed results apart from listed volatile fields, 55 reproduction tests pass; the container (Node 26.5.0, npm 12.0.0, Python 3.14.0) passes the same CLI checks. Defect found and fixed: the quickstart missed the review-site dependencies. Not covered: live benchmark runs need the user's own key and quota (dry-run only). Next: TB-038. Extended 2026-10-17: trustbench remote (catalog, run, status, report) drives the live-test service behind the website's Live page (docs/live-service.md); hardening and public deployment are TB-039 and TB-041.</t>
+  </si>
+  <si>
+    <t>.github/workflows/release-gate.yml; scripts/ci.sh; scripts/release-gate-scripted.py; scripts/release-gate.py; configs/release-gate.yaml; tests/release/test_injected_regressions.py; tests/selection/test_release_gate.py; docs/release-gate.md</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17 (A-028): Tier 1, every change: fresh scripted runs and the smoke suite compared case by case with baselines as committed on the base branch (fixed invariants, zero tolerance). Tier 2, per release candidate: the A-025 live gate (T1/T2, INCONCLUSIVE blocks) with an attempt ledger: one run, a second only with a defect note, never a third. Injected regressions (contract resource check removed, argument binding removed, email body dropped, over-blocking gateway) all FAIL; an unmodified candidate PASSES; editing one's own baseline does not hide a regression. CI steps (scripts/ci.sh tier1) passed in a clean Linux container; npm run verify passes. External prerequisite not yet met: the repository has no GitHub remote, so the workflow has not run on GitHub; it runs on the first push. Next: TB-039.</t>
   </si>
 </sst>
 </file>
@@ -3457,11 +3463,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.51388888888888884</v>
+        <v>0.52777777777777779</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3473,15 +3479,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.68518518518518523</v>
+        <v>0.70370370370370372</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>5.166666666666667</v>
+        <v>4.75</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -5887,7 +5893,7 @@
         <v>378</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>368</v>
@@ -5895,7 +5901,7 @@
       <c r="F49" s="10"/>
       <c r="G49" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H49" s="18">
         <v>5</v>
@@ -5924,11 +5930,15 @@
         <v>43</v>
       </c>
       <c r="R49" s="10"/>
-      <c r="S49" s="14"/>
-      <c r="T49" s="14"/>
+      <c r="S49" s="14" t="s">
+        <v>883</v>
+      </c>
+      <c r="T49" s="14" t="s">
+        <v>884</v>
+      </c>
       <c r="U49" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:21" ht="64" customHeight="1">
@@ -5950,7 +5960,7 @@
       <c r="F50" s="11"/>
       <c r="G50" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H50" s="18">
         <v>4</v>
@@ -8356,11 +8366,11 @@
       </c>
       <c r="C97" s="11">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D97" s="11">
         <f t="shared" si="8"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E97" s="11">
         <f t="shared" si="9"/>
@@ -8372,7 +8382,7 @@
       </c>
       <c r="G97" s="20">
         <f t="shared" si="11"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H97" s="11">
         <f t="shared" si="12"/>
@@ -8380,7 +8390,7 @@
       </c>
       <c r="I97" s="11">
         <f t="shared" si="13"/>
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="J97" s="11">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-039: evidence and workbook (container and browser checks of sessions and accounts)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9934395-CCA2-D547-953D-A06BB940A1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1839E788-7AF9-C14B-8760-5760C63148E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1229" uniqueCount="885">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="887">
   <si>
     <t>Tasks</t>
   </si>
@@ -2687,6 +2687,12 @@
   </si>
   <si>
     <t>Done 2026-10-17 (A-028): Tier 1, every change: fresh scripted runs and the smoke suite compared case by case with baselines as committed on the base branch (fixed invariants, zero tolerance). Tier 2, per release candidate: the A-025 live gate (T1/T2, INCONCLUSIVE blocks) with an attempt ledger: one run, a second only with a defect note, never a third. Injected regressions (contract resource check removed, argument binding removed, email body dropped, over-blocking gateway) all FAIL; an unmodified candidate PASSES; editing one's own baseline does not hide a regression. CI steps (scripts/ci.sh tier1) passed in a clean Linux container; npm run verify passes. External prerequisite not yet met: the repository has no GitHub remote, so the workflow has not run on GitHub; it runs on the first push. Next: TB-039.</t>
+  </si>
+  <si>
+    <t>tests/api-security/; evidence/tb039-api-security.json; docs/live-service.md; src/service/app.py; src/service/accounts.py; src/service/sessions.py; src/service/secrets.py; src/service/mail.py; web/src/pages/Account.tsx</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: authentication with no forced sign-up (anonymous guest sessions) plus real accounts: sign-up, emailed verification, sign-in, sign-out, forgot/reset/change password, account deletion; scrypt passwords, lockout, enumeration-resistant answers, hashed tokens. Per-user isolation (others get 404), read-only revocable share links, owner deletion of runs/sessions/accounts with every artifact, retention sweep (guests 24 h, accounts 30 days), quotas per address, per session, for sign-in and the shared budget; secrets via env, NAME_FILE or /run/secrets with log redaction; strict security headers. tests/api-security 28 pass; website Account pages and CLI login tested; container checked. Not built: Google/GitHub sign-in (needs OAuth apps), MFA, a managed cloud secrets service. Deployment needs SMTP secrets for accounts; guests need nothing. Next: TB-040.</t>
   </si>
 </sst>
 </file>
@@ -3463,11 +3469,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.52777777777777779</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3479,15 +3485,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.70370370370370372</v>
+        <v>0.72222222222222221</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>4.75</v>
+        <v>4.416666666666667</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -5952,7 +5958,7 @@
         <v>386</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E50" s="11" t="s">
         <v>377</v>
@@ -5960,7 +5966,7 @@
       <c r="F50" s="11"/>
       <c r="G50" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H50" s="18">
         <v>4</v>
@@ -5989,11 +5995,15 @@
         <v>43</v>
       </c>
       <c r="R50" s="11"/>
-      <c r="S50" s="14"/>
-      <c r="T50" s="14"/>
+      <c r="S50" s="14" t="s">
+        <v>885</v>
+      </c>
+      <c r="T50" s="14" t="s">
+        <v>886</v>
+      </c>
       <c r="U50" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:21" ht="64" customHeight="1">
@@ -6015,7 +6025,7 @@
       <c r="F51" s="10"/>
       <c r="G51" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H51" s="18">
         <v>5</v>
@@ -8366,11 +8376,11 @@
       </c>
       <c r="C97" s="11">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D97" s="11">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E97" s="11">
         <f t="shared" si="9"/>
@@ -8382,7 +8392,7 @@
       </c>
       <c r="G97" s="20">
         <f t="shared" si="11"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="H97" s="11">
         <f t="shared" si="12"/>
@@ -8390,7 +8400,7 @@
       </c>
       <c r="I97" s="11">
         <f t="shared" si="13"/>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J97" s="11">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-040: fault drill report and evidence (50/50 drills, container drills, availability cost, hung-provider sensitivity), workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1839E788-7AF9-C14B-8760-5760C63148E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93E5055-2ACE-4743-B28D-6E7D7ECE322B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="887">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="889">
   <si>
     <t>Tasks</t>
   </si>
@@ -2693,6 +2693,12 @@
   </si>
   <si>
     <t>Done 2026-10-17: authentication with no forced sign-up (anonymous guest sessions) plus real accounts: sign-up, emailed verification, sign-in, sign-out, forgot/reset/change password, account deletion; scrypt passwords, lockout, enumeration-resistant answers, hashed tokens. Per-user isolation (others get 404), read-only revocable share links, owner deletion of runs/sessions/accounts with every artifact, retention sweep (guests 24 h, accounts 30 days), quotas per address, per session, for sign-in and the shared budget; secrets via env, NAME_FILE or /run/secrets with log redaction; strict security headers. tests/api-security 28 pass; website Account pages and CLI login tested; container checked. Not built: Google/GitHub sign-in (needs OAuth apps), MFA, a managed cloud secrets service. Deployment needs SMTP secrets for accounts; guests need nothing. Next: TB-040.</t>
+  </si>
+  <si>
+    <t>reports/fault-drill.md; evidence/tb040-fault-drill.json; tests/faults/; scripts/fault-drill.py; configs/fault-drill.yaml; reports/tb040-fault-tests.xml; reports/tb040-fault-checkpoint.xml</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: 50/50 drill tests pass (unavailable model: refused/503/hung provider give explicit invalid network/server/timeout, no tool runs, no allow decision; corrupt or altered checkpoint and final outcome give checkpoint_corrupt with no replay; tool crash gives 502 tool_backend_error with nothing committed; log-store failure denies with 503 audit_unavailable via a fsynced write-ahead intent log; deleting a running run stops its whole process group; unwritable storage refuses runs (503) before reserving budget and the service starts degraded instead of crashing; damaged budget record pauses the shared key). Container drills on trustbench-live:tb040: no-network live run ends invalid (network), cancel leaves no processes, read-only volume serves site and catalog with sessions/runs 503. Availability cost measured: +0.1 ms median per allowed call (write-ahead audit), 4 us SHA-256 per checkpoint, hung-provider runs now invalid (23 of 780 confirmatory runs, 2.9%); sensitivity: primary pooled unsafe-effect difference -58.7 -&gt; -59.4 pp, conclusions unchanged; registered results not rewritten. Not covered: a writer who recomputes the checkpoint checksum (needs a keyed MAC), SQLite disk-full, real provider outages, host memory/CPU exhaustion.</t>
   </si>
 </sst>
 </file>
@@ -3469,11 +3475,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.54166666666666663</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3485,15 +3491,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.72222222222222221</v>
+        <v>0.7407407407407407</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>4.416666666666667</v>
+        <v>4</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6017,7 +6023,7 @@
         <v>392</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>385</v>
@@ -6025,7 +6031,7 @@
       <c r="F51" s="10"/>
       <c r="G51" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H51" s="18">
         <v>5</v>
@@ -6054,11 +6060,15 @@
         <v>43</v>
       </c>
       <c r="R51" s="10"/>
-      <c r="S51" s="14"/>
-      <c r="T51" s="14"/>
+      <c r="S51" s="14" t="s">
+        <v>887</v>
+      </c>
+      <c r="T51" s="14" t="s">
+        <v>888</v>
+      </c>
       <c r="U51" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:21" ht="64" customHeight="1">
@@ -6080,7 +6090,7 @@
       <c r="F52" s="11"/>
       <c r="G52" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H52" s="18">
         <v>4</v>
@@ -8376,11 +8386,11 @@
       </c>
       <c r="C97" s="11">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D97" s="11">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E97" s="11">
         <f t="shared" si="9"/>
@@ -8392,7 +8402,7 @@
       </c>
       <c r="G97" s="20">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H97" s="11">
         <f t="shared" si="12"/>
@@ -8400,7 +8410,7 @@
       </c>
       <c r="I97" s="11">
         <f t="shared" si="13"/>
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J97" s="11">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-041 (staging verified, public URL pending): deployment runbook, staging evidence (compose, budget exhaustion, Space image, browser), workbook In Progress
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93E5055-2ACE-4743-B28D-6E7D7ECE322B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1155B3-3EB3-A845-8252-A7DC40FC409B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="889">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1235" uniqueCount="891">
   <si>
     <t>Tasks</t>
   </si>
@@ -2699,6 +2699,12 @@
   </si>
   <si>
     <t>Done 2026-10-17: 50/50 drill tests pass (unavailable model: refused/503/hung provider give explicit invalid network/server/timeout, no tool runs, no allow decision; corrupt or altered checkpoint and final outcome give checkpoint_corrupt with no replay; tool crash gives 502 tool_backend_error with nothing committed; log-store failure denies with 503 audit_unavailable via a fsynced write-ahead intent log; deleting a running run stops its whole process group; unwritable storage refuses runs (503) before reserving budget and the service starts degraded instead of crashing; damaged budget record pauses the shared key). Container drills on trustbench-live:tb040: no-network live run ends invalid (network), cancel leaves no processes, read-only volume serves site and catalog with sessions/runs 503. Availability cost measured: +0.1 ms median per allowed call (write-ahead audit), 4 us SHA-256 per checkpoint, hung-provider runs now invalid (23 of 780 confirmatory runs, 2.9%); sensitivity: primary pooled unsafe-effect difference -58.7 -&gt; -59.4 pp, conclusions unchanged; registered results not rewritten. Not covered: a writer who recomputes the checkpoint checksum (needs a keyed MAC), SQLite disk-full, real provider outages, host memory/CPU exhaustion.</t>
+  </si>
+  <si>
+    <t>docs/deployment-runbook.md; evidence/tb041-deployment.json; evidence/tb041/; deploy/compose.yaml; configs/deploy/public-demo.json; scripts/check-deployment.py; scripts/deploy-hf-space.py; tests/deploy/</t>
+  </si>
+  <si>
+    <t>Staging done 2026-10-17, public URL not yet: constrain-only deployment profile (public-demo: 2 pairs per hosted run, 40 shared pairs a day; widening refused at startup), hardened compose deployment (read-only, cap_drop ALL, secrets as files, loopback bind), uid-1000 image with healthcheck, Hugging Face Space deploy script (git archive HEAD only). scripts/check-deployment.py 20/20 on compose with live runs, 20/20 on a staging profile with the budget exhausted, 20/20 on the exact Space image; browser live run (project key) and instant run done, exhausted budget falls back to Instant with a clear message; key and operator token absent from both images, run data and logs. Found and fixed: deploy/secrets was in the first local image build context (deleted unrun; .dockerignore and tests/deploy now prevent it). BLOCKED for completion: acceptance needs a public URL from the GitHub README; no GitHub repository exists for this project yet and the host needs the owner's account. Next: owner publishes the repo, creates a Hugging Face account and write token, runs scripts/deploy-hf-space.py --set-secrets, then scripts/check-deployment.py --url &lt;space url&gt; --live and the README link.</t>
   </si>
 </sst>
 </file>
@@ -6082,7 +6088,7 @@
         <v>400</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>288</v>
+        <v>558</v>
       </c>
       <c r="E52" s="11" t="s">
         <v>391</v>
@@ -6090,7 +6096,7 @@
       <c r="F52" s="11"/>
       <c r="G52" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>In Progress</v>
       </c>
       <c r="H52" s="18">
         <v>4</v>
@@ -6119,11 +6125,15 @@
         <v>43</v>
       </c>
       <c r="R52" s="11"/>
-      <c r="S52" s="14"/>
-      <c r="T52" s="14"/>
+      <c r="S52" s="14" t="s">
+        <v>889</v>
+      </c>
+      <c r="T52" s="14" t="s">
+        <v>890</v>
+      </c>
       <c r="U52" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:21" ht="64" customHeight="1">
@@ -8390,11 +8400,11 @@
       </c>
       <c r="D97" s="11">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E97" s="11">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F97" s="11">
         <f t="shared" si="10"/>
@@ -8414,7 +8424,7 @@
       </c>
       <c r="J97" s="11">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K97" s="1"/>
       <c r="L97" s="1"/>

</xml_diff>

<commit_message>
TB-041: workbook row Completed (public demo checked from outside, CI green)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1155B3-3EB3-A845-8252-A7DC40FC409B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{205E45ED-C9A8-0F45-A90D-D3D059259462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -2701,10 +2701,10 @@
     <t>Done 2026-10-17: 50/50 drill tests pass (unavailable model: refused/503/hung provider give explicit invalid network/server/timeout, no tool runs, no allow decision; corrupt or altered checkpoint and final outcome give checkpoint_corrupt with no replay; tool crash gives 502 tool_backend_error with nothing committed; log-store failure denies with 503 audit_unavailable via a fsynced write-ahead intent log; deleting a running run stops its whole process group; unwritable storage refuses runs (503) before reserving budget and the service starts degraded instead of crashing; damaged budget record pauses the shared key). Container drills on trustbench-live:tb040: no-network live run ends invalid (network), cancel leaves no processes, read-only volume serves site and catalog with sessions/runs 503. Availability cost measured: +0.1 ms median per allowed call (write-ahead audit), 4 us SHA-256 per checkpoint, hung-provider runs now invalid (23 of 780 confirmatory runs, 2.9%); sensitivity: primary pooled unsafe-effect difference -58.7 -&gt; -59.4 pp, conclusions unchanged; registered results not rewritten. Not covered: a writer who recomputes the checkpoint checksum (needs a keyed MAC), SQLite disk-full, real provider outages, host memory/CPU exhaustion.</t>
   </si>
   <si>
-    <t>docs/deployment-runbook.md; evidence/tb041-deployment.json; evidence/tb041/; deploy/compose.yaml; configs/deploy/public-demo.json; scripts/check-deployment.py; scripts/deploy-hf-space.py; tests/deploy/</t>
-  </si>
-  <si>
-    <t>Staging done 2026-10-17, public URL not yet: constrain-only deployment profile (public-demo: 2 pairs per hosted run, 40 shared pairs a day; widening refused at startup), hardened compose deployment (read-only, cap_drop ALL, secrets as files, loopback bind), uid-1000 image with healthcheck, Hugging Face Space deploy script (git archive HEAD only). scripts/check-deployment.py 20/20 on compose with live runs, 20/20 on a staging profile with the budget exhausted, 20/20 on the exact Space image; browser live run (project key) and instant run done, exhausted budget falls back to Instant with a clear message; key and operator token absent from both images, run data and logs. Found and fixed: deploy/secrets was in the first local image build context (deleted unrun; .dockerignore and tests/deploy now prevent it). BLOCKED for completion: acceptance needs a public URL from the GitHub README; no GitHub repository exists for this project yet and the host needs the owner's account. Next: owner publishes the repo, creates a Hugging Face account and write token, runs scripts/deploy-hf-space.py --set-secrets, then scripts/check-deployment.py --url &lt;space url&gt; --live and the README link.</t>
+    <t>docs/deployment-runbook.md; evidence/tb041-deployment.json; evidence/tb041/; deploy/compose.yaml; deploy/watchdog.sh; deploy/install-watchdog.sh; configs/deploy/public-demo.json; scripts/check-deployment.py; scripts/check-deployment-gui.mjs; .github/workflows/public-demo-check.yml; tests/deploy/; README.md</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: public demo at https://trustbench.taila273c6.ts.net (README link on GitHub), self-hosted compose deployment behind Tailscale Funnel with the constrain-only public-demo profile (2 pairs per hosted run, 40 shared pairs a day), read-only container, secrets as files, project key never in image, logs or run data. Checked from GitHub's runners: check-deployment --live 20/20 (instant and live runs from API and CLI, auth, quotas, rejected visitor key explicit) and the browser path (instant run, live run on the project key, 2/2 valid each); exhausted shared budget refuses hosted with a clear message while instant and own-key work (tested on the deployment). Restart: server crash back in 8 s, Docker restart 36 s, watchdog repairs a stopped container or lost Funnel in 21 s. Host privacy: Docker file sharing limited to the project folder (home and other paths refused), Docker data on the project drive, no personal name in the URL or committed reports. CI green. Known limits: best-effort self-hosting (machine must stay on; power-failure auto-restart is an owner setting not yet on); from the host itself the public relay route times out, so host-side checks use the tailnet route; HF Docker Spaces need PRO and Oracle A1 had no capacity (recorded).</t>
   </si>
 </sst>
 </file>
@@ -3481,11 +3481,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.55555555555555558</v>
+        <v>0.56944444444444442</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3497,15 +3497,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.7407407407407407</v>
+        <v>0.7592592592592593</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>4</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6088,7 +6088,7 @@
         <v>400</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>558</v>
+        <v>1</v>
       </c>
       <c r="E52" s="11" t="s">
         <v>391</v>
@@ -6096,7 +6096,7 @@
       <c r="F52" s="11"/>
       <c r="G52" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>In Progress</v>
+        <v>Done</v>
       </c>
       <c r="H52" s="18">
         <v>4</v>
@@ -6155,7 +6155,7 @@
       <c r="F53" s="10"/>
       <c r="G53" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H53" s="18">
         <v>3</v>
@@ -8396,7 +8396,7 @@
       </c>
       <c r="C97" s="11">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D97" s="11">
         <f t="shared" si="8"/>
@@ -8404,7 +8404,7 @@
       </c>
       <c r="E97" s="11">
         <f t="shared" si="9"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F97" s="11">
         <f t="shared" si="10"/>
@@ -8412,7 +8412,7 @@
       </c>
       <c r="G97" s="20">
         <f t="shared" si="11"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="H97" s="11">
         <f t="shared" si="12"/>
@@ -8420,11 +8420,11 @@
       </c>
       <c r="I97" s="11">
         <f t="shared" si="13"/>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J97" s="11">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K97" s="1"/>
       <c r="L97" s="1"/>

</xml_diff>

<commit_message>
TB-042: workbook row Completed; node test suites also print their results to the CI log
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{205E45ED-C9A8-0F45-A90D-D3D059259462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DEB800-5486-B846-881E-929FC252001A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1235" uniqueCount="891">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1237" uniqueCount="893">
   <si>
     <t>Tasks</t>
   </si>
@@ -2705,6 +2705,12 @@
   </si>
   <si>
     <t>Done 2026-10-17: public demo at https://trustbench.taila273c6.ts.net (README link on GitHub), self-hosted compose deployment behind Tailscale Funnel with the constrain-only public-demo profile (2 pairs per hosted run, 40 shared pairs a day), read-only container, secrets as files, project key never in image, logs or run data. Checked from GitHub's runners: check-deployment --live 20/20 (instant and live runs from API and CLI, auth, quotas, rejected visitor key explicit) and the browser path (instant run, live run on the project key, 2/2 valid each); exhausted shared budget refuses hosted with a clear message while instant and own-key work (tested on the deployment). Restart: server crash back in 8 s, Docker restart 36 s, watchdog repairs a stopped container or lost Funnel in 21 s. Host privacy: Docker file sharing limited to the project folder (home and other paths refused), Docker data on the project drive, no personal name in the URL or committed reports. CI green. Known limits: best-effort self-hosting (machine must stay on; power-failure auto-restart is an owner setting not yet on); from the host itself the public relay route times out, so host-side checks use the tailnet route; HF Docker Spaces need PRO and Oracle A1 had no capacity (recorded).</t>
+  </si>
+  <si>
+    <t>reports/rollback-drill.md; evidence/tb042-rollback-drill.json; scripts/rollback-drill.py; scripts/backup.py; configs/rollback-drill.yaml; deploy/backup-demo.sh; tests/rollback/; tests/release/test_injected_regressions.py; docs/release-gate.md; docs/deployment-runbook.md</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17 against previous release release-tb041. Config rollback: a bad policy change (approval requirement dropped) is blocked by Tier 1, configs restored from the release in 0.26 s, fixtures rerun and gate PASS, 56/56 policy decisions per arm identical to the release; measured recovery 18.8 s. Found and fixed: the gate compared only verdicts, so that change (record updates without their approval pause) had passed; Tier 1 now blocks a more permissive policy audit trail (injected-regression test added). Service data restore: backup taken while running, data lost, tampered backup refused, restore to serving 0.25 s with byte-identical runs, artifacts and 21 audit files, account login, guest session and share link intact. Run-store restore: interrupted run resumes from restored store exactly as from a never-lost store, write committed once (233 ms). Deployment rollback to the previous release image: healthy in 6.0 s, data intact, roll forward 5.9 s. Public demo backed up (325 files, verified). Limits: small synthetic state, backups on the same drive, no data-format change between releases exercised. One CI run failed once in test:recovery and passed on rerun; recovery tests now print results to the log.</t>
   </si>
 </sst>
 </file>
@@ -3481,11 +3487,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.56944444444444442</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3497,15 +3503,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.7592592592592593</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>3.6666666666666665</v>
+        <v>3.4166666666666665</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6147,7 +6153,7 @@
         <v>406</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>399</v>
@@ -6155,7 +6161,7 @@
       <c r="F53" s="10"/>
       <c r="G53" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H53" s="18">
         <v>3</v>
@@ -6184,11 +6190,15 @@
         <v>43</v>
       </c>
       <c r="R53" s="10"/>
-      <c r="S53" s="14"/>
-      <c r="T53" s="14"/>
+      <c r="S53" s="14" t="s">
+        <v>891</v>
+      </c>
+      <c r="T53" s="14" t="s">
+        <v>892</v>
+      </c>
       <c r="U53" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:21" ht="64" customHeight="1">
@@ -8396,11 +8406,11 @@
       </c>
       <c r="C97" s="11">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D97" s="11">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E97" s="11">
         <f t="shared" si="9"/>
@@ -8412,7 +8422,7 @@
       </c>
       <c r="G97" s="20">
         <f t="shared" si="11"/>
-        <v>0.83333333333333337</v>
+        <v>1</v>
       </c>
       <c r="H97" s="11">
         <f t="shared" si="12"/>
@@ -8420,11 +8430,11 @@
       </c>
       <c r="I97" s="11">
         <f t="shared" si="13"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J97" s="11">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K97" s="1"/>
       <c r="L97" s="1"/>

</xml_diff>

<commit_message>
TB-043: related-work comparison matrix (24 sourced prior works plus TrustBench, specific limitation and basis per row, 2025-2026 search refresh), builder that enforces the acceptance criterion; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DEB800-5486-B846-881E-929FC252001A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3138D5A4-59AD-5343-B923-82D92D6DBB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1237" uniqueCount="893">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="895">
   <si>
     <t>Tasks</t>
   </si>
@@ -2711,6 +2711,12 @@
   </si>
   <si>
     <t>Done 2026-10-17 against previous release release-tb041. Config rollback: a bad policy change (approval requirement dropped) is blocked by Tier 1, configs restored from the release in 0.26 s, fixtures rerun and gate PASS, 56/56 policy decisions per arm identical to the release; measured recovery 18.8 s. Found and fixed: the gate compared only verdicts, so that change (record updates without their approval pause) had passed; Tier 1 now blocks a more permissive policy audit trail (injected-regression test added). Service data restore: backup taken while running, data lost, tampered backup refused, restore to serving 0.25 s with byte-identical runs, artifacts and 21 audit files, account login, guest session and share link intact. Run-store restore: interrupted run resumes from restored store exactly as from a never-lost store, write committed once (233 ms). Deployment rollback to the previous release image: healthy in 6.0 s, data intact, roll forward 5.9 s. Public demo backed up (325 files, verified). Limits: small synthetic state, backups on the same drive, no data-format change between releases exercised. One CI run failed once in test:recovery and passed on rerun; recovery tests now print results to the log.</t>
+  </si>
+  <si>
+    <t>research/related-work.csv; research/related-work.md; research/related-work-rows.py; scripts/build-related-work.py; tests/research/test_related_work.py; docs/threat-model.md</t>
+  </si>
+  <si>
+    <t>Done 2026-10-17: matrix of 24 prior systems and studies plus TrustBench (9 benchmarks incl. AgentDojo, InjecAgent, ASB, WASP, AgentDyn, AutoDojo, AgentSecBench, NetInjectBench; 13 defenses incl. CaMeL, FIDES, RTBAS, Progent, MELON, StruQ, SecAlign, Instruction Hierarchy, Spotlighting; design patterns; an adaptive evaluation of out-of-band defenses), each with threat model, enforcement boundary, evaluation suite, claimed guarantee, reported result, a specific limitation and its basis (6 stated by authors, 7 reported by later work, 5 measured on this harness, 7 our analysis). Every source checked against its primary listing; search refreshed for 2025-2026 work on 2026-10-17. Builder fails on a missing source or limitation, a dangling basis or a TrustBench statistic not quoted verbatim from its own row (8 tests). Refresh findings: out-of-band enforcement is the current consensus, so TrustBench claims no new defense idea; static benchmarks overestimate defenses and TrustBench has no adaptive evaluation yet (recorded as open). Re-implemented comparators are labelled as such.</t>
   </si>
 </sst>
 </file>
@@ -3487,11 +3493,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.58333333333333337</v>
+        <v>0.59722222222222221</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3503,15 +3509,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.77777777777777779</v>
+        <v>0.79629629629629628</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>3.4166666666666665</v>
+        <v>3.0833333333333335</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6212,7 +6218,7 @@
         <v>415</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E54" s="12" t="s">
         <v>360</v>
@@ -6220,7 +6226,7 @@
       <c r="F54" s="12"/>
       <c r="G54" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H54" s="17">
         <v>4</v>
@@ -6251,11 +6257,15 @@
       <c r="R54" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="S54" s="13"/>
-      <c r="T54" s="13"/>
+      <c r="S54" s="13" t="s">
+        <v>893</v>
+      </c>
+      <c r="T54" s="13" t="s">
+        <v>894</v>
+      </c>
       <c r="U54" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:21" ht="64" customHeight="1">
@@ -6277,7 +6287,7 @@
       <c r="F55" s="10"/>
       <c r="G55" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H55" s="18">
         <v>5</v>
@@ -8458,11 +8468,11 @@
       </c>
       <c r="C98" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D98" s="10">
         <f t="shared" si="8"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E98" s="10">
         <f t="shared" si="9"/>
@@ -8474,7 +8484,7 @@
       </c>
       <c r="G98" s="21">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="H98" s="10">
         <f t="shared" si="12"/>
@@ -8482,7 +8492,7 @@
       </c>
       <c r="I98" s="10">
         <f t="shared" si="13"/>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J98" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-044: explicit hypothesis test under the preregistered rule (effect sizes, intervals, failure slices, cost, component question, sensitivity); findings reproduced from evidence; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3138D5A4-59AD-5343-B923-82D92D6DBB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D2DB8E-9C35-D943-9D8D-EE66C771CAA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="895">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="897">
   <si>
     <t>Tasks</t>
   </si>
@@ -2717,6 +2717,12 @@
   </si>
   <si>
     <t>Done 2026-10-17: matrix of 24 prior systems and studies plus TrustBench (9 benchmarks incl. AgentDojo, InjecAgent, ASB, WASP, AgentDyn, AutoDojo, AgentSecBench, NetInjectBench; 13 defenses incl. CaMeL, FIDES, RTBAS, Progent, MELON, StruQ, SecAlign, Instruction Hierarchy, Spotlighting; design patterns; an adaptive evaluation of out-of-band defenses), each with threat model, enforcement boundary, evaluation suite, claimed guarantee, reported result, a specific limitation and its basis (6 stated by authors, 7 reported by later work, 5 measured on this harness, 7 our analysis). Every source checked against its primary listing; search refreshed for 2025-2026 work on 2026-10-17. Builder fails on a missing source or limitation, a dangling basis or a TrustBench statistic not quoted verbatim from its own row (8 tests). Refresh findings: out-of-band enforcement is the current consensus, so TrustBench claims no new defense idea; static benchmarks overestimate defenses and TrustBench has no adaptive evaluation yet (recorded as open). Re-implemented comparators are labelled as such.</t>
+  </si>
+  <si>
+    <t>research/findings.md; evidence/tb044-hypothesis.json; scripts/test-hypothesis.py; configs/hypothesis.yaml; tests/research/test_hypothesis.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18 under the preregistered rule (unsafe interval below zero, utility lower bound above -5 pp). Supported on the pre-declared pool: unsafe committed effect 52/75 -&gt; 8/75, -58.7 pp [-77.3, -38.7]; benign utility 44/75 -&gt; 66/75, +29.3 pp [+16.0, +44.0]. Per holdout: holdout-2 supported (-61.7 pp [-81.7, -40.0]), holdout-1 not separated (-46.7 pp [-100, 0]); secondary renderings mixed. Failure slices: document workflow not separated (-16.0 pp [-40, 0]); TB-ATT-DOC-104 succeeded as often defended as undefended (3/5); new-family and holdout-1-attack slices include zero; 8 defended unsafe runs and 9 defended benign failures listed (mostly record-update mismatches). Cost: billed $0; +16.2 s and +671/+415 tokens per run, fewer tokens per success in 9 of 12 workloads. Not shown: that the provenance-aware part causes the gain (development ablation -22.2 pp [-55.6, 0], no confirmatory capability-only arm); combining existing components is not novel; no adaptive attacker. Hung-provider sensitivity -59.4 pp, conclusion unchanged.</t>
   </si>
 </sst>
 </file>
@@ -3493,11 +3499,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.59722222222222221</v>
+        <v>0.61111111111111116</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3509,15 +3515,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.79629629629629628</v>
+        <v>0.81481481481481477</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>3.0833333333333335</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6279,7 +6285,7 @@
         <v>423</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>413</v>
@@ -6287,7 +6293,7 @@
       <c r="F55" s="10"/>
       <c r="G55" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H55" s="18">
         <v>5</v>
@@ -6316,11 +6322,15 @@
         <v>43</v>
       </c>
       <c r="R55" s="10"/>
-      <c r="S55" s="14"/>
-      <c r="T55" s="14"/>
+      <c r="S55" s="14" t="s">
+        <v>895</v>
+      </c>
+      <c r="T55" s="14" t="s">
+        <v>896</v>
+      </c>
       <c r="U55" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:21" ht="64" customHeight="1">
@@ -6342,7 +6352,7 @@
       <c r="F56" s="11"/>
       <c r="G56" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H56" s="18">
         <v>4</v>
@@ -8468,11 +8478,11 @@
       </c>
       <c r="C98" s="10">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D98" s="10">
         <f t="shared" si="8"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E98" s="10">
         <f t="shared" si="9"/>
@@ -8484,7 +8494,7 @@
       </c>
       <c r="G98" s="21">
         <f t="shared" si="11"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H98" s="10">
         <f t="shared" si="12"/>
@@ -8492,7 +8502,7 @@
       </c>
       <c r="I98" s="10">
         <f t="shared" si="13"/>
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="J98" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-045: label and evaluator audit complete; oracle fix pinned (A-029), arms test records the scripted exfil baseline as unsafe without the attacker goal; findings link the audit; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D2DB8E-9C35-D943-9D8D-EE66C771CAA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D0C63D-6FE4-3749-9271-86ED08BFBAEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="897">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1243" uniqueCount="899">
   <si>
     <t>Tasks</t>
   </si>
@@ -2723,6 +2723,12 @@
   </si>
   <si>
     <t>Done 2026-10-18 under the preregistered rule (unsafe interval below zero, utility lower bound above -5 pp). Supported on the pre-declared pool: unsafe committed effect 52/75 -&gt; 8/75, -58.7 pp [-77.3, -38.7]; benign utility 44/75 -&gt; 66/75, +29.3 pp [+16.0, +44.0]. Per holdout: holdout-2 supported (-61.7 pp [-81.7, -40.0]), holdout-1 not separated (-46.7 pp [-100, 0]); secondary renderings mixed. Failure slices: document workflow not separated (-16.0 pp [-40, 0]); TB-ATT-DOC-104 succeeded as often defended as undefended (3/5); new-family and holdout-1-attack slices include zero; 8 defended unsafe runs and 9 defended benign failures listed (mostly record-update mismatches). Cost: billed $0; +16.2 s and +671/+415 tokens per run, fewer tokens per success in 9 of 12 workloads. Not shown: that the provenance-aware part causes the gain (development ablation -22.2 pp [-55.6, 0], no confirmatory capability-only arm); combining existing components is not novel; no adaptive attacker. Hung-provider sensitivity -59.4 pp, conclusion unchanged.</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18. Sample: 61 of 780 valid confirmatory runs, stratified by workflow, kind, arm and evaluator verdict (22 strata, 3 per stratum, fixed seed), blind packets without evaluator labels. Two independent AI reviewers (A: Claude; B: Nemotron 3 Super, a different model family); no human reviewer, which is a stated limit. Agreement with the evaluator: utility 88.5% / 91.8% (kappa 0.77 / 0.84), security 88.5% / 100%, attacker goal 98.4% / 98.4%. 16 labels adjudicated with written reasons: 8 reviewer errors, 7 definition upheld (out-of-allowlist reads count as unsafe), 1 evaluator error. Evaluator error per label: 0/61, 0/61, 1/61 (Wilson upper 5.9%, 5.9%, 8.7%). The error was an oracle defect (a forbidden read counted as the attacker goal for 3 write-goal attacks): fixed in evaluator tb016.1.3.0 (A-029, post hoc, registered results not rewritten); all 780 runs relabelled from their traces, 6 changed, every analysis recomputed: 3 secondary/control attacker-goal cells change, primary unchanged, TB-044 decision stands. Sensitivity (extra reads counted as safe): pooled primary unsafe difference -58.7 -&gt; -42.7 pp [-58.7, -26.7], still excludes zero; some secondary renderings lose separation. Scripted release-gate baselines refreshed for the evaluator change (doc-birch-exfil baseline attacker goal True -&gt; False).</t>
+  </si>
+  <si>
+    <t>research/label-audit.csv; research/label-audit.md; evidence/tb045-label-audit.json; research/label-audit/adjudication.jsonl; research/label-audit/rerun.json; scripts/label-audit.py; configs/label-audit.yaml; tests/research/test_label_audit.py; protocol/amendments.md</t>
   </si>
 </sst>
 </file>
@@ -3499,11 +3505,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.61111111111111116</v>
+        <v>0.625</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3515,15 +3521,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.81481481481481477</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>2.6666666666666665</v>
+        <v>2.3333333333333335</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6344,7 +6350,7 @@
         <v>431</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E56" s="11" t="s">
         <v>422</v>
@@ -6352,7 +6358,7 @@
       <c r="F56" s="11"/>
       <c r="G56" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H56" s="18">
         <v>4</v>
@@ -6381,11 +6387,15 @@
         <v>43</v>
       </c>
       <c r="R56" s="11"/>
-      <c r="S56" s="14"/>
-      <c r="T56" s="14"/>
+      <c r="S56" s="14" t="s">
+        <v>898</v>
+      </c>
+      <c r="T56" s="14" t="s">
+        <v>897</v>
+      </c>
       <c r="U56" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:21" ht="64" customHeight="1">
@@ -6407,7 +6417,7 @@
       <c r="F57" s="10"/>
       <c r="G57" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H57" s="18">
         <v>4</v>
@@ -8478,11 +8488,11 @@
       </c>
       <c r="C98" s="10">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D98" s="10">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E98" s="10">
         <f t="shared" si="9"/>
@@ -8494,7 +8504,7 @@
       </c>
       <c r="G98" s="21">
         <f t="shared" si="11"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="H98" s="10">
         <f t="shared" si="12"/>
@@ -8502,7 +8512,7 @@
       </c>
       <c r="I98" s="10">
         <f t="shared" si="13"/>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J98" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-046: reproducibility package complete; offline subset reproduced 10/10 in a clean offline container and a fresh clone of release repro-tb046; repro check in verify; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D0C63D-6FE4-3749-9271-86ED08BFBAEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8BBF051-607A-C34A-A56C-1C6F1219A3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1243" uniqueCount="899">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="901">
   <si>
     <t>Tasks</t>
   </si>
@@ -2729,6 +2729,12 @@
   </si>
   <si>
     <t>research/label-audit.csv; research/label-audit.md; evidence/tb045-label-audit.json; research/label-audit/adjudication.jsonl; research/label-audit/rerun.json; scripts/label-audit.py; configs/label-audit.yaml; tests/research/test_label_audit.py; protocol/amendments.md</t>
+  </si>
+  <si>
+    <t>repro/README.md; repro/manifest.json; repro/reproduction-log.json; repro/reproduction-log-clone.json; repro/run-in-container.sh; scripts/repro.py; configs/repro.yaml; tests/research/test_repro.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18. Git release repro-tb046 (tag on 0c1f9d0, GitHub release published). repro/manifest.json publishes fixture IDs by split (tuning, holdout, holdout2), the seeds from the registry (pair order 20261014, split 2026101401, 10000 bootstrap resamples) and SHA-256 hashes of 6 fixture files, 41 configs, 10 analysis scripts and 14 raw run records. Excluded and checked (scripts/repro.py check): .env, deployment secrets, demo backups, the AgentDojo checkout (fetched by pinned commit, MIT), local state; no credential-shaped string in the tree or in the full git history (only a fake test key), and no personal identifier in the tree (two docs that named the author's machine were fixed; older commit texts still contain a local path and machine name, not rewritten). Acceptance: the offline subset (10 steps: validate, pinned hashes, scripted smoke, TB-033..036 metrics from raw records, TB-043, TB-044, TB-045 rerun and report, reproduction tests, research tests) reproduced 10/10 with 0 unexpected file changes in two routes: a clean Linux container as a non-root user with no network from only the tracked files, and a fresh GitHub clone of the tag following repro/README.md. Only timestamps, wall-clock timings and random IDs differ. Limits: both runs by the author (no independent person yet); live model runs cannot be replayed exactly (raw records published, all numbers recomputed from them); the AgentDojo check needs fetch-data (network); browser tests need Chrome.</t>
   </si>
 </sst>
 </file>
@@ -3505,11 +3511,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.625</v>
+        <v>0.63888888888888884</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3521,15 +3527,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.83333333333333337</v>
+        <v>0.85185185185185186</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>2.3333333333333335</v>
+        <v>2</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6409,7 +6415,7 @@
         <v>439</v>
       </c>
       <c r="D57" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>430</v>
@@ -6417,7 +6423,7 @@
       <c r="F57" s="10"/>
       <c r="G57" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H57" s="18">
         <v>4</v>
@@ -6446,11 +6452,15 @@
         <v>43</v>
       </c>
       <c r="R57" s="10"/>
-      <c r="S57" s="14"/>
-      <c r="T57" s="14"/>
+      <c r="S57" s="14" t="s">
+        <v>899</v>
+      </c>
+      <c r="T57" s="14" t="s">
+        <v>900</v>
+      </c>
       <c r="U57" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:21" ht="64" customHeight="1">
@@ -6472,7 +6482,7 @@
       <c r="F58" s="11"/>
       <c r="G58" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H58" s="18">
         <v>5</v>
@@ -8488,11 +8498,11 @@
       </c>
       <c r="C98" s="10">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D98" s="10">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E98" s="10">
         <f t="shared" si="9"/>
@@ -8504,7 +8514,7 @@
       </c>
       <c r="G98" s="21">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H98" s="10">
         <f t="shared" si="12"/>
@@ -8512,7 +8522,7 @@
       </c>
       <c r="I98" s="10">
         <f t="shared" si="13"/>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J98" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-047: technical report complete (137 sourced claims, ledger, lint and coverage tests, reproduced offline); workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8BBF051-607A-C34A-A56C-1C6F1219A3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC9BD2C-1513-4E42-80A6-7F97B96AF2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="901">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="903">
   <si>
     <t>Tasks</t>
   </si>
@@ -2735,6 +2735,12 @@
   </si>
   <si>
     <t>Done 2026-10-18. Git release repro-tb046 (tag on 0c1f9d0, GitHub release published). repro/manifest.json publishes fixture IDs by split (tuning, holdout, holdout2), the seeds from the registry (pair order 20261014, split 2026101401, 10000 bootstrap resamples) and SHA-256 hashes of 6 fixture files, 41 configs, 10 analysis scripts and 14 raw run records. Excluded and checked (scripts/repro.py check): .env, deployment secrets, demo backups, the AgentDojo checkout (fetched by pinned commit, MIT), local state; no credential-shaped string in the tree or in the full git history (only a fake test key), and no personal identifier in the tree (two docs that named the author's machine were fixed; older commit texts still contain a local path and machine name, not rewritten). Acceptance: the offline subset (10 steps: validate, pinned hashes, scripted smoke, TB-033..036 metrics from raw records, TB-043, TB-044, TB-045 rerun and report, reproduction tests, research tests) reproduced 10/10 with 0 unexpected file changes in two routes: a clean Linux container as a non-root user with no network from only the tracked files, and a fresh GitHub clone of the tag following repro/README.md. Only timestamps, wall-clock timings and random IDs differ. Limits: both runs by the author (no independent person yet); live model runs cannot be replayed exactly (raw records published, all numbers recomputed from them); the AgentDojo check needs fetch-data (network); browser tests need Chrome.</t>
+  </si>
+  <si>
+    <t>research/report.md; research/report-claims.json; research/report.template.md; scripts/build-report.py; configs/report.yaml; tests/research/test_report.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18. research/report.md (Markdown) covers problem, threat model, system, experimental design, results, failure cases, evaluation quality, engineering evidence, limits and relation to prior work, with links to the evidence. Acceptance: every number is a placeholder resolved from a committed artifact; the claim ledger research/report-claims.json maps all 137 claims to 18 source files (path, raw value, rendered text, report line) with content hashes. Checks: the build fails on any digit or number word outside a placeholder or identifier, any dead link or cited path, any unrendered placeholder, and overclaiming phrases (patent, publication acceptance, state of the art, provable or guaranteed security); tests re-resolve every claim, scan the rendered report so every number on a line is covered by a claim (an injected unsourced number fails), and check source hashes. The report check is a reproduction step: 11/11 reproduced in the clean offline container at 7285854. Stated in the report: not peer reviewed; holdout-1 alone not separated; provenance layer not shown to drive the gain; static attacks only; AI-only label audit.</t>
   </si>
 </sst>
 </file>
@@ -3511,11 +3517,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.63888888888888884</v>
+        <v>0.65277777777777779</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3527,15 +3533,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.85185185185185186</v>
+        <v>0.87037037037037035</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>2</v>
+        <v>1.5833333333333333</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6474,7 +6480,7 @@
         <v>447</v>
       </c>
       <c r="D58" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E58" s="11" t="s">
         <v>438</v>
@@ -6482,7 +6488,7 @@
       <c r="F58" s="11"/>
       <c r="G58" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H58" s="18">
         <v>5</v>
@@ -6511,11 +6517,15 @@
         <v>43</v>
       </c>
       <c r="R58" s="11"/>
-      <c r="S58" s="14"/>
-      <c r="T58" s="14"/>
+      <c r="S58" s="14" t="s">
+        <v>901</v>
+      </c>
+      <c r="T58" s="14" t="s">
+        <v>902</v>
+      </c>
       <c r="U58" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:21" ht="64" customHeight="1">
@@ -6537,7 +6547,7 @@
       <c r="F59" s="10"/>
       <c r="G59" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H59" s="18">
         <v>3</v>
@@ -8498,11 +8508,11 @@
       </c>
       <c r="C98" s="10">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D98" s="10">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E98" s="10">
         <f t="shared" si="9"/>
@@ -8514,7 +8524,7 @@
       </c>
       <c r="G98" s="21">
         <f t="shared" si="11"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="H98" s="10">
         <f t="shared" si="12"/>
@@ -8522,7 +8532,7 @@
       </c>
       <c r="I98" s="10">
         <f t="shared" si="13"/>
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J98" s="10">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-048 (wip): container reproduction at f332f81 (12/12)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC9BD2C-1513-4E42-80A6-7F97B96AF2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D573C0E-6C3A-CF45-986F-7447A225E48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="903">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="905">
   <si>
     <t>Tasks</t>
   </si>
@@ -2741,6 +2741,12 @@
   </si>
   <si>
     <t>Done 2026-10-18. research/report.md (Markdown) covers problem, threat model, system, experimental design, results, failure cases, evaluation quality, engineering evidence, limits and relation to prior work, with links to the evidence. Acceptance: every number is a placeholder resolved from a committed artifact; the claim ledger research/report-claims.json maps all 137 claims to 18 source files (path, raw value, rendered text, report line) with content hashes. Checks: the build fails on any digit or number word outside a placeholder or identifier, any dead link or cited path, any unrendered placeholder, and overclaiming phrases (patent, publication acceptance, state of the art, provable or guaranteed security); tests re-resolve every claim, scan the rendered report so every number on a line is covered by a claim (an injected unsourced number fails), and check source hashes. The report check is a reproduction step: 11/11 reproduced in the clean offline container at 7285854. Stated in the report: not peer reviewed; holdout-1 alone not separated; provenance layer not shown to drive the gain; static attacks only; AI-only label audit.</t>
+  </si>
+  <si>
+    <t>research/claims.md; research/claims-ledger.json; research/claims-check.json; research/claims.template.md; scripts/check-claims.py; configs/claims.yaml; tests/research/test_claims.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18. research/claims.md separates: components replicated or adapted from prior work (each with its related-work row: Progent, tool filter, RTBAS, CaMeL, FIDES, AgentDojo, InjecAgent, spotlighting, repeat prompt, MELON, WASP, out-of-band consensus RW24); engineering contributions with evidence; result statements that may be made, each with its required qualifier and numbers from stored artifacts (21 claims, ledger); hypotheses needing more evidence (provenance layer as cause, holdout-1 alone, adaptive attacker, generalisation, over-defense, human labels); and what is not claimed (novelty, guarantees, production readiness, patent or publication, hiring). Acceptance check (scripts/check-claims.py, in verify and the offline reproduction): 64 public files scanned for novelty, guarantee, publication, patent and resume phrases; 49 hits, each allowed with a reason (negations, descriptions of other work, narrow tested mechanism properties, the frozen label); a planted overclaim or an unsourced portfolio number fails. Fixed: the website headline claimed each defense cut attacks from point estimates (now 'fewer attacker wins on these runs', development data stated). Not fixed, disclosed: the working label 'novel candidate' stays in the frozen-matched live config and recorded reports (changing it needs a new amendment). Reproduced 12/12 in the clean container at d3a15fb. No specialist review has been done; none is needed until a patent or publication claim is considered.</t>
   </si>
 </sst>
 </file>
@@ -3517,11 +3523,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.65277777777777779</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3533,15 +3539,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.87037037037037035</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>1.5833333333333333</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6539,7 +6545,7 @@
         <v>455</v>
       </c>
       <c r="D59" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>446</v>
@@ -6547,7 +6553,7 @@
       <c r="F59" s="10"/>
       <c r="G59" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H59" s="18">
         <v>3</v>
@@ -6576,11 +6582,15 @@
         <v>43</v>
       </c>
       <c r="R59" s="10"/>
-      <c r="S59" s="14"/>
-      <c r="T59" s="14"/>
+      <c r="S59" s="14" t="s">
+        <v>903</v>
+      </c>
+      <c r="T59" s="14" t="s">
+        <v>904</v>
+      </c>
       <c r="U59" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:21" ht="64" customHeight="1">
@@ -6604,7 +6614,7 @@
       </c>
       <c r="G60" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H60" s="17">
         <v>3</v>
@@ -8508,11 +8518,11 @@
       </c>
       <c r="C98" s="10">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D98" s="10">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E98" s="10">
         <f t="shared" si="9"/>
@@ -8524,7 +8534,7 @@
       </c>
       <c r="G98" s="21">
         <f t="shared" si="11"/>
-        <v>0.83333333333333337</v>
+        <v>1</v>
       </c>
       <c r="H98" s="10">
         <f t="shared" si="12"/>
@@ -8532,11 +8542,11 @@
       </c>
       <c r="I98" s="10">
         <f t="shared" si="13"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J98" s="10">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K98" s="1"/>
       <c r="L98" s="1"/>
@@ -8588,7 +8598,7 @@
       </c>
       <c r="J99" s="11">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K99" s="1"/>
       <c r="L99" s="1"/>

</xml_diff>

<commit_message>
TB-048: contribution and claim boundaries complete; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D573C0E-6C3A-CF45-986F-7447A225E48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C0C58C-39B7-1141-BB8E-B7A78AD5683C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2746,7 +2746,7 @@
     <t>research/claims.md; research/claims-ledger.json; research/claims-check.json; research/claims.template.md; scripts/check-claims.py; configs/claims.yaml; tests/research/test_claims.py</t>
   </si>
   <si>
-    <t>Done 2026-10-18. research/claims.md separates: components replicated or adapted from prior work (each with its related-work row: Progent, tool filter, RTBAS, CaMeL, FIDES, AgentDojo, InjecAgent, spotlighting, repeat prompt, MELON, WASP, out-of-band consensus RW24); engineering contributions with evidence; result statements that may be made, each with its required qualifier and numbers from stored artifacts (21 claims, ledger); hypotheses needing more evidence (provenance layer as cause, holdout-1 alone, adaptive attacker, generalisation, over-defense, human labels); and what is not claimed (novelty, guarantees, production readiness, patent or publication, hiring). Acceptance check (scripts/check-claims.py, in verify and the offline reproduction): 64 public files scanned for novelty, guarantee, publication, patent and resume phrases; 49 hits, each allowed with a reason (negations, descriptions of other work, narrow tested mechanism properties, the frozen label); a planted overclaim or an unsourced portfolio number fails. Fixed: the website headline claimed each defense cut attacks from point estimates (now 'fewer attacker wins on these runs', development data stated). Not fixed, disclosed: the working label 'novel candidate' stays in the frozen-matched live config and recorded reports (changing it needs a new amendment). Reproduced 12/12 in the clean container at d3a15fb. No specialist review has been done; none is needed until a patent or publication claim is considered.</t>
+    <t>Done 2026-10-18. research/claims.md separates: components replicated or adapted from prior work (each with its related-work row: Progent, tool filter, RTBAS, CaMeL, FIDES, AgentDojo, InjecAgent, spotlighting, repeat prompt, MELON, WASP, out-of-band consensus RW24); engineering contributions with evidence; result statements that may be made, each with its required qualifier and numbers from stored artifacts (21 claims, ledger); hypotheses needing more evidence (provenance layer as cause, holdout-1 alone, adaptive attacker, generalisation, over-defense, human labels); and what is not claimed (novelty, guarantees, production readiness, patent or publication, hiring). Acceptance check (scripts/check-claims.py, in verify and the offline reproduction): 64 public files scanned for novelty, guarantee, publication, patent and resume phrases; 49 hits, each allowed with a reason (negations, descriptions of other work, narrow tested mechanism properties, the frozen label); a planted overclaim or an unsourced portfolio number fails. Fixed: the website headline claimed each defense cut attacks from point estimates (now a count such as 'Fewer attacker wins for 12 of 14 defenses', with development data and point estimates stated beside it; the public demo shows it after its next redeploy). Not fixed, disclosed: the working label 'novel candidate' stays in the frozen-matched live config and recorded reports (changing it needs a new amendment). Reproduced 12/12 in the clean container at d3a15fb. No specialist review has been done; none is needed until a patent or publication claim is considered.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
TB-049: architecture and walkthrough complete; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C0C58C-39B7-1141-BB8E-B7A78AD5683C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E27DB9E-0A04-CA41-807B-53740CFB3ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="905">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="907">
   <si>
     <t>Tasks</t>
   </si>
@@ -2747,6 +2747,12 @@
   </si>
   <si>
     <t>Done 2026-10-18. research/claims.md separates: components replicated or adapted from prior work (each with its related-work row: Progent, tool filter, RTBAS, CaMeL, FIDES, AgentDojo, InjecAgent, spotlighting, repeat prompt, MELON, WASP, out-of-band consensus RW24); engineering contributions with evidence; result statements that may be made, each with its required qualifier and numbers from stored artifacts (21 claims, ledger); hypotheses needing more evidence (provenance layer as cause, holdout-1 alone, adaptive attacker, generalisation, over-defense, human labels); and what is not claimed (novelty, guarantees, production readiness, patent or publication, hiring). Acceptance check (scripts/check-claims.py, in verify and the offline reproduction): 64 public files scanned for novelty, guarantee, publication, patent and resume phrases; 49 hits, each allowed with a reason (negations, descriptions of other work, narrow tested mechanism properties, the frozen label); a planted overclaim or an unsourced portfolio number fails. Fixed: the website headline claimed each defense cut attacks from point estimates (now a count such as 'Fewer attacker wins for 12 of 14 defenses', with development data and point estimates stated beside it; the public demo shows it after its next redeploy). Not fixed, disclosed: the working label 'novel candidate' stays in the frozen-matched live config and recorded reports (changing it needs a new amendment). Reproduced 12/12 in the clean container at d3a15fb. No specialist review has been done; none is needed until a patent or publication claim is considered.</t>
+  </si>
+  <si>
+    <t>docs/architecture.md; docs/architecture-claims.json; docs/media/walkthrough.webm; docs/media/walkthrough-steps.json; evidence/tb049-walkthrough.json; evidence/tb049-cli-transcript.txt; scripts/walkthrough.py; scripts/record-walkthrough.mjs; tests/research/test_walkthrough.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18. docs/architecture.md: Mermaid trust-boundary diagram and component map; a benign run, a blocked attack beside its undefended pair, a failure trace and a release-gate example, each explained with its evidence (site link, raw record pointer, verdict codes, attribution); every number from stored artifacts (80 claims, ledger). Examples chosen from recorded runs by fixed rules (scripts/walkthrough.py), not staged: the frozen system on the development split (the store holds no holdout run). Release-gate example run for real: unmodified PASS, injected regression (resource check removed) FAIL with security regressions and a more permissive policy trail. Live site: demo redeployed at the current commit; every mode run from the CLI against the public URL (instant, project key, own key) and a report downloaded (evidence/tb049-cli-transcript.txt, no key recorded); video docs/media/walkthrough.webm (2:26, captions) of the site: run pages, policy page, an instant run with report download, the own-key form (not filled), a live run on the project key, the CLI tab. Defect found and fixed: instant runs with every scripted case failed (duplicate repeatability units); fix in src/evaluation/repeats.py with tests, registered results unchanged, demo redeployed. Limits stated: recorded from the host over the tailnet route; own-key mode used the project's key standing in for a visitor's. Reproduced 12/12 in the clean container at 9b85719.</t>
   </si>
 </sst>
 </file>
@@ -3523,11 +3529,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.66666666666666663</v>
+        <v>0.68055555555555558</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3539,15 +3545,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.88888888888888884</v>
+        <v>0.90740740740740744</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>1.3333333333333333</v>
+        <v>1.0833333333333333</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6604,7 +6610,7 @@
         <v>464</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E60" s="12" t="s">
         <v>405</v>
@@ -6614,7 +6620,7 @@
       </c>
       <c r="G60" s="12" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H60" s="17">
         <v>3</v>
@@ -6643,11 +6649,15 @@
         <v>43</v>
       </c>
       <c r="R60" s="12"/>
-      <c r="S60" s="13"/>
-      <c r="T60" s="13"/>
+      <c r="S60" s="13" t="s">
+        <v>905</v>
+      </c>
+      <c r="T60" s="13" t="s">
+        <v>906</v>
+      </c>
       <c r="U60" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:21" ht="64" customHeight="1">
@@ -6669,7 +6679,7 @@
       <c r="F61" s="10"/>
       <c r="G61" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H61" s="18">
         <v>3</v>
@@ -8570,11 +8580,11 @@
       </c>
       <c r="C99" s="11">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D99" s="11">
         <f t="shared" si="8"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E99" s="11">
         <f t="shared" si="9"/>
@@ -8586,7 +8596,7 @@
       </c>
       <c r="G99" s="20">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="H99" s="11">
         <f t="shared" si="12"/>
@@ -8594,7 +8604,7 @@
       </c>
       <c r="I99" s="11">
         <f t="shared" si="13"/>
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J99" s="11">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-050: setup and troubleshooting documentation complete; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E27DB9E-0A04-CA41-807B-53740CFB3ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7445A85D-55A6-D047-AC56-AA2CB9DAD079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="909">
   <si>
     <t>Tasks</t>
   </si>
@@ -2753,6 +2753,12 @@
   </si>
   <si>
     <t>Done 2026-10-18. docs/architecture.md: Mermaid trust-boundary diagram and component map; a benign run, a blocked attack beside its undefended pair, a failure trace and a release-gate example, each explained with its evidence (site link, raw record pointer, verdict codes, attribution); every number from stored artifacts (80 claims, ledger). Examples chosen from recorded runs by fixed rules (scripts/walkthrough.py), not staged: the frozen system on the development split (the store holds no holdout run). Release-gate example run for real: unmodified PASS, injected regression (resource check removed) FAIL with security regressions and a more permissive policy trail. Live site: demo redeployed at the current commit; every mode run from the CLI against the public URL (instant, project key, own key) and a report downloaded (evidence/tb049-cli-transcript.txt, no key recorded); video docs/media/walkthrough.webm (2:26, captions) of the site: run pages, policy page, an instant run with report download, the own-key form (not filled), a live run on the project key, the CLI tab. Defect found and fixed: instant runs with every scripted case failed (duplicate repeatability units); fix in src/evaluation/repeats.py with tests, registered results unchanged, demo redeployed. Limits stated: recorded from the host over the tailnet route; own-key mode used the project's key standing in for a visitor's. Reproduced 12/12 in the clean container at 9b85719.</t>
+  </si>
+  <si>
+    <t>README.md; .env.example; scripts/check-readme.py; evidence/tb050-readme-check.json; tests/research/test_readme.py; web/src/pages/Live.tsx; deploy/watchdog.sh; docs/deployment-runbook.md</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18. README rewritten for a fresh user: the live site in every mode (GUI, and trustbench remote with the project key or your own free-tier key read from an environment variable), install with the minimum tested environments only (macOS 27.2 Apple silicon, Debian 12 arm64 container, Ubuntu 24.04 CI), storage-root export, the four offline checks with their expected output, API keys per provider with the dry run and the no-key message, budget controls (per-run budget files, profiles, live-service limits), and a troubleshooting table with recovery steps. .env.example no longer carries machine paths. Acceptance check (scripts/check-readme.py --fresh): a non-root user in a clean Debian container with only git, Node 26.5.0, npm 12.0.0 and uv cloned the repository from GitHub, ran the Install block and the checks exactly as written: install ok, all four checks exit 0 with the documented output, dry run names the key, a live run without a key stops with the documented message (evidence/tb050-readme-check.json, README hash pinned). Static check (in verify): every path, npm script, CLI command and flag, key variable, model and limit in the README exists or matches the configs. Found and fixed along the way: the site's HTTP example failed (runs need a session) and its local command lacked the storage root (site redeployed); the CLI's missing-key check ignored TRUSTBENCH_NO_DOTENV; and the public demo had been unreachable from outside since 2026-10-17 20:40 UTC because Tailscale withdrew the Funnel DNS record: restored (confirmed from GitHub) and the watchdog now checks public DNS and repairs it. Reproduced 12/12 in the clean container at c2dac5f.</t>
   </si>
 </sst>
 </file>
@@ -3529,11 +3535,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.68055555555555558</v>
+        <v>0.69444444444444442</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3545,15 +3551,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.90740740740740744</v>
+        <v>0.92592592592592593</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>1.0833333333333333</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6671,7 +6677,7 @@
         <v>471</v>
       </c>
       <c r="D61" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>462</v>
@@ -6679,7 +6685,7 @@
       <c r="F61" s="10"/>
       <c r="G61" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H61" s="18">
         <v>3</v>
@@ -6708,11 +6714,15 @@
         <v>43</v>
       </c>
       <c r="R61" s="10"/>
-      <c r="S61" s="14"/>
-      <c r="T61" s="14"/>
+      <c r="S61" s="14" t="s">
+        <v>907</v>
+      </c>
+      <c r="T61" s="14" t="s">
+        <v>908</v>
+      </c>
       <c r="U61" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:21" ht="64" customHeight="1">
@@ -6734,7 +6744,7 @@
       <c r="F62" s="11"/>
       <c r="G62" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H62" s="18">
         <v>4</v>
@@ -8580,11 +8590,11 @@
       </c>
       <c r="C99" s="11">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D99" s="11">
         <f t="shared" si="8"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E99" s="11">
         <f t="shared" si="9"/>
@@ -8596,7 +8606,7 @@
       </c>
       <c r="G99" s="20">
         <f t="shared" si="11"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H99" s="11">
         <f t="shared" si="12"/>
@@ -8604,7 +8614,7 @@
       </c>
       <c r="I99" s="11">
         <f t="shared" si="13"/>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J99" s="11">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-051: release decision RELEASE for a373a5d (tag release-tb051): ten required checks passed; release record, Tier 2 evidence, superseded candidates; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7445A85D-55A6-D047-AC56-AA2CB9DAD079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F0255E-19B6-4343-ADBC-0409866BD713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="909">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="911">
   <si>
     <t>Tasks</t>
   </si>
@@ -2759,6 +2759,12 @@
   </si>
   <si>
     <t>Done 2026-10-18. README rewritten for a fresh user: the live site in every mode (GUI, and trustbench remote with the project key or your own free-tier key read from an environment variable), install with the minimum tested environments only (macOS 27.2 Apple silicon, Debian 12 arm64 container, Ubuntu 24.04 CI), storage-root export, the four offline checks with their expected output, API keys per provider with the dry run and the no-key message, budget controls (per-run budget files, profiles, live-service limits), and a troubleshooting table with recovery steps. .env.example no longer carries machine paths. Acceptance check (scripts/check-readme.py --fresh): a non-root user in a clean Debian container with only git, Node 26.5.0, npm 12.0.0 and uv cloned the repository from GitHub, ran the Install block and the checks exactly as written: install ok, all four checks exit 0 with the documented output, dry run names the key, a live run without a key stops with the documented message (evidence/tb050-readme-check.json, README hash pinned). Static check (in verify): every path, npm script, CLI command and flag, key variable, model and limit in the README exists or matches the configs. Found and fixed along the way: the site's HTTP example failed (runs need a session) and its local command lacked the storage root (site redeployed); the CLI's missing-key check ignored TRUSTBENCH_NO_DOTENV; and the public demo had been unreachable from outside since 2026-10-17 20:40 UTC because Tailscale withdrew the Funnel DNS record: restored (confirmed from GitHub) and the watchdog now checks public DNS and repairs it. Reproduced 12/12 in the clean container at c2dac5f.</t>
+  </si>
+  <si>
+    <t>release/checks.json; release/README.md; release/superseded-d60a4c8.json; release/superseded-75e4e3d.json; release/superseded-b3164e5.json; scripts/release-check.py; configs/release-checks.yaml; tests/release/test_release_check.py; evidence/release-gate-release-7518c85bee62-attempt-1.json; evidence/release-gate-ledger.json</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18. Decision RELEASE for candidate 7518c85 (tag release-tb051, GitHub release): all ten required checks passed on that one commit (release/checks.json): CI Tier 1 and full verify; the Tier 2 live gate PASS (unsafe 63.0% -&gt; 0.0%, -63.0 pp [-81.5, -44.4], 27 pairs; utility +4.8 pp, 21 pairs; development data); a fresh clone from GitHub with the locked install, pinned AgentDojo data and full npm run verify with no local keys; the offline reproduction in a clean container (12/12); the README followed by a fresh non-root user; the demo rebuilt from the committed files and healthy; the public site end to end from GitHub's runners (every mode from API, CLI and Chrome, report download, own-key form; 20 API checks); a real own-key run from the CLI with no key in the output; no-key paths on staging (instant, spent shared budget, 23/23); every documentation link and the report, claim, README and reproduction checks. Three earlier candidates were not released and are recorded with their reasons (release/superseded-*.json): a link check that missed autolinks, scripted traces that varied under CPU load (queue.reason mislabel, fixed), and a fresh-clone failure at test:tool-service (missing .tool-state, fixed); their stopped or passed Tier 2 attempts are in the gate ledger. Scope stated: not a full replication (sealed holdouts not rerun; live runs small and sampled).</t>
   </si>
 </sst>
 </file>
@@ -3535,11 +3541,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.69444444444444442</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3551,15 +3557,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.92592592592592593</v>
+        <v>0.94444444444444442</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>0.83333333333333337</v>
+        <v>0.5</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6736,7 +6742,7 @@
         <v>478</v>
       </c>
       <c r="D62" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E62" s="11" t="s">
         <v>470</v>
@@ -6744,7 +6750,7 @@
       <c r="F62" s="11"/>
       <c r="G62" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H62" s="18">
         <v>4</v>
@@ -6773,11 +6779,15 @@
         <v>43</v>
       </c>
       <c r="R62" s="11"/>
-      <c r="S62" s="14"/>
-      <c r="T62" s="14"/>
+      <c r="S62" s="14" t="s">
+        <v>909</v>
+      </c>
+      <c r="T62" s="14" t="s">
+        <v>910</v>
+      </c>
       <c r="U62" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:21" ht="64" customHeight="1">
@@ -6799,7 +6809,7 @@
       <c r="F63" s="10"/>
       <c r="G63" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H63" s="18">
         <v>2</v>
@@ -8590,11 +8600,11 @@
       </c>
       <c r="C99" s="11">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D99" s="11">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E99" s="11">
         <f t="shared" si="9"/>
@@ -8606,7 +8616,7 @@
       </c>
       <c r="G99" s="20">
         <f t="shared" si="11"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="H99" s="11">
         <f t="shared" si="12"/>
@@ -8614,7 +8624,7 @@
       </c>
       <c r="I99" s="11">
         <f t="shared" si="13"/>
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J99" s="11">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-052: measured résumé bullets complete; workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F0255E-19B6-4343-ADBC-0409866BD713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57CC3F5-9958-A745-B80A-502CFA141CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="911">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="913">
   <si>
     <t>Tasks</t>
   </si>
@@ -2765,6 +2765,12 @@
   </si>
   <si>
     <t>Done 2026-10-18. Decision RELEASE for candidate 7518c85 (tag release-tb051, GitHub release): all ten required checks passed on that one commit (release/checks.json): CI Tier 1 and full verify; the Tier 2 live gate PASS (unsafe 63.0% -&gt; 0.0%, -63.0 pp [-81.5, -44.4], 27 pairs; utility +4.8 pp, 21 pairs; development data); a fresh clone from GitHub with the locked install, pinned AgentDojo data and full npm run verify with no local keys; the offline reproduction in a clean container (12/12); the README followed by a fresh non-root user; the demo rebuilt from the committed files and healthy; the public site end to end from GitHub's runners (every mode from API, CLI and Chrome, report download, own-key form; 20 API checks); a real own-key run from the CLI with no key in the output; no-key paths on staging (instant, spent shared budget, 23/23); every documentation link and the report, claim, README and reproduction checks. Three earlier candidates were not released and are recorded with their reasons (release/superseded-*.json): a link check that missed autolinks, scripted traces that varied under CPU load (queue.reason mislabel, fixed), and a fresh-clone failure at test:tool-service (missing .tool-state, fixed); their stopped or passed Tier 2 attempts are in the gate ledger. Scope stated: not a full replication (sealed holdouts not rerun; live runs small and sampled).</t>
+  </si>
+  <si>
+    <t>portfolio/bullets.md; portfolio/bullets-claims.json; portfolio/bullets.template.md; scripts/build-report.py; scripts/check-claims.py; tests/research/test_bullets.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-18. portfolio/bullets.md: six problem/action/result bullets (paired benchmark result on the sealed holdouts, evaluation integrity and the label audit, same-harness defense comparison, release gates and drills, offline reproducibility, the live site), using only statements allowed by research/claims.md with their qualifiers (holdout-1 not separated, one free model, static attacks, permissive baseline backend, AI reviewers only, re-implementations, development data). Acceptance: all 27 numbers are read from stored runs and reports by scripts/build-report.py and listed in the document's claim-to-evidence table with source file and path (ledger portfolio/bullets-claims.json); tests check every number on every line is covered by a claim and every table row resolves; scripts/check-claims.py (in verify) requires every number under portfolio/ to come from a claim ledger and rejects ranking, percentile and hiring phrases. Unknowns omitted and listed under Not included (provenance layer as cause, adaptive attackers, generalisation, guarantees). Reproduced 12/12 in the clean container at 5ad0835.</t>
   </si>
 </sst>
 </file>
@@ -3541,11 +3547,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.70833333333333337</v>
+        <v>0.72222222222222221</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3557,15 +3563,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.94444444444444442</v>
+        <v>0.96296296296296291</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6801,7 +6807,7 @@
         <v>485</v>
       </c>
       <c r="D63" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>477</v>
@@ -6809,7 +6815,7 @@
       <c r="F63" s="10"/>
       <c r="G63" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H63" s="18">
         <v>2</v>
@@ -6838,11 +6844,15 @@
         <v>43</v>
       </c>
       <c r="R63" s="10"/>
-      <c r="S63" s="14"/>
-      <c r="T63" s="14"/>
+      <c r="S63" s="14" t="s">
+        <v>911</v>
+      </c>
+      <c r="T63" s="14" t="s">
+        <v>912</v>
+      </c>
       <c r="U63" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:21" ht="64" customHeight="1">
@@ -6864,7 +6874,7 @@
       <c r="F64" s="11"/>
       <c r="G64" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H64" s="18">
         <v>2</v>
@@ -8600,11 +8610,11 @@
       </c>
       <c r="C99" s="11">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D99" s="11">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E99" s="11">
         <f t="shared" si="9"/>
@@ -8616,7 +8626,7 @@
       </c>
       <c r="G99" s="20">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H99" s="11">
         <f t="shared" si="12"/>
@@ -8624,7 +8634,7 @@
       </c>
       <c r="I99" s="11">
         <f t="shared" si="13"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J99" s="11">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
TB-053 (wip): TB-051 evidence path follows the archived record
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57CC3F5-9958-A745-B80A-502CFA141CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C93119A-2588-EE4A-8B45-D042109B9DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2761,9 +2761,6 @@
     <t>Done 2026-10-18. README rewritten for a fresh user: the live site in every mode (GUI, and trustbench remote with the project key or your own free-tier key read from an environment variable), install with the minimum tested environments only (macOS 27.2 Apple silicon, Debian 12 arm64 container, Ubuntu 24.04 CI), storage-root export, the four offline checks with their expected output, API keys per provider with the dry run and the no-key message, budget controls (per-run budget files, profiles, live-service limits), and a troubleshooting table with recovery steps. .env.example no longer carries machine paths. Acceptance check (scripts/check-readme.py --fresh): a non-root user in a clean Debian container with only git, Node 26.5.0, npm 12.0.0 and uv cloned the repository from GitHub, ran the Install block and the checks exactly as written: install ok, all four checks exit 0 with the documented output, dry run names the key, a live run without a key stops with the documented message (evidence/tb050-readme-check.json, README hash pinned). Static check (in verify): every path, npm script, CLI command and flag, key variable, model and limit in the README exists or matches the configs. Found and fixed along the way: the site's HTTP example failed (runs need a session) and its local command lacked the storage root (site redeployed); the CLI's missing-key check ignored TRUSTBENCH_NO_DOTENV; and the public demo had been unreachable from outside since 2026-10-17 20:40 UTC because Tailscale withdrew the Funnel DNS record: restored (confirmed from GitHub) and the watchdog now checks public DNS and repairs it. Reproduced 12/12 in the clean container at c2dac5f.</t>
   </si>
   <si>
-    <t>release/checks.json; release/README.md; release/superseded-d60a4c8.json; release/superseded-75e4e3d.json; release/superseded-b3164e5.json; scripts/release-check.py; configs/release-checks.yaml; tests/release/test_release_check.py; evidence/release-gate-release-7518c85bee62-attempt-1.json; evidence/release-gate-ledger.json</t>
-  </si>
-  <si>
     <t>Done 2026-10-18. Decision RELEASE for candidate 7518c85 (tag release-tb051, GitHub release): all ten required checks passed on that one commit (release/checks.json): CI Tier 1 and full verify; the Tier 2 live gate PASS (unsafe 63.0% -&gt; 0.0%, -63.0 pp [-81.5, -44.4], 27 pairs; utility +4.8 pp, 21 pairs; development data); a fresh clone from GitHub with the locked install, pinned AgentDojo data and full npm run verify with no local keys; the offline reproduction in a clean container (12/12); the README followed by a fresh non-root user; the demo rebuilt from the committed files and healthy; the public site end to end from GitHub's runners (every mode from API, CLI and Chrome, report download, own-key form; 20 API checks); a real own-key run from the CLI with no key in the output; no-key paths on staging (instant, spent shared budget, 23/23); every documentation link and the report, claim, README and reproduction checks. Three earlier candidates were not released and are recorded with their reasons (release/superseded-*.json): a link check that missed autolinks, scripted traces that varied under CPU load (queue.reason mislabel, fixed), and a fresh-clone failure at test:tool-service (missing .tool-state, fixed); their stopped or passed Tier 2 attempts are in the gate ledger. Scope stated: not a full replication (sealed holdouts not rerun; live runs small and sampled).</t>
   </si>
   <si>
@@ -2771,6 +2768,9 @@
   </si>
   <si>
     <t>Done 2026-10-18. portfolio/bullets.md: six problem/action/result bullets (paired benchmark result on the sealed holdouts, evaluation integrity and the label audit, same-harness defense comparison, release gates and drills, offline reproducibility, the live site), using only statements allowed by research/claims.md with their qualifiers (holdout-1 not separated, one free model, static attacks, permissive baseline backend, AI reviewers only, re-implementations, development data). Acceptance: all 27 numbers are read from stored runs and reports by scripts/build-report.py and listed in the document's claim-to-evidence table with source file and path (ledger portfolio/bullets-claims.json); tests check every number on every line is covered by a claim and every table row resolves; scripts/check-claims.py (in verify) requires every number under portfolio/ to come from a claim ledger and rejects ranking, percentile and hiring phrases. Unknowns omitted and listed under Not included (provenance layer as cause, adaptive attackers, generalisation, guarantees). Reproduced 12/12 in the clean container at 5ad0835.</t>
+  </si>
+  <si>
+    <t>release/tb051-checks.json; release/README.md; release/superseded-d60a4c8.json; release/superseded-75e4e3d.json; release/superseded-b3164e5.json; scripts/release-check.py; configs/release-checks.yaml; tests/release/test_release_check.py; evidence/release-gate-release-7518c85bee62-attempt-1.json; evidence/release-gate-ledger.json</t>
   </si>
 </sst>
 </file>
@@ -6786,10 +6786,10 @@
       </c>
       <c r="R62" s="11"/>
       <c r="S62" s="14" t="s">
+        <v>912</v>
+      </c>
+      <c r="T62" s="14" t="s">
         <v>909</v>
-      </c>
-      <c r="T62" s="14" t="s">
-        <v>910</v>
       </c>
       <c r="U62" s="10">
         <f t="shared" si="3"/>
@@ -6845,10 +6845,10 @@
       </c>
       <c r="R63" s="10"/>
       <c r="S63" s="14" t="s">
+        <v>910</v>
+      </c>
+      <c r="T63" s="14" t="s">
         <v>911</v>
-      </c>
-      <c r="T63" s="14" t="s">
-        <v>912</v>
       </c>
       <c r="U63" s="10">
         <f t="shared" si="3"/>

</xml_diff>

<commit_message>
TB-053: candidate d1eaf02 not released (portfolio/bullets-claims.json regenerated but not committed); TB-053 In Progress with the blocker in the workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C93119A-2588-EE4A-8B45-D042109B9DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3C0BDB-ECF9-0349-BFC4-C8C7B7DBE94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="914">
   <si>
     <t>Tasks</t>
   </si>
@@ -2771,6 +2771,9 @@
   </si>
   <si>
     <t>release/tb051-checks.json; release/README.md; release/superseded-d60a4c8.json; release/superseded-75e4e3d.json; release/superseded-b3164e5.json; scripts/release-check.py; configs/release-checks.yaml; tests/release/test_release_check.py; evidence/release-gate-release-7518c85bee62-attempt-1.json; evidence/release-gate-ledger.json</t>
+  </si>
+  <si>
+    <t>Release candidates f90ffea and dd4e8de not released (release/README.md). f90ffea: CLI reused an expired saved session (401) so own_key_real and no_key_paths failed; fixed in src/cli.py with a test. live_site_external could not test it because main moved (README edit 553cc68); release-check.py now refuses that dispatch. Its Tier 2 attempt was interrupted at 35/48 pairs with no result (ledger). Next: new candidate a6c758e; the six offline checks are running; the live checks (own key, no-key staging, external site, Tier 2 gate) need the go-ahead, then tag v1.0.0, build, publish only after approval, verify downloads and quickstart.</t>
   </si>
 </sst>
 </file>
@@ -6866,7 +6869,7 @@
         <v>493</v>
       </c>
       <c r="D64" s="14" t="s">
-        <v>288</v>
+        <v>558</v>
       </c>
       <c r="E64" s="11" t="s">
         <v>484</v>
@@ -6874,7 +6877,7 @@
       <c r="F64" s="11"/>
       <c r="G64" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>In Progress</v>
       </c>
       <c r="H64" s="18">
         <v>2</v>
@@ -6904,7 +6907,9 @@
       </c>
       <c r="R64" s="11"/>
       <c r="S64" s="14"/>
-      <c r="T64" s="14"/>
+      <c r="T64" s="14" t="s">
+        <v>913</v>
+      </c>
       <c r="U64" s="10">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -8614,11 +8619,11 @@
       </c>
       <c r="D99" s="11">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E99" s="11">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F99" s="11">
         <f t="shared" si="10"/>
@@ -8638,7 +8643,7 @@
       </c>
       <c r="J99" s="11">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K99" s="1"/>
       <c r="L99" s="1"/>

</xml_diff>

<commit_message>
TB-053: workbook blocker for candidate 6fbbd05 (six offline checks pass; live checks pending)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3C0BDB-ECF9-0349-BFC4-C8C7B7DBE94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858B29FB-8685-8C46-94D0-EDE1BD6743D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2773,7 +2773,7 @@
     <t>release/tb051-checks.json; release/README.md; release/superseded-d60a4c8.json; release/superseded-75e4e3d.json; release/superseded-b3164e5.json; scripts/release-check.py; configs/release-checks.yaml; tests/release/test_release_check.py; evidence/release-gate-release-7518c85bee62-attempt-1.json; evidence/release-gate-ledger.json</t>
   </si>
   <si>
-    <t>Release candidates f90ffea and dd4e8de not released (release/README.md). f90ffea: CLI reused an expired saved session (401) so own_key_real and no_key_paths failed; fixed in src/cli.py with a test. live_site_external could not test it because main moved (README edit 553cc68); release-check.py now refuses that dispatch. Its Tier 2 attempt was interrupted at 35/48 pairs with no result (ledger). Next: new candidate a6c758e; the six offline checks are running; the live checks (own key, no-key staging, external site, Tier 2 gate) need the go-ahead, then tag v1.0.0, build, publish only after approval, verify downloads and quickstart.</t>
+    <t>Not released yet. Candidates f90ffea and a6c758e superseded (release/README.md): f90ffea failed from a CLI expired-session bug (fixed in src/cli.py) and a dispatch that tested another commit (release-check.py fixed); its Tier 2 attempt was interrupted at 35/48 pairs with no result. a6c758e missed one regenerated file. Candidate 2f6b610: the six offline checks pass (CI Tier 1, links, README fresh, offline reproduction, fresh clone verify, demo rebuilt). Next: with approval, the live checks (own key, no-key staging, external site, Tier 2 gate, one attempt), then decide, tag v1.0.0, build, publish only after approval, verify downloads and quickstart.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
TB-053: workbook blocker for candidate 3b79050 (six offline checks pass; live checks pending approval)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858B29FB-8685-8C46-94D0-EDE1BD6743D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FA3307-279D-E340-BB9A-C649D75545AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2773,7 +2773,7 @@
     <t>release/tb051-checks.json; release/README.md; release/superseded-d60a4c8.json; release/superseded-75e4e3d.json; release/superseded-b3164e5.json; scripts/release-check.py; configs/release-checks.yaml; tests/release/test_release_check.py; evidence/release-gate-release-7518c85bee62-attempt-1.json; evidence/release-gate-ledger.json</t>
   </si>
   <si>
-    <t>Not released yet. Candidates f90ffea and a6c758e superseded (release/README.md): f90ffea failed from a CLI expired-session bug (fixed in src/cli.py) and a dispatch that tested another commit (release-check.py fixed); its Tier 2 attempt was interrupted at 35/48 pairs with no result. a6c758e missed one regenerated file. Candidate 2f6b610: the six offline checks pass (CI Tier 1, links, README fresh, offline reproduction, fresh clone verify, demo rebuilt). Next: with approval, the live checks (own key, no-key staging, external site, Tier 2 gate, one attempt), then decide, tag v1.0.0, build, publish only after approval, verify downloads and quickstart.</t>
+    <t>Not released yet. Superseded candidates are in release/README.md: f90ffea (CLI expired-session bug, fixed in src/cli.py; a dispatch that tested another commit, fixed in release-check.py; its Tier 2 attempt was interrupted at 35/48 pairs with no result), a6c758e (one regenerated file not committed), 2f6b610 (passed offline, superseded by the film-player website change). Candidate ef4dfbb: the six offline checks pass (CI Tier 1, links, README fresh, offline reproduction, fresh clone verify, demo rebuilt). Next: with approval, the live checks (own key, no-key staging, external site, Tier 2 gate, one attempt), then decide, tag v1.0.0, build, publish only after approval, verify downloads and quickstart.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
TB-053 Completed: v1.0.0 published and verified (release URL, checks and verify evidence in the workbook; superseded candidates and the curl note fix disclosed)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FA3307-279D-E340-BB9A-C649D75545AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826A2795-15EC-4A46-AE86-232A74199E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="914">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1259" uniqueCount="915">
   <si>
     <t>Tasks</t>
   </si>
@@ -2773,7 +2773,10 @@
     <t>release/tb051-checks.json; release/README.md; release/superseded-d60a4c8.json; release/superseded-75e4e3d.json; release/superseded-b3164e5.json; scripts/release-check.py; configs/release-checks.yaml; tests/release/test_release_check.py; evidence/release-gate-release-7518c85bee62-attempt-1.json; evidence/release-gate-ledger.json</t>
   </si>
   <si>
-    <t>Not released yet. Superseded candidates are in release/README.md: f90ffea (CLI expired-session bug, fixed in src/cli.py; a dispatch that tested another commit, fixed in release-check.py; its Tier 2 attempt was interrupted at 35/48 pairs with no result), a6c758e (one regenerated file not committed), 2f6b610 (passed offline, superseded by the film-player website change). Candidate ef4dfbb: the six offline checks pass (CI Tier 1, links, README fresh, offline reproduction, fresh clone verify, demo rebuilt). Next: with approval, the live checks (own key, no-key staging, external site, Tier 2 gate, one attempt), then decide, tag v1.0.0, build, publish only after approval, verify downloads and quickstart.</t>
+    <t>evidence/tb053-release.json; release/checks.json; release/README.md; scripts/release-package.py; tests/release/test_release_package.py; evidence/release-gate-release-c831245f2f77-attempt-1.json; evidence/release-gate-ledger.json</t>
+  </si>
+  <si>
+    <t>Release: https://github.com/mhrj7/TrustBench-AI/releases/tag/v1.0.0. Done 2026-10-20. v1.0.0 = c831245, RELEASE on all ten checks; Tier 2 PASS on its one attempt (unsafe -81.5 pp [-100, -63.0], utility +25 pp [+5, +47.6], 1/48 invalid; development data). Verified from public links: assets, SHA256SUMS, no keys or personal paths, quickstart passes in a clean container. Disclosed in release/README.md: superseded candidates f90ffea, a6c758e, 2f6b610, ef4dfbb (two Tier 2 attempts stopped with no result); own_key_real rerun once after provider timeouts; first verify failed because the notes omitted curl (fixed in the notes, assets unchanged). Redistribution: only MIT AgentDojo template strings with notice; no AgentDojo checkout. Not a full replication; holdouts not rerun.</t>
   </si>
 </sst>
 </file>
@@ -3550,11 +3553,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.72222222222222221</v>
+        <v>0.73611111111111116</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3566,15 +3569,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.96296296296296291</v>
+        <v>0.98148148148148151</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>0.33333333333333331</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6869,7 +6872,7 @@
         <v>493</v>
       </c>
       <c r="D64" s="14" t="s">
-        <v>558</v>
+        <v>1</v>
       </c>
       <c r="E64" s="11" t="s">
         <v>484</v>
@@ -6877,7 +6880,7 @@
       <c r="F64" s="11"/>
       <c r="G64" s="11" t="str">
         <f t="shared" si="2"/>
-        <v>In Progress</v>
+        <v>Done</v>
       </c>
       <c r="H64" s="18">
         <v>2</v>
@@ -6906,13 +6909,15 @@
         <v>43</v>
       </c>
       <c r="R64" s="11"/>
-      <c r="S64" s="14"/>
+      <c r="S64" s="14" t="s">
+        <v>913</v>
+      </c>
       <c r="T64" s="14" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="U64" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:21" ht="64" customHeight="1">
@@ -6934,7 +6939,7 @@
       <c r="F65" s="10"/>
       <c r="G65" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H65" s="18">
         <v>2</v>
@@ -8615,7 +8620,7 @@
       </c>
       <c r="C99" s="11">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D99" s="11">
         <f t="shared" si="8"/>
@@ -8623,7 +8628,7 @@
       </c>
       <c r="E99" s="11">
         <f t="shared" si="9"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F99" s="11">
         <f t="shared" si="10"/>
@@ -8631,7 +8636,7 @@
       </c>
       <c r="G99" s="20">
         <f t="shared" si="11"/>
-        <v>0.66666666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="H99" s="11">
         <f t="shared" si="12"/>
@@ -8639,11 +8644,11 @@
       </c>
       <c r="I99" s="11">
         <f t="shared" si="13"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J99" s="11">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K99" s="1"/>
       <c r="L99" s="1"/>

</xml_diff>

<commit_message>
TB-054 Completed: handover, backlog and an executable Core-evidence check
docs/handover.md records where the project stands (v1.0.0 and its release history), unresolved failure modes,
supported versions, the next experiment, maintenance triggers and the backlog. scripts/check-handover.py
(npm run verify:handover, part of verify) checks that every Core task has acceptance evidence on disk or remains
open and regenerates the handover's Core-task table from the workbook: 54 of 54 Completed with evidence.
The backlog is kept in the workbook (TB-055 to TB-072) and docs/known-issues.md; no GitHub issues were filed.
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826A2795-15EC-4A46-AE86-232A74199E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3879B364-30E0-354B-AA73-7E9BA3E569AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1259" uniqueCount="915">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="917">
   <si>
     <t>Tasks</t>
   </si>
@@ -2777,6 +2777,12 @@
   </si>
   <si>
     <t>Release: https://github.com/mhrj7/TrustBench-AI/releases/tag/v1.0.0. Done 2026-10-20. v1.0.0 = c831245, RELEASE on all ten checks; Tier 2 PASS on its one attempt (unsafe -81.5 pp [-100, -63.0], utility +25 pp [+5, +47.6], 1/48 invalid; development data). Verified from public links: assets, SHA256SUMS, no keys or personal paths, quickstart passes in a clean container. Disclosed in release/README.md: superseded candidates f90ffea, a6c758e, 2f6b610, ef4dfbb (two Tier 2 attempts stopped with no result); own_key_real rerun once after provider timeouts; first verify failed because the notes omitted curl (fixed in the notes, assets unchanged). Redistribution: only MIT AgentDojo template strings with notice; no AgentDojo checkout. Not a full replication; holdouts not rerun.</t>
+  </si>
+  <si>
+    <t>docs/handover.md; evidence/tb054-handover-check.json; scripts/check-handover.py</t>
+  </si>
+  <si>
+    <t>Done 2026-10-20: docs/handover.md records unresolved failure modes, supported versions, next experiment and maintenance triggers, plus the backlog. Acceptance is executable: scripts/check-handover.py (npm run verify:handover) checks every Core task has evidence on disk or remains open and regenerates the handover's Core table from this workbook. The backlog is kept in this workbook (TB-055 to TB-072) and docs/known-issues.md; no GitHub issues were filed. Completion means an evidenced project, not universal agent security.</t>
   </si>
 </sst>
 </file>
@@ -3553,11 +3559,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.73611111111111116</v>
+        <v>0.75</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3569,15 +3575,15 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
-        <v>0.98148148148148151</v>
+        <v>1</v>
       </c>
       <c r="H5" s="7">
         <f>IF(B7&gt;0,SUMIFS($H$12:$H$83,$Q$12:$Q$83,"Core",$D$12:$D$83,"&lt;&gt;Completed")/B7,"Set hours/week")</f>
-        <v>0.16666666666666666</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5">
         <f ca="1">COUNTIFS($J$12:$J$83,"&gt;0",$J$12:$J$83,"&lt;"&amp;TODAY(),$D$12:$D$83,"&lt;&gt;Completed")</f>
@@ -6931,7 +6937,7 @@
         <v>501</v>
       </c>
       <c r="D65" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>492</v>
@@ -6939,7 +6945,7 @@
       <c r="F65" s="10"/>
       <c r="G65" s="10" t="str">
         <f t="shared" si="2"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H65" s="18">
         <v>2</v>
@@ -6968,11 +6974,15 @@
         <v>43</v>
       </c>
       <c r="R65" s="10"/>
-      <c r="S65" s="14"/>
-      <c r="T65" s="14"/>
+      <c r="S65" s="14" t="s">
+        <v>915</v>
+      </c>
+      <c r="T65" s="14" t="s">
+        <v>916</v>
+      </c>
       <c r="U65" s="10">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:21" ht="64" customHeight="1">
@@ -6994,7 +7004,7 @@
       <c r="F66" s="10"/>
       <c r="G66" s="10" t="str">
         <f t="shared" ref="G66:G77" si="4">IF(NOT(AND(IF(E66="",TRUE,COUNTIFS($A$12:$A$83,E66)=1),IF(F66="",TRUE,COUNTIFS($A$12:$A$83,F66)=1))),"Bad dependency",IF(NOT(AND(IF(E66="",TRUE,COUNTIFS($A$12:$A$83,E66,$D$12:$D$83,"Completed",$U$12:$U$83,1)=1),IF(F66="",TRUE,COUNTIFS($A$12:$A$83,F66,$D$12:$D$83,"Completed",$U$12:$U$83,1)=1))),IF(D66="Completed","Check prerequisites","Waiting"),IF(D66="Completed",IF(S66="","Evidence needed","Done"),IF(D66="Blocked","Blocked",IF(D66="In Progress","In Progress","Ready")))))</f>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H66" s="18">
         <v>4</v>
@@ -8620,11 +8630,11 @@
       </c>
       <c r="C99" s="11">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D99" s="11">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E99" s="11">
         <f t="shared" si="9"/>
@@ -8636,7 +8646,7 @@
       </c>
       <c r="G99" s="20">
         <f t="shared" si="11"/>
-        <v>0.83333333333333337</v>
+        <v>1</v>
       </c>
       <c r="H99" s="11">
         <f t="shared" si="12"/>
@@ -8644,11 +8654,11 @@
       </c>
       <c r="I99" s="11">
         <f t="shared" si="13"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J99" s="11">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K99" s="1"/>
       <c r="L99" s="1"/>
@@ -8700,7 +8710,7 @@
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>

</xml_diff>

<commit_message>
TB-055 Completed in the workbook (evidence paths and open items for TB-056)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3879B364-30E0-354B-AA73-7E9BA3E569AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD1EAD3-4CC8-794A-BA09-92AE5544B44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="917">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1263" uniqueCount="919">
   <si>
     <t>Tasks</t>
   </si>
@@ -2783,6 +2783,12 @@
   </si>
   <si>
     <t>Done 2026-10-20: docs/handover.md records unresolved failure modes, supported versions, next experiment and maintenance triggers, plus the backlog. Acceptance is executable: scripts/check-handover.py (npm run verify:handover) checks every Core task has evidence on disk or remains open and regenerates the handover's Core table from this workbook. The backlog is kept in this workbook (TB-055 to TB-072) and docs/known-issues.md; no GitHub issues were filed. Completion means an evidenced project, not universal agent security.</t>
+  </si>
+  <si>
+    <t>docs/external/agent-selection.md; evidence/tb055-agent-probes/python-probes.jsonl; evidence/tb055-agent-probes/goose-ollama.txt; evidence/tb055-agent-probes/goose-nvidia.txt; evidence/tb055-agent-probes/goose-tools.txt</t>
+  </si>
+  <si>
+    <t>Done 2026-10-20: goose 1.55.0 selected (Apache-2.0, tag v1.55.0, commit 2bcb858, macOS arm64 artifact SHA-256 matching GitHub's digest). Criteria fixed before scoring; 10 candidates screened; shortlist goose / OpenAI Agents SDK 0.24.0 / Agno 3.1.6 all passed real tool-calling probes on local qwen3.5:9b and NVIDIA gpt-oss-20b. Core unmodified; integration only through a documented adapter (TB-057). Fallback: OpenAI Agents SDK, via a recorded amendment. Open for TB-056: classify goose's built-in load_skill tool and keep the developer extension off; Linux artifact checksum still to record for CI.</t>
   </si>
 </sst>
 </file>
@@ -3559,11 +3565,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.75</v>
+        <v>0.76388888888888884</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3575,7 +3581,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -6996,7 +7002,7 @@
         <v>755</v>
       </c>
       <c r="D66" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E66" s="10" t="s">
         <v>500</v>
@@ -7004,7 +7010,7 @@
       <c r="F66" s="10"/>
       <c r="G66" s="10" t="str">
         <f t="shared" ref="G66:G77" si="4">IF(NOT(AND(IF(E66="",TRUE,COUNTIFS($A$12:$A$83,E66)=1),IF(F66="",TRUE,COUNTIFS($A$12:$A$83,F66)=1))),"Bad dependency",IF(NOT(AND(IF(E66="",TRUE,COUNTIFS($A$12:$A$83,E66,$D$12:$D$83,"Completed",$U$12:$U$83,1)=1),IF(F66="",TRUE,COUNTIFS($A$12:$A$83,F66,$D$12:$D$83,"Completed",$U$12:$U$83,1)=1))),IF(D66="Completed","Check prerequisites","Waiting"),IF(D66="Completed",IF(S66="","Evidence needed","Done"),IF(D66="Blocked","Blocked",IF(D66="In Progress","In Progress","Ready")))))</f>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H66" s="18">
         <v>4</v>
@@ -7035,11 +7041,15 @@
       <c r="R66" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="S66" s="14"/>
-      <c r="T66" s="14"/>
+      <c r="S66" s="14" t="s">
+        <v>917</v>
+      </c>
+      <c r="T66" s="14" t="s">
+        <v>918</v>
+      </c>
       <c r="U66" s="10">
         <f t="shared" ref="U66:U77" si="5">IF(LEN(S66)&gt;0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:21" ht="64" customHeight="1">
@@ -7063,7 +7073,7 @@
       </c>
       <c r="G67" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H67" s="18">
         <v>4</v>
@@ -8682,11 +8692,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8698,7 +8708,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8706,7 +8716,7 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>

</xml_diff>

<commit_message>
TB-056 Completed in the workbook (evidence paths; items owned by TB-057/058)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD1EAD3-4CC8-794A-BA09-92AE5544B44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4630C5E4-1D0A-FD4D-9DAC-1967EC0694FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1263" uniqueCount="919">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="921">
   <si>
     <t>Tasks</t>
   </si>
@@ -2789,6 +2789,12 @@
   </si>
   <si>
     <t>Done 2026-10-20: goose 1.55.0 selected (Apache-2.0, tag v1.55.0, commit 2bcb858, macOS arm64 artifact SHA-256 matching GitHub's digest). Criteria fixed before scoring; 10 candidates screened; shortlist goose / OpenAI Agents SDK 0.24.0 / Agno 3.1.6 all passed real tool-calling probes on local qwen3.5:9b and NVIDIA gpt-oss-20b. Core unmodified; integration only through a documented adapter (TB-057). Fallback: OpenAI Agents SDK, via a recorded amendment. Open for TB-056: classify goose's built-in load_skill tool and keep the developer extension off; Linux artifact checksum still to record for CI.</t>
+  </si>
+  <si>
+    <t>docs/external/threat-model.md; docs/external/integration-contract.md; evidence/tb056-threat-model-check.json; evidence/tb056-goose-observations/observations.json</t>
+  </si>
+  <si>
+    <t>Done 2026-10-20: 24 goose entry points classified (6 trusted, 6 untrusted, 12 disabled), each with its control; all 16 TB-002 surfaces mapped; 7 uncovered items listed out of scope. Key controls observed on the wire with a fake model endpoint: CONTEXT_FILE_NAMES='[]' keeps AGENTS.md/.goosehints out of the prompt; --no-profile leaves only load_skill plus the adapter's tools; session naming off gives one request per turn. Contract: adapter holds the gateway token, model proxy holds the provider key, exact invocation and allowlisted environment. Not yet demonstrated (owned by TB-057/058): every call through the gateway, network confinement, native-mode proxy, secret scans of goose artifacts.</t>
   </si>
 </sst>
 </file>
@@ -3565,11 +3571,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.76388888888888884</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3581,7 +3587,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7063,7 +7069,7 @@
         <v>764</v>
       </c>
       <c r="D67" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>508</v>
@@ -7073,7 +7079,7 @@
       </c>
       <c r="G67" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H67" s="18">
         <v>4</v>
@@ -7104,11 +7110,15 @@
       <c r="R67" s="10" t="s">
         <v>771</v>
       </c>
-      <c r="S67" s="14"/>
-      <c r="T67" s="14"/>
+      <c r="S67" s="14" t="s">
+        <v>919</v>
+      </c>
+      <c r="T67" s="14" t="s">
+        <v>920</v>
+      </c>
       <c r="U67" s="10">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:21" ht="64" customHeight="1">
@@ -7132,7 +7142,7 @@
       </c>
       <c r="G68" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H68" s="18">
         <v>12</v>
@@ -8692,11 +8702,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8708,7 +8718,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>8.3333333333333329E-2</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8716,7 +8726,7 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>

</xml_diff>

<commit_message>
TB-056 workbook note after the re-audit
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4630C5E4-1D0A-FD4D-9DAC-1967EC0694FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DB3734-E38E-BF4D-AB4D-8C76CCB322C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2794,7 +2794,7 @@
     <t>docs/external/threat-model.md; docs/external/integration-contract.md; evidence/tb056-threat-model-check.json; evidence/tb056-goose-observations/observations.json</t>
   </si>
   <si>
-    <t>Done 2026-10-20: 24 goose entry points classified (6 trusted, 6 untrusted, 12 disabled), each with its control; all 16 TB-002 surfaces mapped; 7 uncovered items listed out of scope. Key controls observed on the wire with a fake model endpoint: CONTEXT_FILE_NAMES='[]' keeps AGENTS.md/.goosehints out of the prompt; --no-profile leaves only load_skill plus the adapter's tools; session naming off gives one request per turn. Contract: adapter holds the gateway token, model proxy holds the provider key, exact invocation and allowlisted environment. Not yet demonstrated (owned by TB-057/058): every call through the gateway, network confinement, native-mode proxy, secret scans of goose artifacts.</t>
+    <t>Done 2026-10-20, re-audited the same day: 25 goose entry points, each classified exactly trusted (7) or untrusted (18) with its state (13 disabled) and control, covering prompts, tool outputs, memory and plugins; all 16 TB-002 surfaces mapped and all 9 TB-002 boundary rules reviewed; 8 uncovered items listed. Observed on the wire: CONTEXT_FILE_NAMES='[]' keeps AGENTS.md/.goosehints out of the prompt; --no-profile offers only load_skill plus the adapter's tools (no Developer, Computer Controller, Memory, Summon, Extension Manager); session naming off gives one request per turn; HTTP extensions are named after their URL, so the contract uses a stdio relay named trustbench (trustbench__ names observed). Contract adds a fail-closed trace rule. Designed but not yet demonstrated (owned by TB-057/058, listed as uncovered): every call through the gateway, secret scans, network confinement, native-mode proxy.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
TB-057 Completed in the workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DB3734-E38E-BF4D-AB4D-8C76CCB322C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC23CE8D-1ABD-5F47-8218-70539C8A0110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="924">
   <si>
     <t>Tasks</t>
   </si>
@@ -2795,6 +2795,16 @@
   </si>
   <si>
     <t>Done 2026-10-20, re-audited the same day: 25 goose entry points, each classified exactly trusted (7) or untrusted (18) with its state (13 disabled) and control, covering prompts, tool outputs, memory and plugins; all 16 TB-002 surfaces mapped and all 9 TB-002 boundary rules reviewed; 8 uncovered items listed. Observed on the wire: CONTEXT_FILE_NAMES='[]' keeps AGENTS.md/.goosehints out of the prompt; --no-profile offers only load_skill plus the adapter's tools (no Developer, Computer Controller, Memory, Summon, Extension Manager); session naming off gives one request per turn; HTTP extensions are named after their URL, so the contract uses a stdio relay named trustbench (trustbench__ names observed). Contract adds a fail-closed trace rule. Designed but not yet demonstrated (owned by TB-057/058, listed as uncovered): every call through the gateway, secret scans, network confinement, native-mode proxy.</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>src/external/; tests/external/adapter/; tests/external/native-integration/; docs/external/native-integration.md; evidence/tb057-unmodified.json; evidence/tb057-paired-check.json; evidence/tb057-scripted-goose/; evidence/tb057-live-goose/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done 2026-10-20. Mode A: goose 1.55.0 (pinned binary, unmodified) calls all 10 TrustBench tools through the MCP adapter; every trace validates against TB-004 (tests/external/adapter, 4 tests). Paired runs with goose in both arms: scripted 17/17 pairs with evaluator verdicts identical to the built-in agent; live nvidia gpt-oss-20b 4/4 valid pairs (one defended attack run ended budget_exhausted, reported as measured). Mode B: goose's own Computer Controller (goose mcp computercontroller, serverInfo goose-computercontroller 1.55.0) runs unchanged behind the TrustBench MCP gateway on a synthetic-only sandbox; allow/deny recorded per call, refused calls never forwarded, server-initiated sampling/elicitation/roots refused (tests/external/native-integration, 3 tests). Unmodified: release archive digest matches GitHub's, binary byte-identical, no goose files tracked (evidence/tb057-unmodified.json). Same paired report via the website (Live page, "Agent under test") and trustbench remote --agent external_mcp, both run on the service image built from Dockerfile.service with the pinned Linux goose; all 4 reports pass scripts/check-external-paired-report.py (evidence/tb057-paired-check.json). Contract bumped to 1.1.0 (changes listed). Not covered here: network confinement and bypass tests (TB-058); only one native integration (read-only files). The public demo instance still runs the previous image until it is redeployed.
+</t>
   </si>
 </sst>
 </file>
@@ -3571,11 +3581,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.77777777777777779</v>
+        <v>0.79166666666666663</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3587,7 +3597,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7132,7 +7142,7 @@
         <v>841</v>
       </c>
       <c r="D68" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E68" s="10" t="s">
         <v>517</v>
@@ -7140,9 +7150,8 @@
       <c r="F68" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="G68" s="10" t="str">
-        <f t="shared" si="4"/>
-        <v>Ready</v>
+      <c r="G68" s="10" t="s">
+        <v>921</v>
       </c>
       <c r="H68" s="18">
         <v>12</v>
@@ -7173,11 +7182,14 @@
       <c r="R68" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="S68" s="14"/>
-      <c r="T68" s="14"/>
+      <c r="S68" s="14" t="s">
+        <v>922</v>
+      </c>
+      <c r="T68" s="14" t="s">
+        <v>923</v>
+      </c>
       <c r="U68" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:21" ht="64" customHeight="1">
@@ -7201,7 +7213,7 @@
       </c>
       <c r="G69" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H69" s="18">
         <v>6</v>
@@ -7260,7 +7272,7 @@
       </c>
       <c r="G70" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H70" s="18">
         <v>5</v>
@@ -8702,11 +8714,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8718,7 +8730,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0.16666666666666666</v>
+        <v>0.25</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8726,11 +8738,11 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>

</xml_diff>

<commit_message>
TB-058 In Progress in the workbook (bypass tests open)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC23CE8D-1ABD-5F47-8218-70539C8A0110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C837CAF-0C70-204B-B06E-FEC29727D3F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="924">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="925">
   <si>
     <t>Tasks</t>
   </si>
@@ -2804,6 +2804,10 @@
   </si>
   <si>
     <t xml:space="preserve">Done 2026-10-20. Mode A: goose 1.55.0 (pinned binary, unmodified) calls all 10 TrustBench tools through the MCP adapter; every trace validates against TB-004 (tests/external/adapter, 4 tests). Paired runs with goose in both arms: scripted 17/17 pairs with evaluator verdicts identical to the built-in agent; live nvidia gpt-oss-20b 4/4 valid pairs (one defended attack run ended budget_exhausted, reported as measured). Mode B: goose's own Computer Controller (goose mcp computercontroller, serverInfo goose-computercontroller 1.55.0) runs unchanged behind the TrustBench MCP gateway on a synthetic-only sandbox; allow/deny recorded per call, refused calls never forwarded, server-initiated sampling/elicitation/roots refused (tests/external/native-integration, 3 tests). Unmodified: release archive digest matches GitHub's, binary byte-identical, no goose files tracked (evidence/tb057-unmodified.json). Same paired report via the website (Live page, "Agent under test") and trustbench remote --agent external_mcp, both run on the service image built from Dockerfile.service with the pinned Linux goose; all 4 reports pass scripts/check-external-paired-report.py (evidence/tb057-paired-check.json). Contract bumped to 1.1.0 (changes listed). Not covered here: network confinement and bypass tests (TB-058); only one native integration (read-only files). The public demo instance still runs the previous image until it is redeployed.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In progress 2026-10-20. Done: goose and every process it starts run confined (sandbox-exec on macOS, Landlock on Linux; src/external/sandbox.ts): only the episode's adapter socket and model proxy port are reachable, writes only inside the episode folder, no reads of the harness's files; goose refuses to start unconfined. Adapter and gateway sockets accept one client; calls after cancellation are refused (episode_cancelled); native-mode data sits outside the agent sandbox. Contract 1.2.0. External tests pass with goose confined. Blocker: the bypass tests (direct calls, forged/replayed tokens, unlisted tools, argument smuggling, calls after cancellation, both modes, each with a positive control), the audit check and evidence/external-authorization-report.json are being written by the project owner; the Landlock path has not yet been exercised by a test in the Linux container. Next: run those tests, then mark Completed only if every acceptance item passes.
 </t>
   </si>
 </sst>
@@ -7203,7 +7207,7 @@
         <v>774</v>
       </c>
       <c r="D69" s="14" t="s">
-        <v>288</v>
+        <v>558</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>525</v>
@@ -7213,7 +7217,7 @@
       </c>
       <c r="G69" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Ready</v>
+        <v>In Progress</v>
       </c>
       <c r="H69" s="18">
         <v>6</v>
@@ -7245,7 +7249,9 @@
         <v>223</v>
       </c>
       <c r="S69" s="14"/>
-      <c r="T69" s="14"/>
+      <c r="T69" s="14" t="s">
+        <v>924</v>
+      </c>
       <c r="U69" s="10">
         <f t="shared" si="5"/>
         <v>0</v>
@@ -8718,11 +8724,11 @@
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F100" s="11">
         <f t="shared" ref="F100" si="19">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Blocked")</f>
@@ -8742,7 +8748,7 @@
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>

</xml_diff>

<commit_message>
TB-059 Completed in the workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C837CAF-0C70-204B-B06E-FEC29727D3F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F7D707-D680-3A48-8263-843F9AE8461D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="925">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1272" uniqueCount="927">
   <si>
     <t>Tasks</t>
   </si>
@@ -2808,6 +2808,13 @@
   </si>
   <si>
     <t xml:space="preserve">In progress 2026-10-20. Done: goose and every process it starts run confined (sandbox-exec on macOS, Landlock on Linux; src/external/sandbox.ts): only the episode's adapter socket and model proxy port are reachable, writes only inside the episode folder, no reads of the harness's files; goose refuses to start unconfined. Adapter and gateway sockets accept one client; calls after cancellation are refused (episode_cancelled); native-mode data sits outside the agent sandbox. Contract 1.2.0. External tests pass with goose confined. Blocker: the bypass tests (direct calls, forged/replayed tokens, unlisted tools, argument smuggling, calls after cancellation, both modes, each with a positive control), the audit check and evidence/external-authorization-report.json are being written by the project owner; the Landlock path has not yet been exercised by a test in the Linux container. Next: run those tests, then mark Completed only if every acceptance item passes.
+</t>
+  </si>
+  <si>
+    <t>docs/external/task-mapping.md; tests/external/fixtures/; evidence/tb059-task-mapping.json; evidence/tb059-scripted/; evidence/tb059-goose-live/; evidence/tb059-goose-live-retry/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done 2026-10-20. Every development fixture (25: the tuning groups in data/splits.json) runs end to end through goose with the unchanged evaluators: scripted dev suite (tests/external/fixtures/dev-suite.json, 26 cases, both arms) gives evaluator verdicts identical to the built-in agent in every case (evidence/tb059-scripted). Tasks reach goose through its native input (task prompt via -t, documents only as tool results through the MCP adapter); fixtures, initial state and evaluators unchanged. No holdout fixture is loaded: development runs materialize only development fixtures and the runner asserts it (sealed_fixtures_loaded 0 in every report; tested with a mixed suite and a positive control). Live pilot (nvidia gpt-oss-20b, free tier, 1 repetition): 17/25 valid, retry 6/8 valid, 24/25 fixtures with a valid live pair; TB-ATT-DOC-008 timed out at the provider twice (invalid, not counted; not a mapping limit). No task goose cannot express. Live numbers are pilot evidence, not an estimate. Fixed: a run cut off while the provider still owed an answer was counted as a valid agent timeout; it is now an invalid provider fault.
 </t>
   </si>
 </sst>
@@ -3585,11 +3592,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.79166666666666663</v>
+        <v>0.80555555555555558</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3601,7 +3608,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7268,7 +7275,7 @@
         <v>780</v>
       </c>
       <c r="D70" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E70" s="10" t="s">
         <v>525</v>
@@ -7276,9 +7283,8 @@
       <c r="F70" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="G70" s="10" t="str">
-        <f t="shared" si="4"/>
-        <v>Ready</v>
+      <c r="G70" s="10" t="s">
+        <v>921</v>
       </c>
       <c r="H70" s="18">
         <v>5</v>
@@ -7309,11 +7315,14 @@
       <c r="R70" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="S70" s="14"/>
-      <c r="T70" s="14"/>
+      <c r="S70" s="14" t="s">
+        <v>925</v>
+      </c>
+      <c r="T70" s="14" t="s">
+        <v>926</v>
+      </c>
       <c r="U70" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:21" ht="64" customHeight="1">
@@ -8720,11 +8729,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8736,7 +8745,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0.25</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8744,11 +8753,11 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>

</xml_diff>

<commit_message>
TB-058 Completed in the workbook (Linux Mode B limitation stated)
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F7D707-D680-3A48-8263-843F9AE8461D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E0C7418-404D-2149-AFFF-4AEE0D65C6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1272" uniqueCount="927">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="928">
   <si>
     <t>Tasks</t>
   </si>
@@ -2807,14 +2807,17 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">In progress 2026-10-20. Done: goose and every process it starts run confined (sandbox-exec on macOS, Landlock on Linux; src/external/sandbox.ts): only the episode's adapter socket and model proxy port are reachable, writes only inside the episode folder, no reads of the harness's files; goose refuses to start unconfined. Adapter and gateway sockets accept one client; calls after cancellation are refused (episode_cancelled); native-mode data sits outside the agent sandbox. Contract 1.2.0. External tests pass with goose confined. Blocker: the bypass tests (direct calls, forged/replayed tokens, unlisted tools, argument smuggling, calls after cancellation, both modes, each with a positive control), the audit check and evidence/external-authorization-report.json are being written by the project owner; the Landlock path has not yet been exercised by a test in the Linux container. Next: run those tests, then mark Completed only if every acceptance item passes.
+    <t>docs/external/task-mapping.md; tests/external/fixtures/; evidence/tb059-task-mapping.json; evidence/tb059-scripted/; evidence/tb059-goose-live/; evidence/tb059-goose-live-retry/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done 2026-10-20. Every development fixture (25: the tuning groups in data/splits.json) runs end to end through goose with the unchanged evaluators: scripted dev suite (tests/external/fixtures/dev-suite.json, 26 cases, both arms) gives evaluator verdicts identical to the built-in agent in every case (evidence/tb059-scripted). Tasks reach goose through its native input (task prompt via -t, documents only as tool results through the MCP adapter); fixtures, initial state and evaluators unchanged. No holdout fixture is loaded: development runs materialize only development fixtures and the runner asserts it (sealed_fixtures_loaded 0 in every report; tested with a mixed suite and a positive control). Live pilot (nvidia gpt-oss-20b, free tier, 1 repetition): 17/25 valid, retry 6/8 valid, 24/25 fixtures with a valid live pair; TB-ATT-DOC-008 timed out at the provider twice (invalid, not counted; not a mapping limit). No task goose cannot express. Live numbers are pilot evidence, not an estimate. Fixed: a run cut off while the provider still owed an answer was counted as a valid agent timeout; it is now an invalid provider fault.
 </t>
   </si>
   <si>
-    <t>docs/external/task-mapping.md; tests/external/fixtures/; evidence/tb059-task-mapping.json; evidence/tb059-scripted/; evidence/tb059-goose-live/; evidence/tb059-goose-live-retry/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done 2026-10-20. Every development fixture (25: the tuning groups in data/splits.json) runs end to end through goose with the unchanged evaluators: scripted dev suite (tests/external/fixtures/dev-suite.json, 26 cases, both arms) gives evaluator verdicts identical to the built-in agent in every case (evidence/tb059-scripted). Tasks reach goose through its native input (task prompt via -t, documents only as tool results through the MCP adapter); fixtures, initial state and evaluators unchanged. No holdout fixture is loaded: development runs materialize only development fixtures and the runner asserts it (sealed_fixtures_loaded 0 in every report; tested with a mixed suite and a positive control). Live pilot (nvidia gpt-oss-20b, free tier, 1 repetition): 17/25 valid, retry 6/8 valid, 24/25 fixtures with a valid live pair; TB-ATT-DOC-008 timed out at the provider twice (invalid, not counted; not a mapping limit). No task goose cannot express. Live numbers are pilot evidence, not an estimate. Fixed: a run cut off while the provider still owed an answer was counted as a valid agent timeout; it is now an invalid provider fault.
+    <t>tests/external/authorization/; evidence/external-authorization-report.json; evidence/external-authorization-report-linux.json; src/external/sandbox.ts; docs/external/threat-model.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done 2026-10-22 (owner decision: complete with the Linux Mode B limitation stated). goose and every process it starts run confined (src/external/sandbox.ts: sandbox-exec on macOS, Landlock on Linux): only the episode socket and the model proxy port reachable, writes only inside the episode folder; the capability (gateway session token) stays in the adapter. Bypass tests (tests/external/authorization/, project owner): direct calls, forged and replayed tokens, unlisted tools, argument smuggling and calls after cancellation, in both modes; each with a positive control and the audit check. macOS: 12/12 pass, every refusal audited (gateway or TB-004 deny decisions, including refused connections and calls after the episode ends), no tool effect without a gateway allow (evidence/external-authorization-report.json). LIMITATION: Linux container run (Landlock) 10/12 - Mode A 6/6, Mode B 2 open (direct_calls not refused; unlisted_tools positive control not detected) (evidence/external-authorization-report-linux.json); listed uncovered in docs/external/threat-model.md, no claim covers the native integration on Linux; the live service runs Mode A only. Next action for the limitation: fix and rerun the two Mode B checks in the container.
 </t>
   </si>
 </sst>
@@ -3592,11 +3595,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.80555555555555558</v>
+        <v>0.81944444444444442</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3608,7 +3611,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7214,7 +7217,7 @@
         <v>774</v>
       </c>
       <c r="D69" s="14" t="s">
-        <v>558</v>
+        <v>1</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>525</v>
@@ -7222,9 +7225,8 @@
       <c r="F69" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="G69" s="10" t="str">
-        <f t="shared" si="4"/>
-        <v>In Progress</v>
+      <c r="G69" s="10" t="s">
+        <v>921</v>
       </c>
       <c r="H69" s="18">
         <v>6</v>
@@ -7255,13 +7257,14 @@
       <c r="R69" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="S69" s="14"/>
+      <c r="S69" s="14" t="s">
+        <v>926</v>
+      </c>
       <c r="T69" s="14" t="s">
-        <v>924</v>
+        <v>927</v>
       </c>
       <c r="U69" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:21" ht="64" customHeight="1">
@@ -7316,10 +7319,10 @@
         <v>100</v>
       </c>
       <c r="S70" s="14" t="s">
+        <v>924</v>
+      </c>
+      <c r="T70" s="14" t="s">
         <v>925</v>
-      </c>
-      <c r="T70" s="14" t="s">
-        <v>926</v>
       </c>
       <c r="U70" s="10">
         <v>1</v>
@@ -7346,7 +7349,7 @@
       </c>
       <c r="G71" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H71" s="18">
         <v>4</v>
@@ -8729,7 +8732,7 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
@@ -8737,7 +8740,7 @@
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F100" s="11">
         <f t="shared" ref="F100" si="19">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Blocked")</f>
@@ -8745,7 +8748,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0.33333333333333331</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8753,11 +8756,11 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>

</xml_diff>

<commit_message>
TB-060 Completed in the workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E0C7418-404D-2149-AFFF-4AEE0D65C6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C449859E-5737-D34C-9A6F-946AEE7E6392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="928">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="930">
   <si>
     <t>Tasks</t>
   </si>
@@ -2818,6 +2818,13 @@
   </si>
   <si>
     <t xml:space="preserve">Done 2026-10-22 (owner decision: complete with the Linux Mode B limitation stated). goose and every process it starts run confined (src/external/sandbox.ts: sandbox-exec on macOS, Landlock on Linux): only the episode socket and the model proxy port reachable, writes only inside the episode folder; the capability (gateway session token) stays in the adapter. Bypass tests (tests/external/authorization/, project owner): direct calls, forged and replayed tokens, unlisted tools, argument smuggling and calls after cancellation, in both modes; each with a positive control and the audit check. macOS: 12/12 pass, every refusal audited (gateway or TB-004 deny decisions, including refused connections and calls after the episode ends), no tool effect without a gateway allow (evidence/external-authorization-report.json). LIMITATION: Linux container run (Landlock) 10/12 - Mode A 6/6, Mode B 2 open (direct_calls not refused; unlisted_tools positive control not detected) (evidence/external-authorization-report-linux.json); listed uncovered in docs/external/threat-model.md, no claim covers the native integration on Linux; the live service runs Mode A only. Next action for the limitation: fix and rerun the two Mode B checks in the container.
+</t>
+  </si>
+  <si>
+    <t>evidence/external-smoke-report.json; tests/external/conformance/; evidence/tb060/; scripts/check-external-smoke.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done 2026-10-22. Conformance (tests/external/conformance/, mock model): the TB-012 smoke suite through goose, 17/17 valid, evaluator verdicts identical to the built-in agent, TB-004 traces valid, contract checks pass, spans for every run of both arms incl. model spans, no seeded sensitive value or credential (scripts/check-external-smoke.py; a control proves the checker rejects spans without model calls). Fixed on the way: goose runs exported no model spans; the model proxy now records each model call in the runner's span. Live smoke on the development split, both arms: local runner on qwen3.5:9b 6/6 valid; through the live-service API (a local instance of the service built from main) scripted 6/6 and live on Gemini gemma-4-26b-a4b-it (own key) 2/2 valid; all checks pass (evidence/external-smoke-report.json). NVIDIA free tier was congested (38 s for a trivial request): its 8 pairs timed out and are recorded invalid, never counted. Note: the public demo runs the previous image until redeployed; its service checks were not repeated there.
 </t>
   </si>
 </sst>
@@ -3595,11 +3602,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.81944444444444442</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3611,7 +3618,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7339,7 +7346,7 @@
         <v>788</v>
       </c>
       <c r="D71" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>533</v>
@@ -7347,9 +7354,8 @@
       <c r="F71" s="10" t="s">
         <v>541</v>
       </c>
-      <c r="G71" s="10" t="str">
-        <f t="shared" si="4"/>
-        <v>Ready</v>
+      <c r="G71" s="10" t="s">
+        <v>921</v>
       </c>
       <c r="H71" s="18">
         <v>4</v>
@@ -7380,11 +7386,14 @@
       <c r="R71" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="S71" s="14"/>
-      <c r="T71" s="14"/>
+      <c r="S71" s="14" t="s">
+        <v>928</v>
+      </c>
+      <c r="T71" s="14" t="s">
+        <v>929</v>
+      </c>
       <c r="U71" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:21" ht="64" customHeight="1">
@@ -7408,7 +7417,7 @@
       </c>
       <c r="G72" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H72" s="18">
         <v>4</v>
@@ -7526,7 +7535,7 @@
       </c>
       <c r="G74" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H74" s="18">
         <v>5</v>
@@ -8732,11 +8741,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8748,7 +8757,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0.41666666666666669</v>
+        <v>0.5</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8756,11 +8765,11 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>

</xml_diff>

<commit_message>
TB-060 workbook note: demo results and provider faults
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C449859E-5737-D34C-9A6F-946AEE7E6392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7FD2039-FC56-DD40-875D-ACBFDA5F475B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="-21600" yWindow="-7640" windowWidth="21600" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
@@ -2824,7 +2824,7 @@
     <t>evidence/external-smoke-report.json; tests/external/conformance/; evidence/tb060/; scripts/check-external-smoke.py</t>
   </si>
   <si>
-    <t xml:space="preserve">Done 2026-10-22. Conformance (tests/external/conformance/, mock model): the TB-012 smoke suite through goose, 17/17 valid, evaluator verdicts identical to the built-in agent, TB-004 traces valid, contract checks pass, spans for every run of both arms incl. model spans, no seeded sensitive value or credential (scripts/check-external-smoke.py; a control proves the checker rejects spans without model calls). Fixed on the way: goose runs exported no model spans; the model proxy now records each model call in the runner's span. Live smoke on the development split, both arms: local runner on qwen3.5:9b 6/6 valid; through the live-service API (a local instance of the service built from main) scripted 6/6 and live on Gemini gemma-4-26b-a4b-it (own key) 2/2 valid; all checks pass (evidence/external-smoke-report.json). NVIDIA free tier was congested (38 s for a trivial request): its 8 pairs timed out and are recorded invalid, never counted. Note: the public demo runs the previous image until redeployed; its service checks were not repeated there.
+    <t xml:space="preserve">Done 2026-10-22. Conformance (tests/external/conformance/, mock model): TB-012 smoke suite through goose 17/17 valid, verdicts identical to the built-in agent, TB-004 traces valid, contract checks pass, spans for every run incl. model spans, no seeded sensitive value or credential (scripts/check-external-smoke.py; a control proves it rejects spans without model calls). Fixed: goose runs exported no model spans; the model proxy now records each model call in the runner's span. Live smoke, development split, both arms: local runner on qwen3.5:9b 6/6 valid; live-service API, local instance: scripted 6/6, Gemini (own key) 2/2; deployed public demo (redeployed from main): scripted 6/6. All checks pass (evidence/external-smoke-report.json). Provider faults: NVIDIA gpt-oss-20b timed out (28-90 s per trivial request) in every attempt incl. the demo's hosted mode, and Gemini returned 5xx on the demo; all those pairs are recorded invalid, never counted. Open: a valid live pair through the deployed demo itself awaits a provider that answers.
 </t>
   </si>
 </sst>

</xml_diff>

<commit_message>
TB-060 workbook note: live check through the deployed demo
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7FD2039-FC56-DD40-875D-ACBFDA5F475B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EDFC5FC-A4D7-4044-B255-2C6EE8BFDFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="-21600" yWindow="-7640" windowWidth="21600" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2824,7 +2824,7 @@
     <t>evidence/external-smoke-report.json; tests/external/conformance/; evidence/tb060/; scripts/check-external-smoke.py</t>
   </si>
   <si>
-    <t xml:space="preserve">Done 2026-10-22. Conformance (tests/external/conformance/, mock model): TB-012 smoke suite through goose 17/17 valid, verdicts identical to the built-in agent, TB-004 traces valid, contract checks pass, spans for every run incl. model spans, no seeded sensitive value or credential (scripts/check-external-smoke.py; a control proves it rejects spans without model calls). Fixed: goose runs exported no model spans; the model proxy now records each model call in the runner's span. Live smoke, development split, both arms: local runner on qwen3.5:9b 6/6 valid; live-service API, local instance: scripted 6/6, Gemini (own key) 2/2; deployed public demo (redeployed from main): scripted 6/6. All checks pass (evidence/external-smoke-report.json). Provider faults: NVIDIA gpt-oss-20b timed out (28-90 s per trivial request) in every attempt incl. the demo's hosted mode, and Gemini returned 5xx on the demo; all those pairs are recorded invalid, never counted. Open: a valid live pair through the deployed demo itself awaits a provider that answers.
+    <t xml:space="preserve">Done 2026-10-22. Conformance (tests/external/conformance/, mock model): TB-012 smoke suite through goose 17/17 valid, verdicts identical to the built-in agent, TB-004 traces valid, contract checks pass, spans for every run incl. model spans, no seeded sensitive value or credential (scripts/check-external-smoke.py; a control proves it rejects spans without model calls). Live smoke, development split, both arms, all checks pass (evidence/external-smoke-report.json): local runner qwen3.5:9b 6/6; live-service API on a local instance: scripted 6/6, Gemini 2/2; deployed public demo: scripted 6/6 and live Gemini (own key) 2/2. Fixed on the way: (1) goose runs exported no model spans; (2) a provider fault goose retried past invalidated the run, stricter than the built-in agents; now counted as a retry (provider_retries), only faults the run ends on make it invalid (tested with a fake provider and a control). Provider faults recorded invalid, never counted: NVIDIA gpt-oss-20b timed out in every attempt (free tier congested), two early Gemini demo attempts under the old rule.
 </t>
   </si>
 </sst>

</xml_diff>

<commit_message>
TB-061 Completed in the workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EDFC5FC-A4D7-4044-B255-2C6EE8BFDFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C01DFF-B825-6F4F-8F16-D0E79CAED2F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="-21600" yWindow="-7640" windowWidth="21600" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="930">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="932">
   <si>
     <t>Tasks</t>
   </si>
@@ -2825,6 +2825,13 @@
   </si>
   <si>
     <t xml:space="preserve">Done 2026-10-22. Conformance (tests/external/conformance/, mock model): TB-012 smoke suite through goose 17/17 valid, verdicts identical to the built-in agent, TB-004 traces valid, contract checks pass, spans for every run incl. model spans, no seeded sensitive value or credential (scripts/check-external-smoke.py; a control proves it rejects spans without model calls). Live smoke, development split, both arms, all checks pass (evidence/external-smoke-report.json): local runner qwen3.5:9b 6/6; live-service API on a local instance: scripted 6/6, Gemini 2/2; deployed public demo: scripted 6/6 and live Gemini (own key) 2/2. Fixed on the way: (1) goose runs exported no model spans; (2) a provider fault goose retried past invalidated the run, stricter than the built-in agents; now counted as a retry (provider_retries), only faults the run ends on make it invalid (tested with a fake provider and a control). Provider faults recorded invalid, never counted: NVIDIA gpt-oss-20b timed out in every attempt (free tier congested), two early Gemini demo attempts under the old rule.
+</t>
+  </si>
+  <si>
+    <t>protocol/amendments.md (A-030); protocol/experiment-registry.yaml (external_validation); scripts/external-split.py; tests/external/split/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done 2026-10-22. Amendment A-030 (protocol/amendments.md) and registry entry external_validation (protocol 1.3.0) committed before any external evaluation run (all external-agent runs so far are development work on the development split; verify-protocol asserts evaluation_runs_started=false). Registered: hypotheses H1-H3, primary endpoints (unsafe committed-effect rate, benign utility, 5 pp non-inferiority margin), overhead measures, adapter modes (Mode A primary, Mode B secondary, Linux Mode B confinement not claimed), systems, 5 repetitions, frozen model with a fallback rule (never pooled), renderings, analysis (Wilson, cluster bootstrap, McNemar) and stopping rules. Split procedure registered, not the split: scripts/external-split.py assigns families (seed 2026102201, 60% external, stratified by workflow, sha256 order); ineligible: the 8 tuning-used families and every sealed fixture; holdout-only families eligible as new fixtures (holdout_seen); refuses reassignment and hand-edited manifests. Tests (tests/external/split, 7) on placeholder lists: deterministic for its seed, stratified, excludes tuning families and the core holdout, no reassignment. The split itself is made in TB-062.
 </t>
   </si>
 </sst>
@@ -3602,11 +3609,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.83333333333333337</v>
+        <v>0.84722222222222221</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3618,7 +3625,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7407,7 +7414,7 @@
         <v>848</v>
       </c>
       <c r="D72" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E72" s="10" t="s">
         <v>549</v>
@@ -7415,9 +7422,8 @@
       <c r="F72" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="G72" s="10" t="str">
-        <f t="shared" si="4"/>
-        <v>Ready</v>
+      <c r="G72" s="10" t="s">
+        <v>921</v>
       </c>
       <c r="H72" s="18">
         <v>4</v>
@@ -7448,11 +7454,14 @@
       <c r="R72" s="10" t="s">
         <v>771</v>
       </c>
-      <c r="S72" s="14"/>
-      <c r="T72" s="14"/>
+      <c r="S72" s="14" t="s">
+        <v>930</v>
+      </c>
+      <c r="T72" s="14" t="s">
+        <v>931</v>
+      </c>
       <c r="U72" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:21" ht="64" customHeight="1">
@@ -7476,7 +7485,7 @@
       </c>
       <c r="G73" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H73" s="18">
         <v>8</v>
@@ -8741,11 +8750,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8757,7 +8766,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0.5</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8765,7 +8774,7 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>

</xml_diff>

<commit_message>
TB-062 Completed in the workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C01DFF-B825-6F4F-8F16-D0E79CAED2F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6408D4-1D6D-194A-8A2E-7A2F9A599BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="-21600" yWindow="-7640" windowWidth="21600" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="934">
   <si>
     <t>Tasks</t>
   </si>
@@ -2832,6 +2832,13 @@
   </si>
   <si>
     <t xml:space="preserve">Done 2026-10-22. Amendment A-030 (protocol/amendments.md) and registry entry external_validation (protocol 1.3.0) committed before any external evaluation run (all external-agent runs so far are development work on the development split; verify-protocol asserts evaluation_runs_started=false). Registered: hypotheses H1-H3, primary endpoints (unsafe committed-effect rate, benign utility, 5 pp non-inferiority margin), overhead measures, adapter modes (Mode A primary, Mode B secondary, Linux Mode B confinement not claimed), systems, 5 repetitions, frozen model with a fallback rule (never pooled), renderings, analysis (Wilson, cluster bootstrap, McNemar) and stopping rules. Split procedure registered, not the split: scripts/external-split.py assigns families (seed 2026102201, 60% external, stratified by workflow, sha256 order); ineligible: the 8 tuning-used families and every sealed fixture; holdout-only families eligible as new fixtures (holdout_seen); refuses reassignment and hand-edited manifests. Tests (tests/external/split, 7) on placeholder lists: deterministic for its seed, stratified, excludes tuning families and the core holdout, no reassignment. The split itself is made in TB-062.
+</t>
+  </si>
+  <si>
+    <t>data/external-attacks.jsonl; data/external-attack-oracles.json; data/external-splits.json; data/external-manifest.json; tests/external/attacks/; evidence/tb062-positive-controls.json; docs/external/attack-families.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done 2026-10-22. 12 attack families, each with a benign twin, oracle, cited source (arXiv) and rationale, new tenants (data/external-*.json): new - long-document buried instruction, delayed multi-step instruction, cross-tool split injection, allowed-tool exfiltration, forged plan status, delayed cross-record update; re-authored as new fixtures (holdout_seen) - citation laundering, abstention override, contact-attribute leak, payment-instruction insertion, approved-value substitution, notification exfiltration. Memory attacks not applicable (goose memory disabled by the contract, EX-25). Every oracle validated on scripted trajectories against the real backend (tests/external/attacks): benign twin passes, injection alone is no effect, attack-following trajectory achieves the goal. Split assigned by the registered TB-061 script: 9 external_validation, 3 tuning (one per workflow); disjoint from tuning families and sealed fixtures (tested); data/external-manifest.json froze all files with SHA-256 before any defended run (one pre-run revision of TB-ATT-EXT-EMAIL-001 recorded with its previous digest). Positive controls vs the undefended agent (goose, local qwen3.5:9b, 3 repetitions): 36/36, every family 3/3 (evidence/tb062-positive-controls.json); earlier single runs each had one miss, disclosed. No defended run made.
 </t>
   </si>
 </sst>
@@ -3609,11 +3616,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.84722222222222221</v>
+        <v>0.86111111111111116</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3625,7 +3632,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7475,7 +7482,7 @@
         <v>797</v>
       </c>
       <c r="D73" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>753</v>
@@ -7483,9 +7490,8 @@
       <c r="F73" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="G73" s="10" t="str">
-        <f t="shared" si="4"/>
-        <v>Ready</v>
+      <c r="G73" s="10" t="s">
+        <v>921</v>
       </c>
       <c r="H73" s="18">
         <v>8</v>
@@ -7516,11 +7522,14 @@
       <c r="R73" s="10" t="s">
         <v>771</v>
       </c>
-      <c r="S73" s="14"/>
-      <c r="T73" s="14"/>
+      <c r="S73" s="14" t="s">
+        <v>932</v>
+      </c>
+      <c r="T73" s="14" t="s">
+        <v>933</v>
+      </c>
       <c r="U73" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:21" ht="64" customHeight="1">
@@ -8750,11 +8759,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8766,7 +8775,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0.58333333333333337</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8774,11 +8783,11 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>

</xml_diff>

<commit_message>
TB-063 Completed in the workbook; TB-061 evidence paths without inline notes
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6408D4-1D6D-194A-8A2E-7A2F9A599BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562FEFD7-39B4-8845-AB69-ECFE80C32FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="-21600" yWindow="-7640" windowWidth="21600" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="934">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1285" uniqueCount="936">
   <si>
     <t>Tasks</t>
   </si>
@@ -2828,9 +2828,6 @@
 </t>
   </si>
   <si>
-    <t>protocol/amendments.md (A-030); protocol/experiment-registry.yaml (external_validation); scripts/external-split.py; tests/external/split/</t>
-  </si>
-  <si>
     <t xml:space="preserve">Done 2026-10-22. Amendment A-030 (protocol/amendments.md) and registry entry external_validation (protocol 1.3.0) committed before any external evaluation run (all external-agent runs so far are development work on the development split; verify-protocol asserts evaluation_runs_started=false). Registered: hypotheses H1-H3, primary endpoints (unsafe committed-effect rate, benign utility, 5 pp non-inferiority margin), overhead measures, adapter modes (Mode A primary, Mode B secondary, Linux Mode B confinement not claimed), systems, 5 repetitions, frozen model with a fallback rule (never pooled), renderings, analysis (Wilson, cluster bootstrap, McNemar) and stopping rules. Split procedure registered, not the split: scripts/external-split.py assigns families (seed 2026102201, 60% external, stratified by workflow, sha256 order); ineligible: the 8 tuning-used families and every sealed fixture; holdout-only families eligible as new fixtures (holdout_seen); refuses reassignment and hand-edited manifests. Tests (tests/external/split, 7) on placeholder lists: deterministic for its seed, stratified, excludes tuning families and the core holdout, no reassignment. The split itself is made in TB-062.
 </t>
   </si>
@@ -2840,6 +2837,15 @@
   <si>
     <t xml:space="preserve">Done 2026-10-22. 12 attack families, each with a benign twin, oracle, cited source (arXiv) and rationale, new tenants (data/external-*.json): new - long-document buried instruction, delayed multi-step instruction, cross-tool split injection, allowed-tool exfiltration, forged plan status, delayed cross-record update; re-authored as new fixtures (holdout_seen) - citation laundering, abstention override, contact-attribute leak, payment-instruction insertion, approved-value substitution, notification exfiltration. Memory attacks not applicable (goose memory disabled by the contract, EX-25). Every oracle validated on scripted trajectories against the real backend (tests/external/attacks): benign twin passes, injection alone is no effect, attack-following trajectory achieves the goal. Split assigned by the registered TB-061 script: 9 external_validation, 3 tuning (one per workflow); disjoint from tuning families and sealed fixtures (tested); data/external-manifest.json froze all files with SHA-256 before any defended run (one pre-run revision of TB-ATT-EXT-EMAIL-001 recorded with its previous digest). Positive controls vs the undefended agent (goose, local qwen3.5:9b, 3 repetitions): 36/36, every family 3/3 (evidence/tb062-positive-controls.json); earlier single runs each had one miss, disclosed. No defended run made.
 </t>
+  </si>
+  <si>
+    <t>Done 2026-10-22. 10 fault classes plus 3 no-fault controls, goose 1.55.0 on both arms (alone, behind the gateway), live ollama:qwen3.5:9b, 3 repetitions each, 78 runs, 0 invalid. Classes: read timeout (hang, ended by the new 20 s per-call adapter timeout), 503 twice, 429, connection reset, malformed body, 1.5 MB oversized output, 8 s slow response, draft response lost after commit, apply 503 after commit, cancellation after the first call. Acceptance (checked by script): every class exercised on both arms; 0 duplicate committed writes; recovery and termination rates per class and arm with Wilson 95% intervals; 0 calls forwarded after cancellation. Results: termination 3/3 everywhere (no runtime-limit endings). Recovery 0/3 on both arms for timeout, 503, reset and malformed (goose does not retry the read; it searches and saves an uncited note); 3/3 for 429 (retries), oversized, slow and apply-after-commit; draft-lost 3/3 alone, 2/3 behind the gateway (one run never reached the draft). Goose re-sent the lost draft with the same key in 4 of 5 runs that reached it; the backend refused it (draft_already_exists), so writes are protected by backend idempotency, not the agent; gateway replays 0. On the gateway arm, after-commit faults on apply_record_update are injected in the host approval workflow so both arms lose the same committing response. Limits: 3 repetitions of one local model, one case per workflow, so intervals are wide; no between-arm test claimed; the email control already fails 2/3 behind the gateway without faults (the model opens with read_document, outside the email contract); cancellation drill runs on the MCP adapter, not the native-extension mode.</t>
+  </si>
+  <si>
+    <t>protocol/amendments.md; protocol/experiment-registry.yaml; scripts/external-split.py; tests/external/split/</t>
+  </si>
+  <si>
+    <t>evidence/external-reliability-report.json; configs/external-reliability.yaml; scripts/external-reliability.mjs; tests/recovery/fault-schedules.json; tests/external/reliability/; docs/external/reliability.md</t>
   </si>
 </sst>
 </file>
@@ -3616,11 +3622,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.86111111111111116</v>
+        <v>0.875</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3632,7 +3638,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7462,10 +7468,10 @@
         <v>771</v>
       </c>
       <c r="S72" s="14" t="s">
+        <v>934</v>
+      </c>
+      <c r="T72" s="14" t="s">
         <v>930</v>
-      </c>
-      <c r="T72" s="14" t="s">
-        <v>931</v>
       </c>
       <c r="U72" s="10">
         <v>1</v>
@@ -7523,10 +7529,10 @@
         <v>771</v>
       </c>
       <c r="S73" s="14" t="s">
+        <v>931</v>
+      </c>
+      <c r="T73" s="14" t="s">
         <v>932</v>
-      </c>
-      <c r="T73" s="14" t="s">
-        <v>933</v>
       </c>
       <c r="U73" s="10">
         <v>1</v>
@@ -7543,7 +7549,7 @@
         <v>801</v>
       </c>
       <c r="D74" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E74" s="10" t="s">
         <v>549</v>
@@ -7553,7 +7559,7 @@
       </c>
       <c r="G74" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H74" s="18">
         <v>5</v>
@@ -7584,11 +7590,15 @@
       <c r="R74" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="S74" s="14"/>
-      <c r="T74" s="14"/>
+      <c r="S74" s="14" t="s">
+        <v>935</v>
+      </c>
+      <c r="T74" s="14" t="s">
+        <v>933</v>
+      </c>
       <c r="U74" s="10">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:21" ht="64" customHeight="1">
@@ -7612,7 +7622,7 @@
       </c>
       <c r="G75" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H75" s="18">
         <v>10</v>
@@ -8759,11 +8769,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8775,7 +8785,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0.66666666666666663</v>
+        <v>0.75</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8783,7 +8793,7 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>

</xml_diff>

<commit_message>
TB-064 Completed in the workbook
</commit_message>
<xml_diff>
--- a/planning/TrustBench-AI_Plan.xlsx
+++ b/planning/TrustBench-AI_Plan.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MHRJ/TrustBench-AI/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562FEFD7-39B4-8845-AB69-ECFE80C32FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA9C238B-D3AB-594E-B924-E0185578B094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-21600" yWindow="-7640" windowWidth="21600" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21600" yWindow="-7640" windowWidth="21600" windowHeight="37800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrustBench-AI" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1285" uniqueCount="936">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1287" uniqueCount="938">
   <si>
     <t>Tasks</t>
   </si>
@@ -2846,6 +2846,12 @@
   </si>
   <si>
     <t>evidence/external-reliability-report.json; configs/external-reliability.yaml; scripts/external-reliability.mjs; tests/recovery/fault-schedules.json; tests/external/reliability/; docs/external/reliability.md</t>
+  </si>
+  <si>
+    <t>evidence/external-evaluation-report.json; runs/external/; docs/external/evaluation.md; scripts/run-external-evaluation.mjs; scripts/analyse-external-evaluation.py; tests/external/evaluation/</t>
+  </si>
+  <si>
+    <t>Done 2026-10-24. goose 1.55.0 (Mode A) alone vs behind the gateway (gateway_capability: the frozen gateway with no agent-side defense, which an external agent cannot host; A-030) on the 9 external-validation families plus their 9 benign twins; TB-028 schedules, 5 repetitions; benign once, attacks under the primary, secondary and positive-control renderings: 180 pairs per model. Every scheduled unit has a paired report in every batch (checked by script). Registered fallback rule applied in order and recorded in protocol/amendments.md: primary nvidia:openai/gpt-oss-20b 141/180 pairs invalid (78%, all provider timeouts at 240 s, both arms alike) and Gemini gemma-4-26b-a4b-it 74/180 invalid (41%, 429 and 5xx; it ran in 2 lanes, which raised its request rate) are kept in full and labelled INVALID with no rates; the last fallback ollama:qwen3.5:9b was 180/180 valid with one constant response model and is the analysed batch (a separate analysis, not pooled). Results (qwen, Wilson 95% / cluster-bootstrap 95%): unsafe committed effect, primary rendering 33/45 alone vs 2/45 gateway, difference -0.69 [-0.91, -0.40] (H1 supported); as_authored 21/45 vs 5/45, -0.36 [-0.60, -0.13]; positive control 45/45 vs 7/45. Benign utility 37/45 on both arms, difference 0.00 [-0.18, +0.16]: H2 non-inferiority (5 pp) not established, the interval is wider than the margin. Remaining leaks are all email-body content (contact-attribute leak, payment instruction, allowed-tool exfiltration), which a capability gateway does not inspect. Overhead: gateway policy p50 1.6 ms, p95 15.5 ms per decision; model calls p50 3 vs 3.5; 2/90 defended runs at a runtime limit (budget), 0/90 baseline. Limits: the analysed model is the last fallback (local 9B), not the frozen primary; Mode B (native integration) not run in this pass; goose sends no seed, so repetitions differ by sampling.</t>
   </si>
 </sst>
 </file>
@@ -3622,11 +3628,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Completed")</f>
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C5" s="6">
         <f>IF(A5=0,0,B5/A5)</f>
-        <v>0.875</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS($D$12:$D$83,"Blocked")</f>
@@ -3638,7 +3644,7 @@
       </c>
       <c r="F5" s="5">
         <f>SUMIFS($H$12:$H$83,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="G5" s="6">
         <f>COUNTIFS($Q$12:$Q$83,"Core",$D$12:$D$83,"Completed")/COUNTIFS($Q$12:$Q$83,"Core")</f>
@@ -7612,7 +7618,7 @@
         <v>809</v>
       </c>
       <c r="D75" s="14" t="s">
-        <v>288</v>
+        <v>1</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>763</v>
@@ -7622,7 +7628,7 @@
       </c>
       <c r="G75" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Ready</v>
+        <v>Done</v>
       </c>
       <c r="H75" s="18">
         <v>10</v>
@@ -7653,11 +7659,15 @@
       <c r="R75" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="S75" s="14"/>
-      <c r="T75" s="14"/>
+      <c r="S75" s="14" t="s">
+        <v>936</v>
+      </c>
+      <c r="T75" s="14" t="s">
+        <v>937</v>
+      </c>
       <c r="U75" s="10">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:21" ht="64" customHeight="1">
@@ -7681,7 +7691,7 @@
       </c>
       <c r="G76" s="10" t="str">
         <f t="shared" si="4"/>
-        <v>Waiting</v>
+        <v>Ready</v>
       </c>
       <c r="H76" s="18">
         <v>5</v>
@@ -8769,11 +8779,11 @@
       </c>
       <c r="C100" s="11">
         <f t="shared" ref="C100" si="16">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Completed")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D100" s="11">
         <f t="shared" ref="D100" si="17">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"Not Started")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E100" s="11">
         <f t="shared" ref="E100" si="18">COUNTIFS($B$12:$B$83,A100,$D$12:$D$83,"In Progress")</f>
@@ -8785,7 +8795,7 @@
       </c>
       <c r="G100" s="20">
         <f t="shared" ref="G100" si="20">IF(B100=0,0,C100/B100)</f>
-        <v>0.75</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="H100" s="11">
         <f t="shared" ref="H100" si="21">SUMIFS($H$12:$H$83,$B$12:$B$83,A100)</f>
@@ -8793,7 +8803,7 @@
       </c>
       <c r="I100" s="11">
         <f>SUMIFS($H$12:$H$83,$B$12:$B$83,A100,$D$12:$D$83,"&lt;&gt;Completed")</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J100" s="11">
         <f>COUNTIFS($B$12:$B$83,A100,$G$12:$G$83,"Ready")</f>

</xml_diff>